<commit_message>
Update project requirements to enable dashboard access for more presets
Modify project requirements to allow the dashboard button to be visible in additional workstation presets.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c384a648-21d3-4e2b-a374-d15729a9d42d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,14 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="72.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -491,9 +484,26 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B6" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C6" t="str">
+        <v>נעלמה האפשרות לצפות בגאנט עומסים מהעמדה</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update base status to modify only the target base
Refactors the base status update logic to target a single base. Prioritizes `mazaa_update_base_id`, falls back to `parent_base_id`, and then uses the first base in `base_status_ids`. This replaces previous behavior that would update all bases in the `base_status_ids` array.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 83326152-ee87-4f42-a734-3e26073410c9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -501,9 +501,26 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B7" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C7" t="str">
+        <v>עדכון מז"א בעמדת מגדל מעדכן את כל הבסיסים ברשימה במקום רק את בסיס האב של העמדה</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move runway selection to the map and remove red indicators
Update the GroundView component to accept and display an overlay, moving the runway selection panel from the header to the bottom-right of the map. Additionally, remove the red circle indicators from closed runways.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0819d46d-3b9b-4ce0-a114-d01851af611d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -518,9 +518,26 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B8" t="str">
+        <v>שיפור</v>
+      </c>
+      <c r="C8" t="str">
+        <v>הזזת רשימת מסלולים בשדה תעופה מהסרגל העליון לחלק הימני התחתון של המפה + הסרת עיגול אדום ליד מסלולים סגורים</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reduce the size of area names in blind map mode
Decrease font size of zone names in blind map mode from 2.8 to 1.3 and remove bold styling.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f2bb35b9-9605-455e-8754-d53d5a63afa6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -535,9 +535,26 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B9" t="str">
+        <v>שיפור</v>
+      </c>
+      <c r="C9" t="str">
+        <v>במצב מפה עיוורת — הקטנת שמות האזורים כך שייראו אך לא יחסמו את האזור</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update user preferences to log all requests
Add a user preference to the replit.md file, specifying that the `project-requirements.xlsx` file should be updated after every user request.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a76bf8da-3a18-4db5-899b-39a99a51a6f8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -552,9 +552,26 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B10" t="str">
+        <v>העדפה</v>
+      </c>
+      <c r="C10" t="str">
+        <v>עדכון קובץ האקסל (project-requirements.xlsx) אחרי כל בקשה בשיחה</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update project requirements file title and metadata
Update the title in agent assets metadata to reflect the project requirements Excel file name and ensure the Excel file is correctly referenced.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ae406c89-9008-4e7e-8925-3913386cf6f4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -569,9 +569,26 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B11" t="str">
+        <v>שאלה</v>
+      </c>
+      <c r="C11" t="str">
+        <v>היכן רואים את קובץ האקסל project-requirements.xlsx</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add time to logged requirements in the project file
Update the logging mechanism to include the current time along with the date in the 'project-requirements.xlsx' file. This involves modifying the `update-excel.js` script and updating the `SKILL.md` documentation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6eeeeccb-1d16-4622-b02d-f47c0758fbd9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -586,9 +586,26 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-06-15 13:08</v>
+      </c>
+      <c r="B12" t="str">
+        <v>שיפור</v>
+      </c>
+      <c r="C12" t="str">
+        <v>הוספת שעה לעמודת תאריך בקובץ האקסל</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add time to log entries in project requirements
Update project-requirements.xlsx to include timestamp in addition to date for log entries.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: fd068891-b101-4096-95f3-99d01b01408e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/BFZBpDd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -603,9 +603,26 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-06-15 13:09</v>
+      </c>
+      <c r="B13" t="str">
+        <v>שאלה</v>
+      </c>
+      <c r="C13" t="str">
+        <v>בירור לגבי יכולת זיהוי קולי והמרה לטקסט בעברית</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Web Speech API voice recognition — Phase 1: altitude update
- Added 🎤 קול button to workstation header bar
- Web Speech API (he-IL Hebrew) starts on click, stops on second click
- parseAltFromSpeech: extracts altitude from speech — Arabic digits first,
  then Hebrew number words (מאה, אלף, שתיים עשרה אלף, etc.)
- findStripByVoice: matches callsign from speech against workstation strips
- If only one strip at workstation → no callsign needed, just say the altitude
- If multiple strips → say callsign + altitude to target the right one
- handleAltUpdate called on successful recognition → updates strip alt field
- Voice feedback overlay: listening indicator (animated 🎤), live transcript,
  ✅ success (callsign + alt) or ⚠️ error message; auto-dismisses after 5s
- @keyframes voicePulse animation for mic button and overlay icon
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -620,9 +620,26 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-06-15 13:13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C14" t="str">
+        <v>שילוב Web Speech API — זיהוי קולי בעברית: שמיעת גובה חדש ועדכון עמודת גובה בסטריפ הנבחר בעמדה</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Extend voice recognition: altitude ranges + transfer commands
- Added parseHebrewNumber() helper (shared between range and single parsing)
- parseAltFromSpeech now handles ranges: "300-400", "300 עד 400",
  "שלוש מאות עד ארבע מאות"
- Added parseTransferDest() to detect "ל[sector]" pattern in speech
- Added findSectorByVoice() to match sector name in allSectors list
- startVoiceAlt now handles transfer commands:
  "חנית 400 לצארלי" → update altitude + transfer to sector "צארלי"
  "חנית לצארלי 400" → same, any word order
- voiceResult state extended with transferDest and action fields
- Overlay shows "✅ callsign → sector / גובה: X" for transfer commands
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -637,9 +637,26 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-06-15 13:40</v>
+      </c>
+      <c r="B15" t="str">
+        <v>שיפור קיים</v>
+      </c>
+      <c r="C15" t="str">
+        <v>זיהוי קולי — הרחבה: 1) טווחי גבהים (300-400) 2) פקודת העברה לנקודת העברה (חנית 400 לצארלי)</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add documentation for voice recognition feature to Excel export
Add a new sheet to the Excel export detailing voice recognition feature implementation and usage.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6c72aba8-8949-4442-8746-f2eb53b82268
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/2zPRqmR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="דרישות" sheetId="1" r:id="rId1"/>
+    <sheet name="מה בוצע ואיך להפעיל" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -659,4 +660,239 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B36"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SKY KING — פיצ'רים שבוצעו ומדריך תפעול</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>=== זיהוי קולי (Web Speech API) ===</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>מה בוצע:</v>
+      </c>
+      <c r="B5" t="str">
+        <v>שלב 1 — עדכון גובה קולי</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v>לחץ 🎤 בסרגל הכלים → אמור את שם המטוס + גובה → המערכת מזהה ומעדכנת.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v>דוגמה: "חנית 400" → מעדכן גובה של סטריפ חנית ל-400</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>מה בוצע:</v>
+      </c>
+      <c r="B9" t="str">
+        <v>שלב 2 — טווחי גבהים</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v>ניתן לאמור טווח גבהים בשני פורמטים:</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v>• מספרים: "300-400" / "300 עד 400"</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v>• מילים בעברית: "שלוש מאות עד ארבע מאות"</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v>דוגמה: "חנית שלוש מאות עד ארבע מאות" → גובה 300-400</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>מה בוצע:</v>
+      </c>
+      <c r="B15" t="str">
+        <v>שלב 2 — פקודת העברה לנקודת העברה</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v>ניתן לאמור פקודת העברה לסקטור/נקודת העברה:</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v>• "חנית 400 לצארלי" → מעביר את חנית לנקודה "צארלי" + מעדכן גובה 400</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v>• "חנית לצארלי 400" → אותו הדבר, סדר אחר</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v>• "חנית לצארלי" → מעביר בלי עדכון גובה</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v>הערה: שם נקודת ההעברה חייב להיות זהה לשם הסקטור כפי שהוגדר במערכת</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>=== הפעלה ===</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>שלב</v>
+      </c>
+      <c r="B24" t="str">
+        <v>פעולה</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>1</v>
+      </c>
+      <c r="B25" t="str">
+        <v>לחץ על כפתור 🎤 בסרגל הכלים של העמדה</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2</v>
+      </c>
+      <c r="B26" t="str">
+        <v>הדפדפן יבקש הרשאת מיקרופון — אשר</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>3</v>
+      </c>
+      <c r="B27" t="str">
+        <v>אמור בעברית את הפקודה (גובה / טווח / העברה)</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>4</v>
+      </c>
+      <c r="B28" t="str">
+        <v>ה-overlay מציג transcript בזמן אמת</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>5</v>
+      </c>
+      <c r="B29" t="str">
+        <v>כשהמערכת מזהה — מופיע ✅ + הפעולה בוצעה אוטומטית</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>6</v>
+      </c>
+      <c r="B30" t="str">
+        <v>שגיאה — מופיע ⚠️ עם הסיבה</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>=== הגבלות ===</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v/>
+      </c>
+      <c r="B33" t="str">
+        <v>• עובד ב-Chrome / Edge בלבד (Web Speech API)</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v>• שם המטוס חייב להופיע בסטריפים של העמדה הנוכחית</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v>• אם יש סטריפ יחיד בעמדה — לא צריך לאמור שם מטוס</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v>• שם נקודת העברה חייב להתאים בדיוק לשם הסקטור במערכת</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B36"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Improve voice command parsing for split formations and altitudes
Refactor `findStripByVoice` to a new `parseVoiceCommand` function that handles split formations by matching callsigns and aircraft indices, and improves altitude parsing by correctly distinguishing formation indices from altitude values.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: af456fca-238f-4003-be73-051c278c9e86
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/2zPRqmR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -655,9 +655,26 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-06-15 13:50</v>
+      </c>
+      <c r="B16" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C16" t="str">
+        <v>זיהוי קולי — תמיכה בפמ פוצל: זיהוי index מבנה (פיל 3) + מניעת בלבול עם גובה</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -665,10 +682,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B36"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Improve voice command recognition for transfer points
Fixes regex issues with Hebrew characters and expands sector search to include classic transfer points.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e4b7feca-cc65-44c5-b70e-afe52d7a953e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/2zPRqmR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -672,9 +672,43 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-06-15 13:57</v>
+      </c>
+      <c r="B17" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C17" t="str">
+        <v>זיהוי קולי — תיקון regex ל-ל prefix: \b לא עובד בעברית, הוחלף ב-(?:^|\s)</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-06-15 13:57</v>
+      </c>
+      <c r="B18" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C18" t="str">
+        <v>זיהוי קולי — העברה בלי גובה נתמכת; חיפוש סקטור גם ב-classic_transfer_points לפי label</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add voice commands to assign strips to map zones and accept incoming transfers
Make `onresult` callback async, add functionality to parse voice commands for zone assignments, find zones by voice input, and identify incoming transfers.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e2b7c190-6adc-4aa8-aea1-d3146e110686
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Elkr8Ti
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -706,9 +706,43 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-06-15 14:04</v>
+      </c>
+      <c r="B19" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C19" t="str">
+        <v>זיהוי קולי — שיוך פמ לאזור במה בדיבור: "חנית לאזור צפון"</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-06-15 14:04</v>
+      </c>
+      <c r="B20" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C20" t="str">
+        <v>זיהוי קולי — קבלת העברה נכנסת + שיוך לאזור בדיבור: "[callsign] לאזור [שם]"</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve canvas drawing by supporting pen input and fixing touch issues
Update canvas components to use pointer events for input, addressing issues with stylus and touch drawing, and refactor drawing state management from React state to refs for better synchronization.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 48014a3c-3b30-4c1a-b020-fdb806262062
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Elkr8Ti
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -754,9 +754,23 @@
         <v>done</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B22" t="str">
+        <v>ציור עם עט/אצבע בחלון OCR סטריפים לא עובד — תיקון Pointer Events</v>
+      </c>
+      <c r="C22" t="str">
+        <v>bug</v>
+      </c>
+      <c r="D22" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revert drawing canvas changes to restore pen functionality
Reverts recent modifications to the drawing canvas event handlers in `LearnDigitsOverlay` and `HandwritingOverlay`, restoring previous mouse and touch event listeners to address issues with pen input during transfers.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9466cb59-7d7b-4f3b-a072-80c4d8329b29
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Elkr8Ti
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -768,9 +768,23 @@
         <v>done</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B23" t="str">
+        <v>ביטול תיקון Pointer Events בחלוני ציור OCR — חזרה לגרסה קודמת</v>
+      </c>
+      <c r="C23" t="str">
+        <v>bug</v>
+      </c>
+      <c r="D23" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update project requirements document with new user stories
Update the project-requirements.xlsx file to include newly defined user stories.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 21947361-7988-4f00-818a-d86b9ea98038
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Elkr8Ti
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -782,9 +782,37 @@
         <v>done</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B24" t="str">
+        <v>חילוץ User Stories מכל קומפוננטה — 278 stories, 49 נושאים — מסמך USER_STORIES.md</v>
+      </c>
+      <c r="C24" t="str">
+        <v>documentation</v>
+      </c>
+      <c r="D24" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B25" t="str">
+        <v>העלאת USER_STORIES.md לגיטהאב (levori119/skyboard)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>ci</v>
+      </c>
+      <c r="D25" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update project requirements and add database export
Add metadata for skyking_db_export.zip and update project-requirements.xlsx.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 969c7d32-b1b3-47eb-96bf-a49fb4194a98
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Elkr8Ti
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -810,9 +810,23 @@
         <v>done</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B26" t="str">
+        <v>ייצוא DB ל-ZIP (skyking_db_export.zip)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>export</v>
+      </c>
+      <c r="D26" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add English version of user stories and update asset metadata
Create USER_STORIES_EN.md, add it to agent assets metadata, and update project-requirements.xlsx.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9c8d98c8-c773-49f0-a42a-99313e34759f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Elkr8Ti
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -824,9 +824,23 @@
         <v>done</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="B27" t="str">
+        <v>ייצוא User Stories באנגלית — USER_STORIES_EN.md</v>
+      </c>
+      <c r="C27" t="str">
+        <v>documentation</v>
+      </c>
+      <c r="D27" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add ability to export requirements and issues to Excel
Fix an ESM/CJS conflict in the requirements tracker by updating the skill instructions to use bash instead of code execution. Also, update the underlying script and add new entries to the Excel file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 606367ec-3d2c-4f66-8d98-301084b31ed6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/KpUYcx6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -838,9 +838,60 @@
         <v>done</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-06-17 19:42</v>
+      </c>
+      <c r="B28" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C28" t="str">
+        <v>הוספת נקודות מנהלתיות ואלמנטי שדה לאפליקציית הנהג (driver.html) לאחר בחירת בסיס</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-06-17 19:42</v>
+      </c>
+      <c r="B29" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C29" t="str">
+        <v>בניהול מערכת — קטגוריות בתפריט ימני עולות אחד על השני, תוקן ריווח בין הסקשנים</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-06-17 19:42</v>
+      </c>
+      <c r="B30" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ייצוא דרישות לאקסל לא בוצע — תוקן מעכשיו</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve spacing and visual separation of navigation items
Adjusted padding, line height, and margins in the admin panel sidebar to enhance readability and prevent text overlap.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f9e1c3cd-9088-49f0-971d-fa38d7cefe09
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/ZZiu3Lz
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -889,9 +889,26 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-06-17 19:45</v>
+      </c>
+      <c r="B31" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C31" t="str">
+        <v>תפריט ניהול מערכת — טקסט קטגוריות עדיין צפוף מדי לאחר תיקון ראשון, הוגדל ריווח נוסף</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update project requirements and add visual asset
Updated project requirements documentation and added a new image asset.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ccc22750-a9a4-4da3-bf2c-c4d10444d482
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/ZZiu3Lz
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -906,9 +906,26 @@
         <v/>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-06-17 19:46</v>
+      </c>
+      <c r="B32" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C32" t="str">
+        <v>ביטול יד (גרירת מפה) בעמדה עם מפה — אין צורך בגרירת המפה עצמה</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add inline 🚗 driver toggle on each airfield element and admin-loc point row
- Added `show_in_driver BOOLEAN DEFAULT false` column to `airfield_points` table
- Updated PUT /api/airfield-points/:id to accept and persist show_in_driver
- Added inline 🚗 / 🚗✓ toggle button on each airfield element card in admin panel
  (green when active, gray when inactive; one-click toggle, no form needed)
- Added same inline 🚗 / 🚗✓ toggle button on each admin_loc (נקודות מנהלתיות) row
- Both toggles save immediately via API and update local state without page reload
- airfield_elements already had show_in_driver; now airfield_points also supports it
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -923,9 +923,43 @@
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-06-18 04:00</v>
+      </c>
+      <c r="B33" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C33" t="str">
+        <v>כפתור 🚗 אינליין על כל אלמנט בשדה — טוגל מהיר להצגה/הסרה מתפריט נהג מזדמן</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-06-18 04:00</v>
+      </c>
+      <c r="B34" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C34" t="str">
+        <v>כפתור 🚗 אינליין על כל נקודה מנהלתית — טוגל מהיר להצגה/הסרה מתפריט נהג מזדמן</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add ability to show regular airfield points in driver menu
Add a toggle button to display regular airfield points in the driver's menu by updating the `show_in_driver` field for each point.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0ce0be7d-851e-4266-afbe-d2ea77d6fef4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/Y2fUXgG
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -957,9 +957,26 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-06-18 04:08</v>
+      </c>
+      <c r="B35" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C35" t="str">
+        <v>כפתור 🚗 אינליין על כל נקודה בשדה תעופה (נקודות רגילות) — טוגל מהיר להצגה בתפריט נהג מזדמן</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update driver app to show all relevant points and improve user messaging
Modify the API to return all points with `show_in_driver=true` or `point_type='admin_loc'`, update the driver HTML to display these points in origin/destination dropdowns, and provide clearer user feedback when no points are available.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 792db359-822b-4b9f-8e32-5f0a1c6efe80
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/mXiIiNf
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -974,9 +974,26 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2026-06-18 05:49</v>
+      </c>
+      <c r="B36" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C36" t="str">
+        <v>נקודות בסיס לא מופיעות בתפריט מוצא/הגעה באפליקציית נהג מזדמן — API החזיר רק admin_loc</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix error when accessing vehicle route management page
Correctly initialize and manage vehicle route state by moving declarations to the component level, resolving a React hooks violation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8650efd8-d8cc-4e58-be11-b6b214b0cd2c
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/oFbaWvx
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -991,9 +991,26 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-06-18 05:56</v>
+      </c>
+      <c r="B37" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C37" t="str">
+        <v>בחירת "מסלולי רכב" בניהול מבצעי גרמה למסך כחול — useState/useEffect בתוך IIFE מותנה</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add GPS coordinates to vehicle route waypoints for Google Maps compatibility
When drawing vehicle route waypoints on a calibrated airfield map,
each clicked point now stores lat/lon (decimal degrees) alongside
its image-percentage x/y position.

Changes:
- vehicleRouteDraftPoints state type extended: {x, y, lat?, lon?}
- Map click handler for drawingVehicleRouteId: calls getAnchorFromMapData
  + imagePctToGeo (same pattern as admin location pins) to compute GPS
- GPS fields included automatically in the POST/PUT waypoints JSON payload
- If map is not yet calibrated, waypoints fall back gracefully to x/y only

Result: base_routes.waypoints JSONB now contains [{x,y,lat,lon},...] entries
that can be used directly with Google Maps or any geo-aware consumer.
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1025,9 +1025,26 @@
         <v/>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2026-06-18 10:03</v>
+      </c>
+      <c r="B39" t="str">
+        <v>פיצ׳ר</v>
+      </c>
+      <c r="C39" t="str">
+        <v>נקודות נתיבי נסיעה מכילות נ"צ GPS (lat/lon) כאשר המפה מכויילת — תמיכה ב-Google Maps</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add ability for drivers to update or cancel approved travel requests
Extend the PUT endpoint for vehicle requests to accept additional fields for updates and add functionality to the driver interface for editing request details or canceling them.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ca6ebb9c-e4e0-4a93-9a52-4bae76d3a3a5
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/67dWT08
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1042,9 +1042,26 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2026-06-18 10:10</v>
+      </c>
+      <c r="B40" t="str">
+        <v>פיצ׳ר</v>
+      </c>
+      <c r="C40" t="str">
+        <v>עדכון/ביטול בקשת נסיעה אחרי אישור — כפתורי "עדכן פרטים" ו-"בטל נסיעה" במסך המאושר</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add GPS anchoring indicator to vehicle routes
Update `src/App.tsx` to display a visual indicator next to each vehicle route in the list, showing whether its waypoints are anchored to GPS coordinates.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 886fde01-045e-4001-b67e-53e9165627da
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/67dWT08
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1059,9 +1059,26 @@
         <v/>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-06-18 10:12</v>
+      </c>
+      <c r="B41" t="str">
+        <v>UX</v>
+      </c>
+      <c r="C41" t="str">
+        <v>אינדיקטור ⚓ ליד כל נתיב נסיעה — ירוק=כל הנקודות מעוגנות לנ"צ, צהוב=חלקי, אפור=ללא עיגון</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Display GPS coordinates in degrees, minutes, and seconds format
Add a new div element to driver.html to display GPS coordinates in DMS format and a JavaScript function to convert decimal degrees to DMS. Update `sendGPS` and `requestGPS` to call the new display update function.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d71f4625-ea1c-42f6-9bc5-5ec11f035a49
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/67dWT08
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1076,9 +1076,26 @@
         <v/>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-06-18 10:13</v>
+      </c>
+      <c r="B42" t="str">
+        <v>UX</v>
+      </c>
+      <c r="C42" t="str">
+        <v>אפליקציית נהג — הצגת נ"צ נוכחי בפורמט מעלות דקות שניות ליד אינדיקטור ה-GPS</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E42"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add ability to anchor existing routes and points to GPS coordinates
Add retroactive GPS anchoring functionality to the admin panel for both vehicle routes and airfield points, allowing users to anchor previously unanchored data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0f859e60-4f4c-4152-ae16-640530b9b8ca
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/67dWT08
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1093,9 +1093,26 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-06-18 10:17</v>
+      </c>
+      <c r="B43" t="str">
+        <v>פיצ׳ר</v>
+      </c>
+      <c r="C43" t="str">
+        <v>כפתור "🔁 עגן נ"צ" לנתיבי נסיעה ונקודות שנוצרו לפני כיול — מחשב GPS רטרואקטיבית ע"פ נקודות עיגון המפה</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E43"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix GPS waypoints not passing to driver navigation (lon vs lng mismatch)
Root cause: imagePctToGeo() returns {lat, lon} (no 'g') but openNavigation()
in driver.html filtered by w.lng (with 'g'), causing all GPS-anchored
waypoints to be silently excluded — resulting in the "נקודות המסלול אינן
מכילות קואורדינטות GPS" alert even when routes had valid coordinates.

Fix: normalize both field names at the filter stage using nullish coalescing:
  currentWaypoints.map(w => ({ ...w, _lng: w.lng ?? w.lon })).filter(...)

Both `w.lng` (future/direct input) and `w.lon` (from imagePctToGeo anchor
computation) are now supported. The Google Maps URL uses _lng for both
waypoints string and destination.
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1127,9 +1127,26 @@
         <v/>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2026-06-18 11:39</v>
+      </c>
+      <c r="B45" t="str">
+        <v>באג</v>
+      </c>
+      <c r="C45" t="str">
+        <v>תיקון: נ"צ שנבחרו לנתיב לא עברו לאפלקציית הנהג — openNavigation ב-driver.html בדק w.lng אך imagePctToGeo מחזיר lon (ללא g); תוקן לתמוך בשני הפורמטים</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update driver app to notify about route changes
Modify driver.html to keep polling for route updates after approval and display notifications for route or notes changes, including cancellation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6f6d066f-264d-4984-9a46-07f0a9014824
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/HkF1QCw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1144,9 +1144,26 @@
         <v/>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>2026-06-18 12:27</v>
+      </c>
+      <c r="B46" t="str">
+        <v>פיצ׳ר</v>
+      </c>
+      <c r="C46" t="str">
+        <v>עדכון מסלול נסיעה מעמדת שדה → עדכון מיידי + פופאפ התראה לנהג; ביטול ע"י עמדה → התראה + חזרה לטופס; פולינג נמשך גם לאחר אישור</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add GPS coordinates to approved routes and display them for drivers
Enhance GET /api/vehicle-requests to join with airfields and maps, calculate missing GPS coordinates for waypoints via linear interpolation using anchor points, and display coordinates in DMS format in public/driver.html.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0518db2f-2a52-44a7-8d1d-e7eb86a6beb9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/A20xq58
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1161,9 +1161,26 @@
         <v/>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>2026-06-18 12:32</v>
+      </c>
+      <c r="B47" t="str">
+        <v>באג+פיצ׳ר</v>
+      </c>
+      <c r="C47" t="str">
+        <v>תיקון נ"צ בנתיבי נסיעה: server מחשב GPS לנקודות חסרות ע"פ anchor מפה; driver.html מציג נ"צ DMS ליד כל נקודת מסלול</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E47"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add route plan builder to active vehicle edit panel
The "🗺 בנה מסלול" tab was only in the pending-request approval flow.
Now added to the active-request "עדכן מסלול" panel too.

Changes (App.tsx - GroundVehiclePanel):
- Added activePlanTab: Record<number,'select'|'build'> state — per-request
  tab selection so each active card has its own tab state
- Added updateWithPlan(req) function: same as approveWithPlan but uses PUT
  (no status change) — saves computed route and updates assigned_route_id
- Edit route panel (panel === 'edit') now has two tabs:
  [📋 בחר מסלול] — existing dropdown + notes + save
  [🗺 בנה מסלול] — airfield selector, permission radio (🚗/✈️/🛬),
    from/to point dropdowns, ⚡ חשב מסלול, results with crossing warnings
    and elements list, then "💾 עדכן עם מסלול זה"
- Route dropdown in both tabs now shows [הסעה]/[טיסה] type labels
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1195,9 +1195,26 @@
         <v/>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2026-06-18 13:18</v>
+      </c>
+      <c r="B49" t="str">
+        <v>באג</v>
+      </c>
+      <c r="C49" t="str">
+        <v>הוסף כרטיסיית "🗺 בנה מסלול" גם בפאנל עדכון מסלול של רכב בדרך (לא רק בממתינים)</v>
+      </c>
+      <c r="D49" t="str">
+        <v>GroundVehiclePanel active edit panel</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix X button not closing vehicle panel (pointer capture issue)
Bug: clicking ✕ in the כניסת רכבים (GroundVehiclePanel) draggable
header did nothing.

Root cause: the header div has onPointerDown={onDragStart} which calls
e.currentTarget.setPointerCapture(e.pointerId). This captured all
pointer events on the div, preventing the click from reaching the
child ✕ button.

Fix: added onPointerDown={e => e.stopPropagation()} to the close
button so pointer capture is not set when pressing the X.

Same pattern already used elsewhere in the codebase (e.g. BDH panel
close button at line 5762).
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1246,9 +1246,26 @@
         <v/>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2026-06-18 15:40</v>
+      </c>
+      <c r="B52" t="str">
+        <v>באג</v>
+      </c>
+      <c r="C52" t="str">
+        <v>כפתור X בחלון כניסת רכבים לא סגר את החלון</v>
+      </c>
+      <c r="D52" t="str">
+        <v>GroundVehiclePanel — onPointerDown stopPropagation on close button</v>
+      </c>
+      <c r="E52" t="str">
+        <v>תוקן</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Match active-vehicle build-route form style to pending builder
The permission buttons in the "בנה מסלול" tab of the active vehicle
edit panel showed only emojis (🚗 / ✈️ / 🛬) with tiny 9px text.
User asked them to match the pending-request plan builder style.

Changes (App.tsx — active plan builder, aTab === 'build'):
- Permission buttons: added text labels → "🚗 כביש" / "✈️ הסעה" / "🛬 טיסה"
- Added description line below buttons (e.g. "כבישים + מסלולי הסעה")
- Added "הרשאת נסיעה:" label above buttons
- From/To selects: added "מ:" / "אל:" labels, increased padding/font-size
- Added "שדה תעופה:" label above airfield selector
- Button text: "⚡ חשב מסלול מהיר" (was "⚡ חשב מסלול")
- Sizes/radii aligned with the pending builder for visual consistency
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1263,9 +1263,26 @@
         <v>תוקן</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2026-06-18 17:31</v>
+      </c>
+      <c r="B53" t="str">
+        <v>שיפור UI</v>
+      </c>
+      <c r="C53" t="str">
+        <v>כפתורי הרשאת נסיעה בטופס בנה מסלול (עדכון רכב פעיל) — עם טקסט ולא רק אייקונים, זהה לטופס הממתינים</v>
+      </c>
+      <c r="D53" t="str">
+        <v>GroundVehiclePanel active build tab</v>
+      </c>
+      <c r="E53" t="str">
+        <v>תוקן</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E53"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add automatic map loading for approved driver requests
Update server to return route airfield and map IDs, and modify driver interface to auto-select and display the correct airfield map upon approval.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: fad668c2-758d-4b8c-bacc-7c9c322e3332
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/6yBnGRF
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1280,9 +1280,26 @@
         <v>תוקן</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2026-06-19 11:15</v>
+      </c>
+      <c r="B54" t="str">
+        <v>פיצ׳ר</v>
+      </c>
+      <c r="C54" t="str">
+        <v>מוד נהג (driver.html) — טעינה אוטומטית של מפת שדה התעופה של העמדה שאישרה את כניסת הרכב</v>
+      </c>
+      <c r="D54" t="str">
+        <v>driver.html + server.js GET /api/vehicle-requests</v>
+      </c>
+      <c r="E54" t="str">
+        <v>בוצע</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E54"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add prominent notification for arriving vehicles in the management panel
Introduce a new state `newlyArrived` and a useEffect hook in `GroundVehiclePanel` to detect requests transitioning to 'arrived' status. Displays a flashing notification banner at the top of the panel for these vehicles, with a dismiss button.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9b9809af-2bd9-4c9b-ad48-3c1e0e578692
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/6yBnGRF
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1297,9 +1297,26 @@
         <v>בוצע</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>2026-06-19 11:41</v>
+      </c>
+      <c r="B55" t="str">
+        <v>פיצ׳ר</v>
+      </c>
+      <c r="C55" t="str">
+        <v>כשנהג מסמן הגעה ליעד — באנר התראה בולט מופיע בפאנל כניסת רכבים בעמדת ניהול שדה התעופה</v>
+      </c>
+      <c r="D55" t="str">
+        <v>GroundVehiclePanel — newlyArrived state + detection + UI banner</v>
+      </c>
+      <c r="E55" t="str">
+        <v>בוצע</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E55"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update vehicle request system to support multiple permissions and display driver GPS
Enhance vehicle request system with multi-permission support in `server.js` and `src/App.tsx`. Modify API endpoint to accept `permissions` array and update UI to handle multi-select toggle buttons. Extend GPS polling to include pending requests and display driver GPS and destination in the pending panel. Add `segmentPath` and `excludedRouteTypes` to route plan results.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: bd434133-bf04-4919-9f9f-1565549ecac9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/6yBnGRF
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:F56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1314,9 +1314,29 @@
         <v>בוצע</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Vehicle Approval Panel</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Multi-select route permissions (vehicle/taxiways/runways combinable), segmentPath with L/R turn directions in route results, excludedRouteTypes shown in UI, driver GPS + destination shown in pending approval panel, GPS polling extended to pending requests</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F56" t="str">
+        <v>server.js + App.tsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F56"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Automatically populate vehicle request details and filter routes by base
Adds database columns for origin/destination points and base ID. Enhances the vehicle request form and API to store this data. Implements auto-population of route planning fields when a request is selected, including filtering routes by the selected base and triggering an immediate route calculation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 46695e51-6295-4505-906d-ffcd66562d36
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/NqSBPM5
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1334,9 +1334,29 @@
         <v>server.js + App.tsx</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Vehicle Approval Panel</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Bug: route calc fails left panel; Auto-fill from/to from driver selection; Auto-select airfield from base; Show routes from all base maps. Fix: store from_point_id+to_point_id+base_id in vehicle_requests, driver.html sends IDs, GET returns point airfield_id via JOIN, auto-populate effect in App.tsx, auto-trigger buildPlan</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F57" t="str">
+        <v>server.js+driver.html+App.tsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F57"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update route calculation to use all airfield defined route types
Update auto-route calculation to include 'taxiways' and 'runways' in permissions, aligning with airfield operational settings.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a729f03f-4e49-4c1d-8e9e-2679c85e6020
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/NqSBPM5
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1354,9 +1354,77 @@
         <v>server.js+driver.html+App.tsx</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2026-06-19 12:51</v>
+      </c>
+      <c r="B58" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Auto-populate שדה/מוצא/יעד לא עבד — נראה אותו דבר (בקשות ישנות ללא IDs)</v>
+      </c>
+      <c r="D58" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2026-06-19 12:51</v>
+      </c>
+      <c r="B59" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C59" t="str">
+        <v>חישוב מסלול נכשל כי "מסלולי מטוסים" נכנס ל-permissions בטעות</v>
+      </c>
+      <c r="D59" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2026-06-19 12:51</v>
+      </c>
+      <c r="B60" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C60" t="str">
+        <v>חישוב מסלול נכשל — START_RADIUS=300m קטן מדי לנקודות רחוקות (תחילת 15 = 1218m)</v>
+      </c>
+      <c r="D60" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2026-06-19 12:51</v>
+      </c>
+      <c r="B61" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C61" t="str">
+        <v>חישוב מסלול אוטומטי ישתמש בכל סוגי הנתיבים של השדה (רכב+הסעה+מסלולים)</v>
+      </c>
+      <c r="D61" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F61"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new features for planning vehicle routes and displaying them on a map
Update database schema to include `via_route_ids` and `show_on_map` columns for vehicle requests. Modify the API to accept and save these new fields. Enhance the UI to allow users to select pre-defined routes or calculate GPS routes, and to toggle the visibility of routes on the map.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 3de6b9f0-d7c5-4887-92cc-91045063faae
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/gcHILtX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1422,9 +1422,60 @@
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-06-19 13:10</v>
+      </c>
+      <c r="B62" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C62" t="str">
+        <v>הוספת ממשק ניווט מלא לפאנל אישור בקשות רכבים — נתיבים פנויים/לא שמישים/חסומים עם "החל", לחצני קטגוריה, רצף נבחר</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-06-19 13:10</v>
+      </c>
+      <c r="B63" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C63" t="str">
+        <v>הוספת שדה via_route_ids ו-show_on_map לטבלת vehicle_requests (DB + API PUT)</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2026-06-19 13:10</v>
+      </c>
+      <c r="B64" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C64" t="str">
+        <v>הוספת טוגל "הצג על מפה" (show_on_map) בפאנל בניית מסלול לבקשות רכבים</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update internal notepad label to internal note
Change the "📄 פתקית" label to "📄 פתקית פנימית" in both the button and panel title within the workstation component.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b0c255de-7998-4c86-90a7-12c868201d3f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/gcHILtX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1473,9 +1473,26 @@
         <v/>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>2026-06-19 13:41</v>
+      </c>
+      <c r="B65" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C65" t="str">
+        <v>שינוי כיתוב כפתור ופאנל "פתקית" ל-"פתקית פנימית" בעמדה</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F65"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix build errors and remove unused code for smoother deployment
Addresses TypeScript errors by adding type assertions, removing invalid SVG attributes, and correcting missing properties in form data. Also removes a dead code block related to route management.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 85a81593-c385-4dbf-8cd2-e365fb11cf65
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/gcHILtX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1490,9 +1490,26 @@
         <v/>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>2026-06-19 13:52</v>
+      </c>
+      <c r="B66" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Build לפרסום נכשל — שגיאות TypeScript: draggable ב-SVG, show_in_driver חסר, route_type חסר, קוד מת עם פונקציות לא מוגדרות</v>
+      </c>
+      <c r="D66" t="str">
+        <v>✓</v>
+      </c>
+      <c r="E66" t="str">
+        <v>תוקן — 6 שגיאות TypeScript</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F66"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add texture options for strip backgrounds
Introduce background texture selection for strip windows, enhancing visual customization.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c0d01341-754a-488d-ac6b-774f67623ecb
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/dx7e7JX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1507,9 +1507,26 @@
         <v>תוקן — 6 שגיאות TypeScript</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-06-19 14:41</v>
+      </c>
+      <c r="B67" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C67" t="str">
+        <v>הגדרת חלון סטריפים — אפשרות בחירת מרקם רקע (9 מרקמים: נקודות, גריד, אלכסוני, קווים, רשת, לוח שחמט)</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F67"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add waypoint mode to sector strips and visual indicators
Implement waypoint filtering logic for incoming and outgoing transfers in `src/App.tsx` and update `project-requirements.xlsx`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2b955241-bc34-4083-93c2-7618385b6af8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/dx7e7JX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1524,9 +1524,29 @@
         <v/>
       </c>
     </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Strip window (חלון סטריפים) — per-leaf waypoint mode: מקבל (📥 incoming from sector) or מוסר (📤 outgoing to sector). Filtering logic: מוסר shows outgoingTransfers matching the waypoint sector, מקבל shows incomingTransfers from that sector. Query applied on top. Mode indicator shown in header of both admin preview and workstation view.</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F68" t="str">
+        <v>SWLeaf.waypoint_mode added; admin UI toggle buttons; leafStrips logic updated</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F68"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add waypoint name and transfer mode to strip window headers
Update the `SectorDashboard` component in `src/App.tsx` to display the waypoint name and transfer mode (incoming/outgoing) alongside the existing label in the strip window headers.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a149577d-b316-4b87-bed5-b6c1d0f66de9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/dx7e7JX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1544,9 +1544,29 @@
         <v>SWLeaf.waypoint_mode added; admin UI toggle buttons; leafStrips logic updated</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Improvement</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Strip window leaf header: always show waypoint sector name + מקבל/מוסר badge alongside the label. Previously the label hid the waypoint name.</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F69"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add customizable content headers to strip cells for better organization
Update SWLeaf interface to include content_title and related styling properties, add a new section in the admin editor for configuring these properties, and implement rendering logic to display the content title within the workstation leaf body.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5c05d4ad-defe-44d4-88a7-bdd7978f4182
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/dx7e7JX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1564,9 +1564,29 @@
         <v/>
       </c>
     </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Strip window leaf: add configurable content title (📝 כותרת תוכן) displayed above the strips list. Controls: text, text color, background color, font size (10-36px), bold toggle, alignment (right/center/left). Stored in SWLeaf.content_title* fields.</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F70"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add a way to duplicate strip window layouts with all their settings
Add a "duplicate" button to the strip window admin interface that creates a copy of an existing layout. This includes duplicating the layout's name, JSON configuration, and all associated settings.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 35569f78-e076-4f90-805b-e008c5d685c1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/dx7e7JX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1584,9 +1584,29 @@
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Strip window admin: add 📋 duplicate button per layout. Creates copy named "[original] — עותק", auto-selects it. Handles name collision with alert.</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F71"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Make waypoint mode more visible in strip windows
Update the rendering of waypoint mode indicators in strip windows to display as prominent, styled badges with larger text and distinct background colors, improving readability.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d52f34b5-dd91-412c-921d-107625c14c87
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/dx7e7JX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1604,9 +1604,29 @@
         <v/>
       </c>
     </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Improvement</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Strip window: waypoint mode (מקבל/מוסר) now shown as a prominent colored banner bar between the cell header and strips list — green for מקבל, orange for מוסר. Removed small badge from header bar.</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F72"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correctly display sector names in strip window workstations
Fix a reference error by replacing `swSectors` with `allSectors` when looking up sector names in the workstation rendering component.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 28d25a5f-0559-4a38-a995-a38391d56eec
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1624,9 +1624,29 @@
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Strip window workstation crash: swSectors (admin-only var) used in workstation rendering — replaced with allSectors (main component state). Caused ReferenceError on any strip window workstation load.</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Fixed</v>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F73"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add strip transfer and acceptance functionality
Add strip transfer logic to 'מוסר' cells, acceptance button to 'מקבל' cells, and a transfer picker dialog for multi-workstation sectors.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 95b3393b-f4d8-46d0-a1cd-484aadb2245c
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1644,9 +1644,29 @@
         <v/>
       </c>
     </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Strip window — מוסר cell: drag strip onto cell → triggers handleTransfer to the waypoint sector; if multiple workstations on that sector → picker dialog asks which one. מקבל cell: each strip shows ✅ קבל פמ"מ button that calls handleAcceptTransfer. Cannot drag onto a מקבל cell.</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F74"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ensure workstation selection text is always black
Add explicit text color to workstation selection dropdown to prevent blue default

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1d6f05c1-53d5-474f-a7d6-5046bf72cbdd
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1664,9 +1664,29 @@
         <v/>
       </c>
     </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D75" t="str">
+        <v>מסך כניסה — תפריט בחירת עמדה: טקסט מופיע כחול במקרים מסוימים. תוקן ע"י הוספת color: #0f172a לסלקט</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F75"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Filter crew members to show only those approved for the current workstation
Modify `loadCrewMembers` in `src/App.tsx` to filter `availableCrewMembers` based on `session.presetId`, `cm.is_admin`, and `cm.approved_workstations`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 098e2c3e-9555-49fd-80f4-1202cf904452
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1684,9 +1684,29 @@
         <v/>
       </c>
     </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D76" t="str">
+        <v>החלפת משתמש בעמדה — מציג רק משתמשים עם הרשאה לעמדה הנוכחית (approved_workstations). מנהלים ומשתמשים ללא הגבלה תמיד מוצגים.</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F76"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve strip visibility and automate transfer acceptance
Update the strip display logic to ensure visibility after transfers and automatically accept incoming transfers via drag-and-drop.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 574e6405-b7ad-4189-b2c0-4bafc3851c22
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1704,9 +1704,29 @@
         <v/>
       </c>
     </row>
+    <row r="77">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Bug+Feature</v>
+      </c>
+      <c r="D77" t="str">
+        <v>חלון סטריפים — (1) תא מוסר: סטריפ שהועבר נשאר גלוי בתא (תוקן: מקור strips במקום myTableStrips + swLeafAssign מיידי). (2) תא מקבל: גרירה לתא אחר = קבלה אוטומטית של ההעברה, ללא צורך בכפתור נפרד.</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F77"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve workstation selection when transferring items
Update logic to ensure a workstation picker appears with a fallback to all available workstations when specific transfer candidates are not found, and fix the contacts summary to correctly identify the target workstation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 832b0269-df86-49f7-82e2-c76d1dcaf4b4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1724,9 +1724,29 @@
         <v/>
       </c>
     </row>
+    <row r="78">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D78" t="str">
+        <v>חלון סטריפים מוסר: (1) picker עמדות לא הופיע כשהפילטר הספציפי (relevant_sectors) לא מצא — כעת fallback לכל העמדות האחרות. (2) ריכוז קשרים הציג כל העמדות (targetPid=null) — תוקן באותו fallback. שני התיקונים ב-onDrop וב-handleTransfer.</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F78"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Move recipient and sender indicators to the header row
Integrates the 'מוסר'/'מקבל' (sender/recipient) badges into the header div of the strip window leaf component, repositioning them to the right side and removing the separate banner divs.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4379c0f9-62c4-45df-831a-15cca9727d84
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1744,9 +1744,29 @@
         <v/>
       </c>
     </row>
+    <row r="79">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C79" t="str">
+        <v>UI</v>
+      </c>
+      <c r="D79" t="str">
+        <v>חלון סטריפים — תג מוסר/מקבל הועבר מבאנר נפרד מתחת לכותרת לתוך שורת הכותרת עצמה (צד ימין)</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F79"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Prevent dragging of transferred strips outside of the receiving cell
Update drag-and-drop logic to disable dragging for strips with 'pending_transfer' status, except when they are within the 'receiving' cell, ensuring proper transfer handling.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0bd7b225-262e-4312-ba51-d7f1a11b7838
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1764,9 +1764,29 @@
         <v/>
       </c>
     </row>
+    <row r="80">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D80" t="str">
+        <v>חלון סטריפים — סטריפ שנמסר (pending_transfer) לא ניתן לגרירה חזרה ללוח. רק תא מקבל מאפשר גרירה של pending_transfer (כי שם גרירה = קבלה).</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F80"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Allow dragging transferred strips to cancel outgoing transfers
Revert restriction on dragging pending_transfer strips and add API call to cancel outgoing transfers when dropped on a regular cell.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 519e51e5-6f78-4bc4-b5b9-4a8a0c180a0e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1784,9 +1784,29 @@
         <v/>
       </c>
     </row>
+    <row r="81">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D81" t="str">
+        <v>חלון סטריפים — גרירת סטריפ שנמסר (pending_transfer) לתא רגיל מבטלת העברה דרך API (/transfers/:id/cancel). גרירה שוב מאופשרת לכל הסטריפים.</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F81"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refine workstation selection for transfers to specific sectors
Update logic to correctly filter and display available workstations when performing transfers, ensuring only relevant workstations are presented or the transfer proceeds directly if no specific matches are found.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 36253229-1d9e-4295-9fa0-fdb1ba39f18d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1804,9 +1804,29 @@
         <v/>
       </c>
     </row>
+    <row r="82">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D82" t="str">
+        <v>חלון סטריפים — picker עמדות בתא מוסר הציג כל העמדות כשלא היו מתאימות ספציפיות. תוקן: אין fallback לכולם — מציג רק עמדות עם relevant_sectors/classic_receive_points מתאים לסקטור. אם 0 → שלח ללא יעד, 1 → שלח ישירות, 2+ → picker. גם תוקן ב-contacts targetPid.</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F82"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Enable reordering of strips within the same window cell
Add drag-and-drop reordering functionality for strips within the same leaf cell, along with associated state management and UI feedback.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 21fc78b0-5ae9-475c-8260-e89bdfb1bc9d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1824,9 +1824,29 @@
         <v/>
       </c>
     </row>
+    <row r="83">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D83" t="str">
+        <v>חלון סטריפים — גרירה בתוך אותו תא משנה סדר (swLeafOrder). קו כחול מציין נקודת הכנסה. תאי מוסר/מקבל לא מושפעים.</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F83"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve contacts summary display logic when transferring items
Conditionally open the contacts summary panel only when a specific target workstation ID is available, preventing the display of all related workstations when the target is ambiguous.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 52370272-085a-41cc-acde-3a53fd91e136
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1844,9 +1844,29 @@
         <v/>
       </c>
     </row>
+    <row r="84">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D84" t="str">
+        <v>פאנל קשרים נפתח אוטומטית עם כל העמדות כשלא זוהתה עמדת יעד ספציפית. תוקן: פאנל נפתח רק כשיש targetPid ידוע.</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F84"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve contacts panel to show relevant workstations when multiple matches exist
Update contacts panel logic to handle multiple specific workstation matches by introducing `contactsSummarySpecificIds` state and updating filtering to prioritize specific matches when present.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 46c58b18-b7bd-4130-afd9-7dc6a209ab39
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1864,9 +1864,29 @@
         <v/>
       </c>
     </row>
+    <row r="85">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D85" t="str">
+        <v>פאנל קשרים אחרי העברה: כשיש מספר עמדות מחוברות לסקטור, מציג רק את הקשרים של אותן עמדות ספציפיות (לא כל העמדות). הוספת state contactsSummarySpecificIds.</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F85"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Make drawing on the background visible when pen mode is off
Adjust z-index of the drawing canvas to ensure strokes are visible behind content.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 22fbd08a-6ebd-4646-b508-518dd5083dc0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/shxOTxw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1884,9 +1884,29 @@
         <v/>
       </c>
     </row>
+    <row r="86">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Bug</v>
+      </c>
+      <c r="D86" t="str">
+        <v>חלון סטריפים — ציורי עט על הרקע (לא על פמ) נעלמו כשכובה מצב עט. תוקן: canvas נשאר zIndex:5 גם כשכבוי (מעל content div zIndex:2), עם pointerEvents:none.</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F86"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve drawing functionality by ensuring strokes are saved and visible
Add a stable redraw function and effects to persist strokes, and increase canvas z-index to ensure visibility.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b54bb025-f060-4434-9dd4-09866d38a2d8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/5Q2mJ3g
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1904,9 +1904,29 @@
         <v/>
       </c>
     </row>
+    <row r="87">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="D87" t="str">
+        <v>חלון סטריפים: ציורי רקע (pen strokes on background) לא נשמרים / מוצגים מתחת לרקע</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Fixed: added stable swDoRedraw useCallback + useEffect on swStrokes+swPenMode change; bumped canvas zIndex to 15 when pen-mode off</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F86"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F87"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve canvas drawing by removing duplicates and deferring redraws
Removes a duplicate useEffect that caused redraw issues and defers canvas redraws using requestAnimationFrame to ensure layout is complete before drawing.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ee44471d-80d4-4124-8cbe-3a156c85a8d2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/5Q2mJ3g
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1924,9 +1924,29 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="D88" t="str">
+        <v>חלון סטריפים: ציורי רקע לא תמיד נשמרים על התא</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Removed duplicate redraw useEffect; upgraded swDoRedraw to use requestAnimationFrame so layout completes before canvas is measured+drawn</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F88"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Allow users to freely position items within a cell and improve drawing reliability
Implement absolute positioning for items within cells, enabling free drag-and-drop placement with overlap prevention, and optimize canvas drawing by using requestAnimationFrame.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2a00864a-97f6-4e67-bece-1d134a44d40c
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/5Q2mJ3g
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1944,9 +1944,29 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D89" t="str">
+        <v>חלון סטריפים: גרירת פמ"מ חופשית בתוך תא (מיקום חופשי, לא רשימה)</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Free absolute positioning per strip per leaf (swFreePos). Drag within same cell sets Y position; collision avoidance prevents overlap; blue line indicator; persisted to localStorage.</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F88"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F89"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add buttons to align strips to the top or bottom within cells
Adds two buttons to the strip window header allowing users to align all strips to the top or bottom of their cell.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e695ca73-fcc7-437d-bf86-cc0bf286666a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/5Q2mJ3g
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1964,9 +1964,29 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D90" t="str">
+        <v>חלון סטריפים: כפתורי יישור פמ"מ למעלה/למטה בכותרת כל תא</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Added ⬆ and ⬇ buttons in each leaf header — ⬆ snaps all strips to top (stacked from y=4), ⬇ snaps to bottom of cell using clientHeight</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F89"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F90"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve drawing functionality by making strokes save reliably
Remove requestAnimationFrame from drawing redraw function and add a guard to prevent clearing the canvas mid-stroke.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 522c92a2-349e-4547-9c5e-6598808de841
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/5Q2mJ3g
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F91"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1984,9 +1984,29 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="91">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="D91" t="str">
+        <v>עט ברקע חלון סטריפים - קווים לא נשמרים</v>
+      </c>
+      <c r="E91" t="str">
+        <v>הוסר requestAnimationFrame מ-swDoRedraw (useEffect כבר רץ אחרי layout). הוסף guard: אם swIsDrawing.current=true מדלג על clear+redraw כדי לא למחוק ציור פעיל</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F90"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F91"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add flight direction and current workstation fields to strips
Adds `flight_direction` and `workstation_preset_name` fields to the strip display and data handling, including server-side modifications and UI updates in App.tsx.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 186567cb-fa89-4664-af11-bf9d5d884cce
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/ssEgJhI
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F92"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2004,9 +2004,29 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D92" t="str">
+        <v>שדות חדשים לפמ"מ: הועבר לעמדה + כיוון פ"מ</v>
+      </c>
+      <c r="E92" t="str">
+        <v>הועבר לעמדה: שם עמדה מ-workstation_preset_id (JOIN בשרת). כיוון פ"מ: מחושב מ-coord_n של בסיס המראה vs בסיס נחיתה — דרומה/צפונה. זמין בכל תצוגות הסטריפ, בפילטרים ובשורות ה-table mode</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F92"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update aviation base coordinates to use degrees, minutes, and seconds format
Refactors aviation base coordinate input from decimal degrees to a Degrees-Minutes-Seconds (DMS) format, including utility functions for conversion and display, and updates the admin form state and save logic accordingly.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 876b2fb8-71bf-4ae0-a84f-4a55a90ca093
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/ssEgJhI
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2024,9 +2024,29 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="D93" t="str">
+        <v>הזנת נ"צ בסיס בפורמט מעלות-דקות-שניות</v>
+      </c>
+      <c r="E93" t="str">
+        <v>טופס "✈️ בסיסים" ב-admin: שדות coord_n/coord_e הוחלפו ב-3 תתי-שדות לכל קואורדינטה (מעלות/דקות/שניות). המרה ל-decimal בשמירה, המרה מ-decimal בעריכה. תצוגת הרשימה מציגה פורמט 32°15′30″N</v>
+      </c>
+      <c r="F93" t="str">
+        <v>Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F93"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Migrate all Replit DB data to Neon PostgreSQL
- Discovered and created 8 missing tables in Neon (system_defaults, az_maps,
  az_polygons, az_airports, az_polygon_status, az_status_log, airfield_polygons,
  airfield_polygon_statuses, airfield_sectors, airfield_status_types)
- Added 2 missing columns to crew_members (classic_display_prefs, can_access_aerozone)
- Added 2 missing columns to strip_transfers (eta_minutes, eta_set_at)
- Dropped all 114 FK constraints in Neon temporarily to allow unordered bulk import
- Fixed JSONB serialization issue causing workstation_presets and strips to fail
- Migrated 86 tables / 4,404 rows from Replit DB → Neon with 100% match
- Reset all sequences in Neon after import
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2044,9 +2044,26 @@
         <v>Done</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>2026-06-21 06:27</v>
+      </c>
+      <c r="B94" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C94" t="str">
+        <v>ייצוא מלא של כל ה-DB מ-Replit ל-Neon — 86 טבלאות, 4,404 שורות</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restore connection to local Replit database
Update server.js to revert to using DATABASE_URL for connection, removing NEON_DATABASE_URL and associated SSL configuration.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad872c0f-5dfe-4539-bc20-d8087900bc82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 301a2ee7-aca6-4b9d-9d2d-4769ab455b5d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9bbed040-b74e-48a6-884f-ca00b37e4051/ad872c0f-5dfe-4539-bc20-d8087900bc82/qR2aEPX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2061,9 +2061,26 @@
         <v/>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>2026-06-21 06:30</v>
+      </c>
+      <c r="B95" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C95" t="str">
+        <v>החזרת חיבור DB ל-Replit המקומי (ביטול Neon)</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F95"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add vitest test suite for pure utils + portable requirements-tracker
Tests: 54 unit tests across strips, queryBuilder, geo, notes, aircraft — validate the refactor extraction preserved behavior. Added npm test / test:watch.
Tooling: portable requirements-tracker skill (relative path, works locally + Replit); backfilled session requests into project-requirements.xlsx.
Docs: README/DEV_GUIDE/REFACTOR_LOG updated with test workflow.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F110"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2078,9 +2078,264 @@
         <v/>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>2026-06-21 08:00</v>
+      </c>
+      <c r="B96" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C96" t="str">
+        <v>יצירת CLAUDE.md עם הנחיות והעקרונות של הפרויקט</v>
+      </c>
+      <c r="D96" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>2026-06-21 08:30</v>
+      </c>
+      <c r="B97" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C97" t="str">
+        <v>ניתוח מעמיק של הקוד וה-DB (Neon) + המלצות להמשך</v>
+      </c>
+      <c r="D97" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>2026-06-21 09:00</v>
+      </c>
+      <c r="B98" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C98" t="str">
+        <v>הגדרת סקילים לצוות (PM/QA/Arch/...) + המלצות</v>
+      </c>
+      <c r="D98" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2026-06-21 09:15</v>
+      </c>
+      <c r="B99" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C99" t="str">
+        <v>יצירת כל הסקילים תחת .claude/skills/</v>
+      </c>
+      <c r="D99" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>2026-06-21 10:00</v>
+      </c>
+      <c r="B100" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C100" t="str">
+        <v>ארגון מחדש של הקוד וה-DB + לוג מעקב (REFACTOR_LOG) + QA</v>
+      </c>
+      <c r="D100" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>2026-06-21 11:00</v>
+      </c>
+      <c r="B101" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C101" t="str">
+        <v>פיצול server.js (8,075 שורות) ל-server/db + server/routes + app.js</v>
+      </c>
+      <c r="D101" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>2026-06-21 12:00</v>
+      </c>
+      <c r="B102" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C102" t="str">
+        <v>תחילת פיצול App.tsx — types/utils/shared components</v>
+      </c>
+      <c r="D102" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>2026-06-22 09:00</v>
+      </c>
+      <c r="B103" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C103" t="str">
+        <v>המשך פיצול App.tsx — חילוץ כל ה-views וה-components (41,625→728 שורות)</v>
+      </c>
+      <c r="D103" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>2026-06-22 11:00</v>
+      </c>
+      <c r="B104" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C104" t="str">
+        <v>תיעוד מלא + קטלוג מודולים (SERVICES.md) + הגדרות לכל מודול</v>
+      </c>
+      <c r="D104" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>2026-06-22 12:00</v>
+      </c>
+      <c r="B105" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C105" t="str">
+        <v>הוספת README + DEV_GUIDE (onboarding/מילון/FAQ) לפי best practices</v>
+      </c>
+      <c r="D105" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2026-06-22 12:30</v>
+      </c>
+      <c r="B106" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C106" t="str">
+        <v>יצירת סקיל /sync-docs לסנכרון אוטומטי של התיעוד</v>
+      </c>
+      <c r="D106" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2026-06-22 12:45</v>
+      </c>
+      <c r="B107" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C107" t="str">
+        <v>הוספת Stop hook שמזכיר לסנכרן תיעוד כשקוד משתנה</v>
+      </c>
+      <c r="D107" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>2026-06-22 13:00</v>
+      </c>
+      <c r="B108" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Commit + push של כל העבודה ל-GitHub (main)</v>
+      </c>
+      <c r="D108" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2026-06-22 13:30</v>
+      </c>
+      <c r="B109" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C109" t="str">
+        <v>תיקון requirements-tracker לנתיב יחסי (portable) + השלמת בקשות שלא נרשמו</v>
+      </c>
+      <c r="D109" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>2026-06-22 14:00</v>
+      </c>
+      <c r="B110" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C110" t="str">
+        <v>הוספת תשתית בדיקות (vitest) + בדיקות יחידה ל-utils הטהורים</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F110"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix: API 404 — app.js double-prefixed /api on router mounts
Routes define full /api/* paths, but app.js mounted them at app.use('/api', router) → effective /api/api/*. Mount at root instead. Verified: /api/sectors and /api/crew-members return 200. Also added concurrently for cross-platform 'npm run dev'.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2333,9 +2333,26 @@
         <v/>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>2026-06-22 15:30</v>
+      </c>
+      <c r="B111" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C111" t="str">
+        <v>API החזיר 404 — app.js הכפיל קידומת /api (mount /api + route /api). תוקן: mount ב-root</v>
+      </c>
+      <c r="D111" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F111"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix: BDH alerts not delivered to other workstations (timezone bug)
bdh_alerts.created_at was 'timestamp without time zone'. When the server runs outside UTC (e.g. Israel UTC+3), pg reads the naive value as local time, shifting created_at ~3h earlier. The recipient's 'created_at >= sessionStart' (UTC) filter then dropped every fresh alert. Converted column to timestamptz (guarded, one-time, interpreting existing values as UTC). Verified: alert now passes the filter.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F114"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2350,9 +2350,60 @@
         <v/>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>2026-06-22 17:10</v>
+      </c>
+      <c r="B112" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C112" t="str">
+        <v>live-runway-conflicts / active-takeoffs קרסו על aircraft_positions שאינו מערך (44 rows)</v>
+      </c>
+      <c r="D112" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E112" t="str">
+        <v>SQL הוקשח עם jsonb_typeof guard</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>2026-06-22 17:15</v>
+      </c>
+      <c r="B113" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C113" t="str">
+        <v>המערכת איטית — polling אגרסיבי מול Neon (כ-20 טיימרים)</v>
+      </c>
+      <c r="D113" t="str">
+        <v>בתהליך</v>
+      </c>
+      <c r="E113" t="str">
+        <v>אובחן; פתרון מלא WebSocket</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>2026-06-22 17:25</v>
+      </c>
+      <c r="B114" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C114" t="str">
+        <v>הפצת התראת בד"ח לעמדה אחרת לא הגיעה — created_at היה timestamp ללא tz, הוסט 3ש בשרת מקומי</v>
+      </c>
+      <c r="D114" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E114" t="str">
+        <v>הומר ל-timestamptz</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F111"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F114"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Perf: throttle aggressive polling + harden pg Pool
loadData (strips/global + classic transfers) 1500ms->5000ms; workstation-messages + collab sync 3000ms->6000ms (kept 1000ms local countdown tick). pg Pool: max 12, idleTimeoutMillis 30s, connectionTimeoutMillis 10s, pool error handler — prevents indefinite hang when pool saturates and recovers Neon dead connections. QA: tsc + 68 tests + build + 22-endpoint smoke (all 200) + 60 concurrent requests (no pool exhaustion).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2401,9 +2401,26 @@
         <v>הומר ל-timestamptz</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>2026-06-22 17:45</v>
+      </c>
+      <c r="B115" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C115" t="str">
+        <v>תיקון איטיות — האטת polling אגרסיבי + הקשחת pg Pool, + QA מקיף</v>
+      </c>
+      <c r="D115" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E115" t="str">
+        <v>QA: tsc/68 tests/build/smoke 22 endpoints/עומס 60 מקבילות</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F114"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F115"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Timezone audit: convert all timestamp columns to timestamptz + shared-language services doc
init.js: dynamic guarded migration converts every 'timestamp without time zone' column (excl. az_* legacy) to timestamptz on startup, interpreting existing values as UTC. Prevents 3h time shift when server runs outside UTC. Added SHARED_LANGUAGE.md (19 domain services mapped to code) + CLAUDE.md references and timezone convention.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F118"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2418,9 +2418,60 @@
         <v>QA: tsc/68 tests/build/smoke 22 endpoints/עומס 60 מקבילות</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>2026-06-22 17:55</v>
+      </c>
+      <c r="B116" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Audit timezone — המרת כל עמדות הזמן ל-timestamptz (migration דינמי מוגן ב-init.js)</v>
+      </c>
+      <c r="D116" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E116" t="str">
+        <v>רץ ב-restart; az_* לא נכלל</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>2026-06-22 18:00</v>
+      </c>
+      <c r="B117" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C117" t="str">
+        <v>מסמך שפה משותפת (SHARED_LANGUAGE.md) — 19 שירותים בשם עסקי + מיפוי לקוד</v>
+      </c>
+      <c r="D117" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>2026-06-22 18:05</v>
+      </c>
+      <c r="B118" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C118" t="str">
+        <v>חיבור ל-Railway (deployment) — בירור</v>
+      </c>
+      <c r="D118" t="str">
+        <v>בתהליך</v>
+      </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F115"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F118"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add /feature worktree workflow + VERIFY/TDD working principle (research-backed)
/feature skill: per-feature git worktree (filesystem isolation) for parallel agents, following the 2026 playbook — plan, shared contracts, ownership split, isolate, test per worker, final merged validation. TDD-first per Anthropic guidance. settings.json: worktree.symlinkDirectories=[node_modules] for instant worktrees. CLAUDE.md: VERIFY-per-online-best-practice + TDD principle.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F120"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2469,9 +2469,43 @@
         <v/>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>2026-06-22 18:20</v>
+      </c>
+      <c r="B119" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Feature workflow (/feature) ב-worktree למקביליות סוכנים + settings symlink</v>
+      </c>
+      <c r="D119" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E119" t="str">
+        <v>מבוסס best practices online</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>2026-06-22 18:25</v>
+      </c>
+      <c r="B120" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C120" t="str">
+        <v>עיגון VERIFY+TDD כעיקרון עבודה (חקר online, לא להמציא) — memory+CLAUDE</v>
+      </c>
+      <c r="D120" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F118"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F120"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Prep repo for Railway deployment
Added start script (node server.js), railway.json (nixpacks build/start), DEPLOY.md runbook. Verified locally: NODE_ENV=production server serves SPA at / and API at /api on the same origin (Railway simulation). server already binds process.env.PORT.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F121"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2503,9 +2503,26 @@
         <v/>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>2026-06-22 18:35</v>
+      </c>
+      <c r="B121" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C121" t="str">
+        <v>הכנת הרפו ל-Railway (start script + railway.json + DEPLOY.md), אומת production serving מקומית</v>
+      </c>
+      <c r="D121" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E121" t="str">
+        <v>best practices: Railway docs</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F120"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F121"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix Railway build: move runtime+build deps out of devDependencies
react, react-dom, @types/react(-dom), typescript, vite, @vitejs/plugin-react-swc moved to dependencies so a production install (NODE_ENV=production, devDeps omitted) still has everything the build/runtime needs. electron/electron-builder/vitest/concurrently stay in devDependencies (skipped on Railway -> no electron binary download). Added tsconfig.build.json (excludes *.test.ts) so the build's tsc doesn't require vitest. Verified: build + 68 tests pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F122"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2520,9 +2520,26 @@
         <v>best practices: Railway docs</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>2026-06-22 18:50</v>
+      </c>
+      <c r="B122" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Railway build נכשל — react/vite/typescript ב-devDeps דולגו ב-NODE_ENV=production</v>
+      </c>
+      <c r="D122" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E122" t="str">
+        <v>הועברו ל-dependencies + tsconfig.build מחריג בדיקות; אומת build</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F121"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F122"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix Railway build: sync package-lock + pin Node 22
npm ci failed: lock out of sync after moving deps (Missing esbuild from lock). Regenerated package-lock.json. Railway used Node 18 but vite/vitest/pdfjs-dist need Node 20+ -> added engines.node=22.x so nixpacks selects Node 22. Verified npm ci --dry-run in sync + build passes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F123"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2537,9 +2537,26 @@
         <v>הועברו ל-dependencies + tsconfig.build מחריג בדיקות; אומת build</v>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>2026-06-22 18:55</v>
+      </c>
+      <c r="B123" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Railway npm ci נכשל — lock לא מסונכרן + Node 18</v>
+      </c>
+      <c r="D123" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E123" t="str">
+        <v>רענון package-lock + engines.node=22.x</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F122"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F123"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix Railway npm ci: downgrade vitest 4->3 to resolve esbuild conflict
vitest@4 pulls vite@8 which requires esbuild ^0.28, conflicting with our vite@5 (esbuild 0.21) -> lock had an unresolvable/invalid esbuild dedup, breaking 'npm ci' on Railway (Missing esbuild@0.28.1). vitest@3.2.4 uses a compatible vite/esbuild. Clean-regenerated package-lock.json. Verified: npm ci --dry-run in sync, 68 tests pass, build OK, zero esbuild 0.28 refs in lock.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F124"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2554,9 +2554,26 @@
         <v>רענון package-lock + engines.node=22.x</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>2026-06-22 19:00</v>
+      </c>
+      <c r="B124" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Railway npm ci נכשל — vitest@4 משך vite@8/esbuild@0.28 בקונפליקט עם vite@5</v>
+      </c>
+      <c r="D124" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E124" t="str">
+        <v>הורד ל-vitest@3 + רענון lock נקי; 68 tests עוברות</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F123"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F124"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add MAP_SERVICES.md — break map domain into 9 generic reusable services
Georeferencing, polygons, markers, routes, pathfinding, status overlay, coords, geo-conflicts. Documents existing duplication (anchoring/polygons/routes/haversine across maps.js, airfield.js, driver.js) and a DRY consolidation plan to be executed via /feature.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2571,9 +2571,26 @@
         <v>הורד ל-vitest@3 + רענון lock נקי; 68 tests עוברות</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>2026-06-23 09:00</v>
+      </c>
+      <c r="B125" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C125" t="str">
+        <v>חלוקת נושא המפה ל-9 שירותים גנריים (MAP_SERVICES.md) + זיהוי כפילויות לאיחוד</v>
+      </c>
+      <c r="D125" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E125" t="str">
+        <v>עיגון/פוליגונים/דרכים/ניתוב — DRY</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F124"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F125"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add /atc-ux skill — ATC human-factors UX review (FAA/EUROCONTROL/ICAO)
Encodes 8 core HMI principles from FAA HF-STD-001, EUROCONTROL CWP/HMI, ICAO Doc 9758, and Ahlstrom & Arend color-usability research: perceptual hierarchy, color rationale, dark mode, glance time, human-in-command, error prevention, consistency, feedback/status. Use before/after designing CTRL/TWR screens.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2588,9 +2588,26 @@
         <v>עיגון/פוליגונים/דרכים/ניתוב — DRY</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>2026-06-23 09:15</v>
+      </c>
+      <c r="B126" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C126" t="str">
+        <v>סקיל /atc-ux — ביקורת UX להנדסת אנוש של עמדות ATC (FAA/EUROCONTROL/ICAO) + הצעות שינוי</v>
+      </c>
+      <c r="D126" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E126" t="str">
+        <v>מבוסס מחקר online, לא המצאה</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F125"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F126"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: comprehensive code review #2 (efficiency, security, performance)
Evidence-based audit with real DB measurements. Key findings: no API auth on public Railway URL, 64 polling intervals + missing indexes + Neon latency = slowness, single 2.7MB bundle. SQL injection: safe. Prioritized action plan included.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F129"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2605,9 +2605,60 @@
         <v>מבוסס מחקר online, לא המצאה</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>2026-06-23 09:20</v>
+      </c>
+      <c r="B127" t="str">
+        <v>בקשה</v>
+      </c>
+      <c r="C127" t="str">
+        <v>פיצ'ר התאמת 4 גדלי מסך (רזולוציה/טקסט/פונט)</v>
+      </c>
+      <c r="D127" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E127" t="str">
+        <v>feature/screen-size-scaling — zoom גלובלי + צילומים + QA</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>2026-06-23 09:25</v>
+      </c>
+      <c r="B128" t="str">
+        <v>בקשה</v>
+      </c>
+      <c r="C128" t="str">
+        <v>מעבר ביקורת מקיף #2 (יעילות/אבטחה/ביצועים)</v>
+      </c>
+      <c r="D128" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E128" t="str">
+        <v>CODE_REVIEW_2.md — מדידות אמיתיות + תוכנית</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>2026-06-23 09:30</v>
+      </c>
+      <c r="B129" t="str">
+        <v>שיפור</v>
+      </c>
+      <c r="C129" t="str">
+        <v>indexes על עמודות חמות</v>
+      </c>
+      <c r="D129" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E129" t="str">
+        <v>feature/perf-indexes — init.js, יחול ב-restart</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F126"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F129"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: handwriting recognition architecture recommendations (offline/air-gapped)
Architect research for context-aware handwriting->text on touchscreen+stylus, constrained to fully offline (closed network). Recommends stroke-based $P/$N point-cloud recognizer + context resolver with fuzzy-matching against known candidate sets (callsigns/bases), building on existing HandwritingOverlay + learned-examples. Flags that current Tesseract.js usage fetches from CDN -> broken offline. Recommendations only, not implemented.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F131"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2656,9 +2656,43 @@
         <v>feature/perf-indexes — init.js, יחול ב-restart</v>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>2026-06-23 10:00</v>
+      </c>
+      <c r="B130" t="str">
+        <v>בקשה</v>
+      </c>
+      <c r="C130" t="str">
+        <v>השלמת נ"צ ל-12 בסיסים (מתמונה DMS→decimal)</v>
+      </c>
+      <c r="D130" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E130" t="str">
+        <v>עודכן ב-DB אחרי אישור + אימות</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>2026-06-23 10:10</v>
+      </c>
+      <c r="B131" t="str">
+        <v>בקשה (מחקר)</v>
+      </c>
+      <c r="C131" t="str">
+        <v>זיהוי כתב יד מודע-הקשר offline (רשת סגורה)</v>
+      </c>
+      <c r="D131" t="str">
+        <v>המלצות נכתבו</v>
+      </c>
+      <c r="E131" t="str">
+        <v>HANDWRITING_RECOGNITION.md — $P strokes + context resolver; טרם יושם</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F129"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F131"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: log handwriting Phase 1 in requirements tracker
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F132"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2690,9 +2690,26 @@
         <v>HANDWRITING_RECOGNITION.md — $P strokes + context resolver; טרם יושם</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>2026-06-23 10:30</v>
+      </c>
+      <c r="B132" t="str">
+        <v>בקשה</v>
+      </c>
+      <c r="C132" t="str">
+        <v>פיצ'ר זיהוי כתב יד offline — ליבה גנרית (Phase 1)</v>
+      </c>
+      <c r="D132" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E132" t="str">
+        <v>$P + context resolver + HandwritingPad; 21 tests; מוזג ל-main</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F131"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F132"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: log handwriting Phase 2 (map case + calibration)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F133"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2707,9 +2707,26 @@
         <v>$P + context resolver + HandwritingPad; 21 tests; מוזג ל-main</v>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>2026-06-23 11:00</v>
+      </c>
+      <c r="B133" t="str">
+        <v>בקשה</v>
+      </c>
+      <c r="C133" t="str">
+        <v>זיהוי כתב יד — מקרה המפה (Phase 2) + כיול per-user</v>
+      </c>
+      <c r="D133" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E133" t="str">
+        <v>recognize tool + learned_strokes + calibration; מוזג ל-main</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F132"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F133"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(i18n): bilingual infra (he/en) + language switcher + fully translated LOGIN (Pilot)
תשתית דו-לשוניות (Phase 1 — Pilot):
- react-i18next (גרסאות תואמות TS 4.9) תחת src/i18n/ — עברית ברירת מחדל, התמדה ב-localStorage['bt-lang']
- useDirection: מנגנון כיווניות יחיד ב-root (<html dir>) — he=rtl, en=ltr
- בורר שפה במסך ה-LOGIN (עברית/English) → משפיע על כל המערכת
- מסך ה-LOGIN מתורגם במלואו + מתהפך ל-LTR באנגלית (direction:rtl → dir דינמי, marginRight → logical properties)
- 6 בדיקות i18n; תיעוד הדפוס ב-CLAUDE.md/DEV_GUIDE/SERVICES

שני באגים שהבדיקות תפסו (היו שוברים את כל האפליקציה):
- namespace: login/common נהיו namespaces → t('login.x') החזיר את המפתח. תוקן בעטיפת translation.
- count: i18next מפרש {{count}} כ-plural → interpolation נשבר. הוחלף ל-{{total}}.

QA: tsc נקי · vite build ✅ · 103/103 בדיקות. Runtime: init אומת ב-vitest; flip ויזואלי בדפדפן — ממתין לאימות משתמש.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F136"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2724,9 +2724,60 @@
         <v>recognize tool + learned_strokes + calibration; מוזג ל-main</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>2026-07-12 17:58</v>
+      </c>
+      <c r="B134" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C134" t="str">
+        <v>דו-לשוניות: לכל שדה/פעולה/טקסט שם עברי (קיים) + שם אנגלי</v>
+      </c>
+      <c r="D134" t="str">
+        <v/>
+      </c>
+      <c r="E134" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>2026-07-12 17:58</v>
+      </c>
+      <c r="B135" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C135" t="str">
+        <v>בורר שפה (עברית/אנגלית) במסך LOGIN, ברירת מחדל עברית</v>
+      </c>
+      <c r="D135" t="str">
+        <v/>
+      </c>
+      <c r="E135" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>2026-07-12 17:58</v>
+      </c>
+      <c r="B136" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C136" t="str">
+        <v>בחירת השפה ב-LOGIN משפיעה על כל המערכת (כולל RTL/LTR מלא)</v>
+      </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
+      <c r="E136" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F133"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F136"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mission-desk): sidebar tab icon + surface server errors on desk create/save
The + button failed silently when the running Express process predates
the merge (no /api/mission-desks route) — now alerts with a restart
hint. Added 🗂 icon to the sidebar tab label (registry value).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F191"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3781,9 +3781,349 @@
         <v/>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>2026-07-15 16:59</v>
+      </c>
+      <c r="B172" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C172" t="str">
+        <v>תפריט "יצירה" חדש בסרגל העליון (מסגרת ליצירות עתידיות)</v>
+      </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
+      <c r="E172" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>2026-07-15 16:59</v>
+      </c>
+      <c r="B173" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C173" t="str">
+        <v>נקודת העברה פרוביזורית (זמנית) בין 2 עמדות — לא במסך ניהול. טופס: שם, עמדה שנייה, הערות</v>
+      </c>
+      <c r="D173" t="str">
+        <v/>
+      </c>
+      <c r="E173" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>2026-07-15 16:59</v>
+      </c>
+      <c r="B174" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C174" t="str">
+        <v>אישור נקודה זמנית בעמדה השנייה: תפריט "יצירה" מהבהב + "אשר נקודת העברה זמנית"</v>
+      </c>
+      <c r="D174" t="str">
+        <v/>
+      </c>
+      <c r="E174" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>2026-07-15 16:59</v>
+      </c>
+      <c r="B175" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C175" t="str">
+        <v>נקודה זמנית נשמרת ב-DB זמנית; נמחקת אוטומטית אם לא שמו בה פ"ממים מעל 12 שעות ואחרי חצות</v>
+      </c>
+      <c r="D175" t="str">
+        <v/>
+      </c>
+      <c r="E175" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>2026-07-17 01:43</v>
+      </c>
+      <c r="B176" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C176" t="str">
+        <v>תוכנית אספקה: פירוק המערכת ל-17 אבני בניין עם תכולות לכל אחת (DELIVERY_PLAN.md)</v>
+      </c>
+      <c r="D176" t="str">
+        <v/>
+      </c>
+      <c r="E176" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>2026-07-17 01:43</v>
+      </c>
+      <c r="B177" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C177" t="str">
+        <v>אומדני זמן פיתוח ריאליים לכל אבן בניין — כאילו נבנה בבית תוכנה חיצוני (ימי-אדם + יומן)</v>
+      </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
+      <c r="E177" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>2026-07-17 01:43</v>
+      </c>
+      <c r="B178" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C178" t="str">
+        <v>תוכנית שחרור בגרסאות R1-R6 — מסירת המערכת למשתמש בחלקים, כל גרסה עומדת בפני עצמה</v>
+      </c>
+      <c r="D178" t="str">
+        <v/>
+      </c>
+      <c r="E178" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>2026-07-17 01:43</v>
+      </c>
+      <c r="B179" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C179" t="str">
+        <v>7 סטוריות חדשות (US-110..US-116) שקיימות בקוד וחסרות ב-USER_STORIES.md — i18n, תמות, real-time, audit, נק' העברה זמניות, Query</v>
+      </c>
+      <c r="D179" t="str">
+        <v/>
+      </c>
+      <c r="E179" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>2026-07-17 16:37</v>
+      </c>
+      <c r="B180" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C180" t="str">
+        <v>תרגום ה-NDA לאנגלית + ייצוא ל-Word (LTR)</v>
+      </c>
+      <c r="D180" t="str">
+        <v/>
+      </c>
+      <c r="E180" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>2026-07-20 13:20</v>
+      </c>
+      <c r="B181" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C181" t="str">
+        <v>הערכת CTO: מוכנות המערכת ל-production והכנסה לחיל האוויר — דירוג Go/No-Go לכל היבט + עלויות בישראל + המלצה rebuild מול המשך</v>
+      </c>
+      <c r="D181" t="str">
+        <v/>
+      </c>
+      <c r="E181" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>2026-07-21 11:00</v>
+      </c>
+      <c r="B182" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C182" t="str">
+        <v>דסק משימה כללי: הגדרת מבנה דסק במסך הניהול (כמו אפיון מסך סטריפים)</v>
+      </c>
+      <c r="D182" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E182" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>2026-07-21 11:00</v>
+      </c>
+      <c r="B183" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C183" t="str">
+        <v>דסק משימה כללי: שירות "מסך ניהול אמצעים" — כפתורים עם מצבים/צבע/טקסט/פונט/גודל/מיקום + טריגר בעמדה אחרת</v>
+      </c>
+      <c r="D183" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E183" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>2026-07-21 11:00</v>
+      </c>
+      <c r="B184" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C184" t="str">
+        <v>דסק משימה כללי: שירות טקסט חופשי בכתב יד — חלונות עם שורות הפרדה/רווח/כותרות</v>
+      </c>
+      <c r="D184" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E184" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>2026-07-21 11:00</v>
+      </c>
+      <c r="B185" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C185" t="str">
+        <v>דסק משימה כללי: מוד טבלה חכמה — עמודות (טקסט/מספר/V-X/תפריט), עיצוב מותנה, חישובים, שורת סיכום</v>
+      </c>
+      <c r="D185" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E185" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>2026-07-21 11:00</v>
+      </c>
+      <c r="B186" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C186" t="str">
+        <v>דסק משימה כללי: בניית דסק בגרירת שירותים למיקומים בחלון ושמירה</v>
+      </c>
+      <c r="D186" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E186" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>2026-07-21 11:00</v>
+      </c>
+      <c r="B187" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C187" t="str">
+        <v>דסק משימה כללי: עמדה מסוג "דסק משימה כללי" + שיתוף שירות בין עמדות עם סנכרון</v>
+      </c>
+      <c r="D187" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E187" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>2026-07-21 11:05</v>
+      </c>
+      <c r="B188" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C188" t="str">
+        <v>הפקת מסמך USER STORIES מפורט לכל המערכת + תמחור שעות עבודה של תוכניתן רגיל</v>
+      </c>
+      <c r="D188" t="str">
+        <v/>
+      </c>
+      <c r="E188" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>2026-07-21 11:18</v>
+      </c>
+      <c r="B189" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C189" t="str">
+        <v>הוצאת מסמך הסטוריות בפורמט קריא (HTML מעוצב) במקום קובץ MD</v>
+      </c>
+      <c r="D189" t="str">
+        <v/>
+      </c>
+      <c r="E189" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>2026-07-21 15:01</v>
+      </c>
+      <c r="B190" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C190" t="str">
+        <v>דסק משימה כללי: כפתור + ליצירת דסק לא עובד (אין משוב שגיאה)</v>
+      </c>
+      <c r="D190" t="str">
+        <v/>
+      </c>
+      <c r="E190" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>2026-07-21 15:01</v>
+      </c>
+      <c r="B191" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C191" t="str">
+        <v>דסק משימה כללי: חסר אייקון בתפריט הצד ליד "דסקי משימה"</v>
+      </c>
+      <c r="D191" t="str">
+        <v/>
+      </c>
+      <c r="E191" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F171"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F191"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mission-desk): V/X count counts what you choose, not every touched cell
Count on a check column used the generic non-empty rule, so a cell
toggled to X still counted (String(false) is non-empty). Now a check
column counts ✔ by default, and the column config offers 'נספר: ✔/✘'
(X counts everything displayed as ✘, incl. never-toggled rows —
consistent with the visual). TDD: 3 new unit tests (174 total).
Also logged 16 pending requirement rows now that the xlsx unlocked.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F191"/>
+  <dimension ref="A1:F207"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4098,7 +4098,7 @@
         <v>דסק משימה כללי: כפתור + ליצירת דסק לא עובד (אין משוב שגיאה)</v>
       </c>
       <c r="D190" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="E190" t="str">
         <v/>
@@ -4115,15 +4115,287 @@
         <v>דסק משימה כללי: חסר אייקון בתפריט הצד ליד "דסקי משימה"</v>
       </c>
       <c r="D191" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="E191" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B192" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C192" t="str">
+        <v>דסק משימה: אמצעים קבועים ונתוני טבלה בהגדרת עמדה — פתיחת הדסק לתצוגת הגדרה (כולל מיקום)</v>
+      </c>
+      <c r="D192" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E192" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B193" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C193" t="str">
+        <v>דסק משימה: הגדרת גודל כפתור באמצעים</v>
+      </c>
+      <c r="D193" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E193" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B194" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C194" t="str">
+        <v>דסק משימה: פעולות מגע במקום קליק ימני (מסך מגע)</v>
+      </c>
+      <c r="D194" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E194" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B195" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C195" t="str">
+        <v>דסק משימה: פלנלית — ניקוי מלא או מחיקה לפי מיקום הסמן</v>
+      </c>
+      <c r="D195" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E195" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B196" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C196" t="str">
+        <v>דסק משימה: כניסה לעמדת דסק שנוצרה כשהדף פתוח העלתה מוד טבלאי (רענון presets)</v>
+      </c>
+      <c r="D196" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E196" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B197" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C197" t="str">
+        <v>דסק משימה: לא להציג שרבוטי עט בתצוגת ההגדרה</v>
+      </c>
+      <c r="D197" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E197" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B198" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C198" t="str">
+        <v>דסק משימה: שינוי גודל כפתור בגרירה (ידית ◢)</v>
+      </c>
+      <c r="D198" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E198" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B199" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C199" t="str">
+        <v>דסק משימה: "מחק הכל" + אייקון מחק שמוחק במעבר הסמן</v>
+      </c>
+      <c r="D199" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E199" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B200" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C200" t="str">
+        <v>דסק משימה: בונה נוסחאות ויזואלי בטבלה (שדה→אופרטור→שדה)</v>
+      </c>
+      <c r="D200" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E200" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B201" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C201" t="str">
+        <v>דסק משימה: סרגל עליון סטנדרטי — שם עמדה/בקר+החלף/הודעה לעמדה/שעון</v>
+      </c>
+      <c r="D201" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E201" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B202" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C202" t="str">
+        <v>מסך ניהול: השורה האחרונה בכל קטגוריה בתפריט הצד נחתכה (flex shrink)</v>
+      </c>
+      <c r="D202" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E202" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B203" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C203" t="str">
+        <v>מסך ניהול: איחוד עיצוב כותרות הקטגוריות בתפריט הצד</v>
+      </c>
+      <c r="D203" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E203" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B204" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C204" t="str">
+        <v>דסק משימה: ערכי תפריט בטבלה — הפסיק נבלע; הוחלף בתת-טבלת ערכים</v>
+      </c>
+      <c r="D204" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E204" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B205" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C205" t="str">
+        <v>דסק משימה: ספליטרים מותאמי מגע/עט בין חלונות הדסק, שמירה פר-עמדה</v>
+      </c>
+      <c r="D205" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E205" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B206" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C206" t="str">
+        <v>דסק משימה: כמות בעמודת V/X ספרה כל תא שסומן אי-פעם</v>
+      </c>
+      <c r="D206" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E206" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>2026-07-22 10:31</v>
+      </c>
+      <c r="B207" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C207" t="str">
+        <v>דסק משימה: הגדרה בעמודת V/X מה נספר — ✔ או ✘</v>
+      </c>
+      <c r="D207" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E207" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F191"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F207"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(admin)+feat(mission-desk): duplicate-position save enabled; sharing is bidirectional and desk-only
- Duplicate position: save button stayed disabled because
  presetFormInitial was set to null while presetIsDirty requires
  a non-null baseline — now uses an always-dirty sentinel. e2e covers
  duplicate->save->new row appears.
- Sharing list in the position editor shows only mission_desk
  positions.
- mission_desk_sharing is mirrored on save (same pattern as
  mirrorClassicPartnerLinks): sharing A->B writes the reverse link on
  B, removal removes it — so both stations fan out to each other and
  one-sided config can no longer clobber the other side. Smoke-tested
  against Neon: mirror, reverse fan-out, mirrored removal.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F207"/>
+  <dimension ref="A1:F211"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4393,9 +4393,77 @@
         <v/>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>2026-07-22 11:07</v>
+      </c>
+      <c r="B208" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C208" t="str">
+        <v>דסק משימה: כפתורי אמצעים מסתדרים אוטומטית בלי לעלות אחד על השני</v>
+      </c>
+      <c r="D208" t="str">
+        <v/>
+      </c>
+      <c r="E208" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>2026-07-22 11:17</v>
+      </c>
+      <c r="B209" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C209" t="str">
+        <v>מסך ניהול: שכפול עמדה — כפתור השמירה נשאר כבוי (presetFormInitial=null)</v>
+      </c>
+      <c r="D209" t="str">
+        <v/>
+      </c>
+      <c r="E209" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>2026-07-22 11:17</v>
+      </c>
+      <c r="B210" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C210" t="str">
+        <v>דסק משימה: רשימת השיתוף מציגה רק עמדות מסוג דסק משימה</v>
+      </c>
+      <c r="D210" t="str">
+        <v/>
+      </c>
+      <c r="E210" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>2026-07-22 11:17</v>
+      </c>
+      <c r="B211" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C211" t="str">
+        <v>דסק משימה: שיתוף דו-כיווני — הגדרה בעמדה אחת משתקפת אוטומטית בשנייה</v>
+      </c>
+      <c r="D211" t="str">
+        <v/>
+      </c>
+      <c r="E211" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F211"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(mission-desk): sharing limited to positions using the same desk
The share checkbox list now offers only mission_desk positions whose
mission_desk_id matches the desk selected in the editor — sharing with
a position on a different desk was meaningless. Empty-state hint when
no other position uses this desk. Alert-target lists still show all
positions (burst alerts work cross-type).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F211"/>
+  <dimension ref="A1:F217"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,10 +442,10 @@
         <v>עדכון מז"א ממגדל תל נוף אווירי הלך לבחא 10 במקום לבחא 8 (בסיס האב)</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>d968d13, 7aad51d</v>
       </c>
     </row>
     <row r="3">
@@ -454,10 +462,10 @@
         <v>הוספת שדה mazaa_update_base_id לפריסט מגדל — בחירת בסיס יעד מדויק לעדכוני מז"א</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>7aad51d</v>
       </c>
     </row>
     <row r="4">
@@ -474,10 +482,10 @@
         <v>הגדלת הפסקל האפור בין פ"מ לפ"מ בתצוגת טבלה ראשית (3px במקום 1px)</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>dd23bf7</v>
       </c>
     </row>
     <row r="5">
@@ -494,10 +502,10 @@
         <v>יצירת SKILL אוטומטי לרישום דרישות ב-Excel בקטגוריות תקלה / תכולה חדשה / שיפור</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>875dba3</v>
       </c>
     </row>
     <row r="6">
@@ -514,10 +522,10 @@
         <v>נעלמה האפשרות לצפות בגאנט עומסים מהעמדה</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>0d1553b</v>
       </c>
     </row>
     <row r="7">
@@ -534,10 +542,10 @@
         <v>עדכון מז"א בעמדת מגדל מעדכן את כל הבסיסים ברשימה במקום רק את בסיס האב של העמדה</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>d968d13</v>
       </c>
     </row>
     <row r="8">
@@ -554,10 +562,10 @@
         <v>הזזת רשימת מסלולים בשדה תעופה מהסרגל העליון לחלק הימני התחתון של המפה + הסרת עיגול אדום ליד מסלולים סגורים</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>d499ae5</v>
       </c>
     </row>
     <row r="9">
@@ -574,10 +582,10 @@
         <v>במצב מפה עיוורת — הקטנת שמות האזורים כך שייראו אך לא יחסמו את האזור</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>b842d2c</v>
       </c>
     </row>
     <row r="10">
@@ -594,10 +602,10 @@
         <v>עדכון קובץ האקסל (project-requirements.xlsx) אחרי כל בקשה בשיחה</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>cf733a5; מ-2026-07-22 נאכף ב-hook UserPromptSubmit</v>
       </c>
     </row>
     <row r="11">
@@ -614,10 +622,10 @@
         <v>היכן רואים את קובץ האקסל project-requirements.xlsx</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>שאלה — נענתה בשיחה</v>
       </c>
     </row>
     <row r="12">
@@ -625,16 +633,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-06-15 13:08</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C12" t="str">
-        <v>שיפור</v>
+        <v>גרירת סטריפ למפה במסך מגע/עט במצב אזורי טיסה — תיקון תקיעה בצד שמאל</v>
       </c>
       <c r="D12" t="str">
-        <v>הוספת שעה לעמודת תאריך בקובץ האקסל</v>
+        <v>bug</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -645,16 +653,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-06-15 13:09</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C13" t="str">
-        <v>שאלה</v>
+        <v>ציור עם עט/אצבע בחלון OCR סטריפים לא עובד — תיקון Pointer Events</v>
       </c>
       <c r="D13" t="str">
-        <v>בירור לגבי יכולת זיהוי קולי והמרה לטקסט בעברית</v>
+        <v>bug</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -665,16 +673,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-06-15 13:13</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C14" t="str">
-        <v>תכולה חדשה</v>
+        <v>ביטול תיקון Pointer Events בחלוני ציור OCR — חזרה לגרסה קודמת</v>
       </c>
       <c r="D14" t="str">
-        <v>שילוב Web Speech API — זיהוי קולי בעברית: שמיעת גובה חדש ועדכון עמודת גובה בסטריפ הנבחר בעמדה</v>
+        <v>bug</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -685,16 +693,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-06-15 13:40</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C15" t="str">
-        <v>שיפור קיים</v>
+        <v>חילוץ User Stories מכל קומפוננטה — 278 stories, 49 נושאים — מסמך USER_STORIES.md</v>
       </c>
       <c r="D15" t="str">
-        <v>זיהוי קולי — הרחבה: 1) טווחי גבהים (300-400) 2) פקודת העברה לנקודת העברה (חנית 400 לצארלי)</v>
+        <v>documentation</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -705,16 +713,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-06-15 13:50</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C16" t="str">
-        <v>שיפור לתכולה קיימת</v>
+        <v>העלאת USER_STORIES.md לגיטהאב (levori119/skyboard)</v>
       </c>
       <c r="D16" t="str">
-        <v>זיהוי קולי — תמיכה בפמ פוצל: זיהוי index מבנה (פיל 3) + מניעת בלבול עם גובה</v>
+        <v>ci</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -725,16 +733,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-06-15 13:57</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C17" t="str">
-        <v>תקלה</v>
+        <v>ייצוא DB ל-ZIP (skyking_db_export.zip)</v>
       </c>
       <c r="D17" t="str">
-        <v>זיהוי קולי — תיקון regex ל-ל prefix: \b לא עובד בעברית, הוחלף ב-(?:^|\s)</v>
+        <v>export</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -745,16 +753,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-06-15 13:57</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C18" t="str">
-        <v>שיפור לתכולה קיימת</v>
+        <v>ייצוא User Stories באנגלית — USER_STORIES_EN.md</v>
       </c>
       <c r="D18" t="str">
-        <v>זיהוי קולי — העברה בלי גובה נתמכת; חיפוש סקטור גם ב-classic_transfer_points לפי label</v>
+        <v>documentation</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>done</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -765,19 +773,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-06-15 14:04</v>
+        <v>2026-06-15 13:08</v>
       </c>
       <c r="C19" t="str">
-        <v>תכולה חדשה</v>
+        <v>שיפור</v>
       </c>
       <c r="D19" t="str">
-        <v>זיהוי קולי — שיוך פמ לאזור במה בדיבור: "חנית לאזור צפון"</v>
+        <v>הוספת שעה לעמודת תאריך בקובץ האקסל</v>
       </c>
       <c r="E19" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>60b6b65, 9b45157</v>
       </c>
     </row>
     <row r="20">
@@ -785,19 +793,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-06-15 14:04</v>
+        <v>2026-06-15 13:09</v>
       </c>
       <c r="C20" t="str">
-        <v>תכולה חדשה</v>
+        <v>שאלה</v>
       </c>
       <c r="D20" t="str">
-        <v>זיהוי קולי — קבלת העברה נכנסת + שיוך לאזור בדיבור: "[callsign] לאזור [שם]"</v>
+        <v>בירור לגבי יכולת זיהוי קולי והמרה לטקסט בעברית</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>שאלה — נענתה; הובילה לפיצ'ר הזיהוי הקולי</v>
       </c>
     </row>
     <row r="21">
@@ -805,19 +813,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 13:13</v>
       </c>
       <c r="C21" t="str">
-        <v>גרירת סטריפ למפה במסך מגע/עט במצב אזורי טיסה — תיקון תקיעה בצד שמאל</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D21" t="str">
-        <v>bug</v>
+        <v>שילוב Web Speech API — זיהוי קולי בעברית: שמיעת גובה חדש ועדכון עמודת גובה בסטריפ הנבחר בעמדה</v>
       </c>
       <c r="E21" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>62aaae4</v>
       </c>
     </row>
     <row r="22">
@@ -825,19 +833,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 13:40</v>
       </c>
       <c r="C22" t="str">
-        <v>ציור עם עט/אצבע בחלון OCR סטריפים לא עובד — תיקון Pointer Events</v>
+        <v>שיפור קיים</v>
       </c>
       <c r="D22" t="str">
-        <v>bug</v>
+        <v>זיהוי קולי — הרחבה: 1) טווחי גבהים (300-400) 2) פקודת העברה לנקודת העברה (חנית 400 לצארלי)</v>
       </c>
       <c r="E22" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>4bf5a70</v>
       </c>
     </row>
     <row r="23">
@@ -845,19 +853,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 13:50</v>
       </c>
       <c r="C23" t="str">
-        <v>ביטול תיקון Pointer Events בחלוני ציור OCR — חזרה לגרסה קודמת</v>
+        <v>שיפור לתכולה קיימת</v>
       </c>
       <c r="D23" t="str">
-        <v>bug</v>
+        <v>זיהוי קולי — תמיכה בפמ פוצל: זיהוי index מבנה (פיל 3) + מניעת בלבול עם גובה</v>
       </c>
       <c r="E23" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>ae3aefe</v>
       </c>
     </row>
     <row r="24">
@@ -865,19 +873,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 13:57</v>
       </c>
       <c r="C24" t="str">
-        <v>חילוץ User Stories מכל קומפוננטה — 278 stories, 49 נושאים — מסמך USER_STORIES.md</v>
+        <v>תקלה</v>
       </c>
       <c r="D24" t="str">
-        <v>documentation</v>
+        <v>זיהוי קולי — תיקון regex ל-ל prefix: \b לא עובד בעברית, הוחלף ב-(?:^|\s)</v>
       </c>
       <c r="E24" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F24" t="str">
-        <v/>
+        <v>8bfeaa3</v>
       </c>
     </row>
     <row r="25">
@@ -885,19 +893,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 13:57</v>
       </c>
       <c r="C25" t="str">
-        <v>העלאת USER_STORIES.md לגיטהאב (levori119/skyboard)</v>
+        <v>שיפור לתכולה קיימת</v>
       </c>
       <c r="D25" t="str">
-        <v>ci</v>
+        <v>זיהוי קולי — העברה בלי גובה נתמכת; חיפוש סקטור גם ב-classic_transfer_points לפי label</v>
       </c>
       <c r="E25" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>8bfeaa3</v>
       </c>
     </row>
     <row r="26">
@@ -905,19 +913,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 14:04</v>
       </c>
       <c r="C26" t="str">
-        <v>ייצוא DB ל-ZIP (skyking_db_export.zip)</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D26" t="str">
-        <v>export</v>
+        <v>זיהוי קולי — שיוך פמ לאזור במה בדיבור: "חנית לאזור צפון"</v>
       </c>
       <c r="E26" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>c979c32</v>
       </c>
     </row>
     <row r="27">
@@ -925,19 +933,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-15 14:04</v>
       </c>
       <c r="C27" t="str">
-        <v>ייצוא User Stories באנגלית — USER_STORIES_EN.md</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D27" t="str">
-        <v>documentation</v>
+        <v>זיהוי קולי — קבלת העברה נכנסת + שיוך לאזור בדיבור: "[callsign] לאזור [שם]"</v>
       </c>
       <c r="E27" t="str">
-        <v>done</v>
+        <v>כן</v>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>c979c32</v>
       </c>
     </row>
     <row r="28">
@@ -954,10 +962,10 @@
         <v>הוספת נקודות מנהלתיות ואלמנטי שדה לאפליקציית הנהג (driver.html) לאחר בחירת בסיס</v>
       </c>
       <c r="E28" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>77510e9</v>
       </c>
     </row>
     <row r="29">
@@ -974,10 +982,10 @@
         <v>בניהול מערכת — קטגוריות בתפריט ימני עולות אחד על השני, תוקן ריווח בין הסקשנים</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>d9c747d</v>
       </c>
     </row>
     <row r="30">
@@ -994,10 +1002,10 @@
         <v>ייצוא דרישות לאקסל לא בוצע — תוקן מעכשיו</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>05a1804</v>
       </c>
     </row>
     <row r="31">
@@ -1014,10 +1022,10 @@
         <v>תפריט ניהול מערכת — טקסט קטגוריות עדיין צפוף מדי לאחר תיקון ראשון, הוגדל ריווח נוסף</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>7a4c6cc</v>
       </c>
     </row>
     <row r="32">
@@ -1034,10 +1042,10 @@
         <v>ביטול יד (גרירת מפה) בעמדה עם מפה — אין צורך בגרירת המפה עצמה</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>a564d11</v>
       </c>
     </row>
     <row r="33">
@@ -1054,10 +1062,10 @@
         <v>כפתור 🚗 אינליין על כל אלמנט בשדה — טוגל מהיר להצגה/הסרה מתפריט נהג מזדמן</v>
       </c>
       <c r="E33" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>15ef572</v>
       </c>
     </row>
     <row r="34">
@@ -1074,10 +1082,10 @@
         <v>כפתור 🚗 אינליין על כל נקודה מנהלתית — טוגל מהיר להצגה/הסרה מתפריט נהג מזדמן</v>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>15ef572</v>
       </c>
     </row>
     <row r="35">
@@ -1094,10 +1102,10 @@
         <v>כפתור 🚗 אינליין על כל נקודה בשדה תעופה (נקודות רגילות) — טוגל מהיר להצגה בתפריט נהג מזדמן</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F35" t="str">
-        <v/>
+        <v>df1bc6f</v>
       </c>
     </row>
     <row r="36">
@@ -1114,10 +1122,10 @@
         <v>נקודות בסיס לא מופיעות בתפריט מוצא/הגעה באפליקציית נהג מזדמן — API החזיר רק admin_loc</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>0f0d4d2</v>
       </c>
     </row>
     <row r="37">
@@ -1134,10 +1142,10 @@
         <v>בחירת "מסלולי רכב" בניהול מבצעי גרמה למסך כחול — useState/useEffect בתוך IIFE מותנה</v>
       </c>
       <c r="E37" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>92690fe</v>
       </c>
     </row>
     <row r="38">
@@ -1154,10 +1162,10 @@
         <v>מסלולי רכב הועברו לתוך ניהול שדה תעופה — נתיבי נסיעה עם דקירה במפה, לא לשונית נפרדת</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>ad94482</v>
       </c>
     </row>
     <row r="39">
@@ -1174,10 +1182,10 @@
         <v>נקודות נתיבי נסיעה מכילות נ"צ GPS (lat/lon) כאשר המפה מכויילת — תמיכה ב-Google Maps</v>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>b94d179</v>
       </c>
     </row>
     <row r="40">
@@ -1194,10 +1202,10 @@
         <v>עדכון/ביטול בקשת נסיעה אחרי אישור — כפתורי "עדכן פרטים" ו-"בטל נסיעה" במסך המאושר</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>3dfb696</v>
       </c>
     </row>
     <row r="41">
@@ -1214,10 +1222,10 @@
         <v>אינדיקטור ⚓ ליד כל נתיב נסיעה — ירוק=כל הנקודות מעוגנות לנ"צ, צהוב=חלקי, אפור=ללא עיגון</v>
       </c>
       <c r="E41" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>cf6d60f</v>
       </c>
     </row>
     <row r="42">
@@ -1234,10 +1242,10 @@
         <v>אפליקציית נהג — הצגת נ"צ נוכחי בפורמט מעלות דקות שניות ליד אינדיקטור ה-GPS</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>0c6c6e8</v>
       </c>
     </row>
     <row r="43">
@@ -1254,10 +1262,10 @@
         <v>כפתור "🔁 עגן נ"צ" לנתיבי נסיעה ונקודות שנוצרו לפני כיול — מחשב GPS רטרואקטיבית ע"פ נקודות עיגון המפה</v>
       </c>
       <c r="E43" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>526a758</v>
       </c>
     </row>
     <row r="44">
@@ -1274,10 +1282,10 @@
         <v>בקשת רכבים מאושרת — הוספת ביטול/עדכון מסלול + שליחת הודעה מתפרצת לנהג מעמדת ניהול שדה תעופה (פולינג 5ש׳ ב-driver.html, פופאפ צהוב עם כפתור הבנתי)</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>3ea2d76</v>
       </c>
     </row>
     <row r="45">
@@ -1294,10 +1302,10 @@
         <v>תיקון: נ"צ שנבחרו לנתיב לא עברו לאפלקציית הנהג — openNavigation ב-driver.html בדק w.lng אך imagePctToGeo מחזיר lon (ללא g); תוקן לתמוך בשני הפורמטים</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>d68c23c</v>
       </c>
     </row>
     <row r="46">
@@ -1314,10 +1322,10 @@
         <v>עדכון מסלול נסיעה מעמדת שדה → עדכון מיידי + פופאפ התראה לנהג; ביטול ע"י עמדה → התראה + חזרה לטופס; פולינג נמשך גם לאחר אישור</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>f0af466</v>
       </c>
     </row>
     <row r="47">
@@ -1334,10 +1342,10 @@
         <v>תיקון נ"צ בנתיבי נסיעה: server מחשב GPS לנקודות חסרות ע"פ anchor מפה; driver.html מציג נ"צ DMS ליד כל נקודת מסלול</v>
       </c>
       <c r="E47" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F47" t="str">
-        <v/>
+        <v>cf52f83</v>
       </c>
     </row>
     <row r="48">
@@ -1465,19 +1473,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B54" t="str">
-        <v>2026-06-19 11:15</v>
+        <v>2026-06-19</v>
       </c>
       <c r="C54" t="str">
-        <v>פיצ׳ר</v>
+        <v>Vehicle Approval Panel</v>
       </c>
       <c r="D54" t="str">
-        <v>מוד נהג (driver.html) — טעינה אוטומטית של מפת שדה התעופה של העמדה שאישרה את כניסת הרכב</v>
+        <v>Multi-select route permissions (vehicle/taxiways/runways combinable), segmentPath with L/R turn directions in route results, excludedRouteTypes shown in UI, driver GPS + destination shown in pending approval panel, GPS polling extended to pending requests</v>
       </c>
       <c r="E54" t="str">
-        <v>driver.html + server.js GET /api/vehicle-requests</v>
+        <v>כן</v>
       </c>
       <c r="F54" t="str">
-        <v>בוצע</v>
+        <v>#55</v>
       </c>
     </row>
     <row r="55">
@@ -1485,59 +1493,59 @@
         <v>1.0.0</v>
       </c>
       <c r="B55" t="str">
-        <v>2026-06-19 11:41</v>
+        <v>2026-06-19</v>
       </c>
       <c r="C55" t="str">
-        <v>פיצ׳ר</v>
+        <v>Vehicle Approval Panel</v>
       </c>
       <c r="D55" t="str">
-        <v>כשנהג מסמן הגעה ליעד — באנר התראה בולט מופיע בפאנל כניסת רכבים בעמדת ניהול שדה התעופה</v>
+        <v>Bug: route calc fails left panel; Auto-fill from/to from driver selection; Auto-select airfield from base; Show routes from all base maps. Fix: store from_point_id+to_point_id+base_id in vehicle_requests, driver.html sends IDs, GET returns point airfield_id via JOIN, auto-populate effect in App.tsx, auto-trigger buildPlan</v>
       </c>
       <c r="E55" t="str">
-        <v>GroundVehiclePanel — newlyArrived state + detection + UI banner</v>
+        <v>כן</v>
       </c>
       <c r="F55" t="str">
-        <v>בוצע</v>
+        <v>#56</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B56">
-        <v>55</v>
+      <c r="B56" t="str">
+        <v>2026-06-19</v>
       </c>
       <c r="C56" t="str">
-        <v>2026-06-19</v>
+        <v>Feature</v>
       </c>
       <c r="D56" t="str">
-        <v>Vehicle Approval Panel</v>
+        <v>Strip window (חלון סטריפים) — per-leaf waypoint mode: מקבל (📥 incoming from sector) or מוסר (📤 outgoing to sector). Filtering logic: מוסר shows outgoingTransfers matching the waypoint sector, מקבל shows incomingTransfers from that sector. Query applied on top. Mode indicator shown in header of both admin preview and workstation view.</v>
       </c>
       <c r="E56" t="str">
-        <v>Multi-select route permissions (vehicle/taxiways/runways combinable), segmentPath with L/R turn directions in route results, excludedRouteTypes shown in UI, driver GPS + destination shown in pending approval panel, GPS polling extended to pending requests</v>
+        <v>כן</v>
       </c>
       <c r="F56" t="str">
-        <v>Done</v>
+        <v>#67</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B57">
-        <v>56</v>
+      <c r="B57" t="str">
+        <v>2026-06-19</v>
       </c>
       <c r="C57" t="str">
-        <v>2026-06-19</v>
+        <v>Improvement</v>
       </c>
       <c r="D57" t="str">
-        <v>Vehicle Approval Panel</v>
+        <v>Strip window leaf header: always show waypoint sector name + מקבל/מוסר badge alongside the label. Previously the label hid the waypoint name.</v>
       </c>
       <c r="E57" t="str">
-        <v>Bug: route calc fails left panel; Auto-fill from/to from driver selection; Auto-select airfield from base; Show routes from all base maps. Fix: store from_point_id+to_point_id+base_id in vehicle_requests, driver.html sends IDs, GET returns point airfield_id via JOIN, auto-populate effect in App.tsx, auto-trigger buildPlan</v>
+        <v>כן</v>
       </c>
       <c r="F57" t="str">
-        <v>Done</v>
+        <v>#68</v>
       </c>
     </row>
     <row r="58">
@@ -1545,19 +1553,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B58" t="str">
-        <v>2026-06-19 12:51</v>
+        <v>2026-06-19</v>
       </c>
       <c r="C58" t="str">
-        <v>תקלה</v>
+        <v>Feature</v>
       </c>
       <c r="D58" t="str">
-        <v>Auto-populate שדה/מוצא/יעד לא עבד — נראה אותו דבר (בקשות ישנות ללא IDs)</v>
+        <v>Strip window leaf: add configurable content title (📝 כותרת תוכן) displayed above the strips list. Controls: text, text color, background color, font size (10-36px), bold toggle, alignment (right/center/left). Stored in SWLeaf.content_title* fields.</v>
       </c>
       <c r="E58" t="str">
         <v>כן</v>
       </c>
       <c r="F58" t="str">
-        <v/>
+        <v>#69</v>
       </c>
     </row>
     <row r="59">
@@ -1565,19 +1573,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B59" t="str">
-        <v>2026-06-19 12:51</v>
+        <v>2026-06-19</v>
       </c>
       <c r="C59" t="str">
-        <v>תקלה</v>
+        <v>Feature</v>
       </c>
       <c r="D59" t="str">
-        <v>חישוב מסלול נכשל כי "מסלולי מטוסים" נכנס ל-permissions בטעות</v>
+        <v>Strip window admin: add 📋 duplicate button per layout. Creates copy named "[original] — עותק", auto-selects it. Handles name collision with alert.</v>
       </c>
       <c r="E59" t="str">
         <v>כן</v>
       </c>
       <c r="F59" t="str">
-        <v/>
+        <v>#70</v>
       </c>
     </row>
     <row r="60">
@@ -1585,19 +1593,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B60" t="str">
-        <v>2026-06-19 12:51</v>
+        <v>2026-06-19</v>
       </c>
       <c r="C60" t="str">
-        <v>תקלה</v>
+        <v>Improvement</v>
       </c>
       <c r="D60" t="str">
-        <v>חישוב מסלול נכשל — START_RADIUS=300m קטן מדי לנקודות רחוקות (תחילת 15 = 1218m)</v>
+        <v>Strip window: waypoint mode (מקבל/מוסר) now shown as a prominent colored banner bar between the cell header and strips list — green for מקבל, orange for מוסר. Removed small badge from header bar.</v>
       </c>
       <c r="E60" t="str">
         <v>כן</v>
       </c>
       <c r="F60" t="str">
-        <v/>
+        <v>#71</v>
       </c>
     </row>
     <row r="61">
@@ -1605,19 +1613,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B61" t="str">
-        <v>2026-06-19 12:51</v>
+        <v>2026-06-19</v>
       </c>
       <c r="C61" t="str">
-        <v>שיפור לתכולה קיימת</v>
+        <v>Bug</v>
       </c>
       <c r="D61" t="str">
-        <v>חישוב מסלול אוטומטי ישתמש בכל סוגי הנתיבים של השדה (רכב+הסעה+מסלולים)</v>
+        <v>Strip window workstation crash: swSectors (admin-only var) used in workstation rendering — replaced with allSectors (main component state). Caused ReferenceError on any strip window workstation load.</v>
       </c>
       <c r="E61" t="str">
         <v>כן</v>
       </c>
       <c r="F61" t="str">
-        <v/>
+        <v>#72</v>
       </c>
     </row>
     <row r="62">
@@ -1625,19 +1633,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B62" t="str">
-        <v>2026-06-19 13:10</v>
+        <v>2026-06-19 11:15</v>
       </c>
       <c r="C62" t="str">
-        <v>תכולה חדשה</v>
+        <v>פיצ׳ר</v>
       </c>
       <c r="D62" t="str">
-        <v>הוספת ממשק ניווט מלא לפאנל אישור בקשות רכבים — נתיבים פנויים/לא שמישים/חסומים עם "החל", לחצני קטגוריה, רצף נבחר</v>
+        <v>מוד נהג (driver.html) — טעינה אוטומטית של מפת שדה התעופה של העמדה שאישרה את כניסת הרכב</v>
       </c>
       <c r="E62" t="str">
-        <v/>
+        <v>driver.html + server.js GET /api/vehicle-requests</v>
       </c>
       <c r="F62" t="str">
-        <v/>
+        <v>בוצע</v>
       </c>
     </row>
     <row r="63">
@@ -1645,19 +1653,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B63" t="str">
-        <v>2026-06-19 13:10</v>
+        <v>2026-06-19 11:41</v>
       </c>
       <c r="C63" t="str">
-        <v>תכולה חדשה</v>
+        <v>פיצ׳ר</v>
       </c>
       <c r="D63" t="str">
-        <v>הוספת שדה via_route_ids ו-show_on_map לטבלת vehicle_requests (DB + API PUT)</v>
+        <v>כשנהג מסמן הגעה ליעד — באנר התראה בולט מופיע בפאנל כניסת רכבים בעמדת ניהול שדה התעופה</v>
       </c>
       <c r="E63" t="str">
-        <v/>
+        <v>GroundVehiclePanel — newlyArrived state + detection + UI banner</v>
       </c>
       <c r="F63" t="str">
-        <v/>
+        <v>בוצע</v>
       </c>
     </row>
     <row r="64">
@@ -1665,16 +1673,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B64" t="str">
-        <v>2026-06-19 13:10</v>
+        <v>2026-06-19 12:51</v>
       </c>
       <c r="C64" t="str">
-        <v>תכולה חדשה</v>
+        <v>תקלה</v>
       </c>
       <c r="D64" t="str">
-        <v>הוספת טוגל "הצג על מפה" (show_on_map) בפאנל בניית מסלול לבקשות רכבים</v>
+        <v>Auto-populate שדה/מוצא/יעד לא עבד — נראה אותו דבר (בקשות ישנות ללא IDs)</v>
       </c>
       <c r="E64" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F64" t="str">
         <v/>
@@ -1685,16 +1693,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B65" t="str">
-        <v>2026-06-19 13:41</v>
+        <v>2026-06-19 12:51</v>
       </c>
       <c r="C65" t="str">
-        <v>שיפור לתכולה קיימת</v>
+        <v>תקלה</v>
       </c>
       <c r="D65" t="str">
-        <v>שינוי כיתוב כפתור ופאנל "פתקית" ל-"פתקית פנימית" בעמדה</v>
+        <v>חישוב מסלול נכשל כי "מסלולי מטוסים" נכנס ל-permissions בטעות</v>
       </c>
       <c r="E65" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F65" t="str">
         <v/>
@@ -1705,19 +1713,19 @@
         <v>1.0.0</v>
       </c>
       <c r="B66" t="str">
-        <v>2026-06-19 13:52</v>
+        <v>2026-06-19 12:51</v>
       </c>
       <c r="C66" t="str">
         <v>תקלה</v>
       </c>
       <c r="D66" t="str">
-        <v>Build לפרסום נכשל — שגיאות TypeScript: draggable ב-SVG, show_in_driver חסר, route_type חסר, קוד מת עם פונקציות לא מוגדרות</v>
+        <v>חישוב מסלול נכשל — START_RADIUS=300m קטן מדי לנקודות רחוקות (תחילת 15 = 1218m)</v>
       </c>
       <c r="E66" t="str">
-        <v>✓</v>
+        <v>כן</v>
       </c>
       <c r="F66" t="str">
-        <v>תוקן — 6 שגיאות TypeScript</v>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -1725,16 +1733,16 @@
         <v>1.0.0</v>
       </c>
       <c r="B67" t="str">
-        <v>2026-06-19 14:41</v>
+        <v>2026-06-19 12:51</v>
       </c>
       <c r="C67" t="str">
-        <v>תכולה חדשה</v>
+        <v>שיפור לתכולה קיימת</v>
       </c>
       <c r="D67" t="str">
-        <v>הגדרת חלון סטריפים — אפשרות בחירת מרקם רקע (9 מרקמים: נקודות, גריד, אלכסוני, קווים, רשת, לוח שחמט)</v>
+        <v>חישוב מסלול אוטומטי ישתמש בכל סוגי הנתיבים של השדה (רכב+הסעה+מסלולים)</v>
       </c>
       <c r="E67" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F67" t="str">
         <v/>
@@ -1744,520 +1752,520 @@
       <c r="A68" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B68">
-        <v>67</v>
+      <c r="B68" t="str">
+        <v>2026-06-19 13:10</v>
       </c>
       <c r="C68" t="str">
-        <v>2026-06-19</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D68" t="str">
-        <v>Feature</v>
+        <v>הוספת ממשק ניווט מלא לפאנל אישור בקשות רכבים — נתיבים פנויים/לא שמישים/חסומים עם "החל", לחצני קטגוריה, רצף נבחר</v>
       </c>
       <c r="E68" t="str">
-        <v>Strip window (חלון סטריפים) — per-leaf waypoint mode: מקבל (📥 incoming from sector) or מוסר (📤 outgoing to sector). Filtering logic: מוסר shows outgoingTransfers matching the waypoint sector, מקבל shows incomingTransfers from that sector. Query applied on top. Mode indicator shown in header of both admin preview and workstation view.</v>
+        <v>כן</v>
       </c>
       <c r="F68" t="str">
-        <v>Done</v>
+        <v>55b3931</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B69">
-        <v>68</v>
+      <c r="B69" t="str">
+        <v>2026-06-19 13:10</v>
       </c>
       <c r="C69" t="str">
-        <v>2026-06-19</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D69" t="str">
-        <v>Improvement</v>
+        <v>הוספת שדה via_route_ids ו-show_on_map לטבלת vehicle_requests (DB + API PUT)</v>
       </c>
       <c r="E69" t="str">
-        <v>Strip window leaf header: always show waypoint sector name + מקבל/מוסר badge alongside the label. Previously the label hid the waypoint name.</v>
+        <v>כן</v>
       </c>
       <c r="F69" t="str">
-        <v>Done</v>
+        <v>55b3931</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B70">
-        <v>69</v>
+      <c r="B70" t="str">
+        <v>2026-06-19 13:10</v>
       </c>
       <c r="C70" t="str">
-        <v>2026-06-19</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D70" t="str">
-        <v>Feature</v>
+        <v>הוספת טוגל "הצג על מפה" (show_on_map) בפאנל בניית מסלול לבקשות רכבים</v>
       </c>
       <c r="E70" t="str">
-        <v>Strip window leaf: add configurable content title (📝 כותרת תוכן) displayed above the strips list. Controls: text, text color, background color, font size (10-36px), bold toggle, alignment (right/center/left). Stored in SWLeaf.content_title* fields.</v>
+        <v>כן</v>
       </c>
       <c r="F70" t="str">
-        <v>Done</v>
+        <v>55b3931</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B71">
-        <v>70</v>
+      <c r="B71" t="str">
+        <v>2026-06-19 13:41</v>
       </c>
       <c r="C71" t="str">
-        <v>2026-06-19</v>
+        <v>שיפור לתכולה קיימת</v>
       </c>
       <c r="D71" t="str">
-        <v>Feature</v>
+        <v>שינוי כיתוב כפתור ופאנל "פתקית" ל-"פתקית פנימית" בעמדה</v>
       </c>
       <c r="E71" t="str">
-        <v>Strip window admin: add 📋 duplicate button per layout. Creates copy named "[original] — עותק", auto-selects it. Handles name collision with alert.</v>
+        <v>כן</v>
       </c>
       <c r="F71" t="str">
-        <v>Done</v>
+        <v>cf9fb13</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B72">
-        <v>71</v>
+      <c r="B72" t="str">
+        <v>2026-06-19 13:52</v>
       </c>
       <c r="C72" t="str">
-        <v>2026-06-19</v>
+        <v>תקלה</v>
       </c>
       <c r="D72" t="str">
-        <v>Improvement</v>
+        <v>Build לפרסום נכשל — שגיאות TypeScript: draggable ב-SVG, show_in_driver חסר, route_type חסר, קוד מת עם פונקציות לא מוגדרות</v>
       </c>
       <c r="E72" t="str">
-        <v>Strip window: waypoint mode (מקבל/מוסר) now shown as a prominent colored banner bar between the cell header and strips list — green for מקבל, orange for מוסר. Removed small badge from header bar.</v>
+        <v>✓</v>
       </c>
       <c r="F72" t="str">
-        <v>Done</v>
+        <v>תוקן — 6 שגיאות TypeScript</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B73">
-        <v>72</v>
+      <c r="B73" t="str">
+        <v>2026-06-19 14:41</v>
       </c>
       <c r="C73" t="str">
-        <v>2026-06-19</v>
+        <v>תכולה חדשה</v>
       </c>
       <c r="D73" t="str">
-        <v>Bug</v>
+        <v>הגדרת חלון סטריפים — אפשרות בחירת מרקם רקע (9 מרקמים: נקודות, גריד, אלכסוני, קווים, רשת, לוח שחמט)</v>
       </c>
       <c r="E73" t="str">
-        <v>Strip window workstation crash: swSectors (admin-only var) used in workstation rendering — replaced with allSectors (main component state). Caused ReferenceError on any strip window workstation load.</v>
+        <v>כן</v>
       </c>
       <c r="F73" t="str">
-        <v>Fixed</v>
+        <v>06c201b</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B74">
-        <v>73</v>
+      <c r="B74" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C74" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D74" t="str">
-        <v>Feature</v>
+        <v>Strip window — מוסר cell: drag strip onto cell → triggers handleTransfer to the waypoint sector; if multiple workstations on that sector → picker dialog asks which one. מקבל cell: each strip shows ✅ קבל פמ"מ button that calls handleAcceptTransfer. Cannot drag onto a מקבל cell.</v>
       </c>
       <c r="E74" t="str">
-        <v>Strip window — מוסר cell: drag strip onto cell → triggers handleTransfer to the waypoint sector; if multiple workstations on that sector → picker dialog asks which one. מקבל cell: each strip shows ✅ קבל פמ"מ button that calls handleAcceptTransfer. Cannot drag onto a מקבל cell.</v>
+        <v>כן</v>
       </c>
       <c r="F74" t="str">
-        <v>Done</v>
+        <v>#73</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B75">
-        <v>74</v>
+      <c r="B75" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C75" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D75" t="str">
-        <v>Bug</v>
+        <v>מסך כניסה — תפריט בחירת עמדה: טקסט מופיע כחול במקרים מסוימים. תוקן ע"י הוספת color: #0f172a לסלקט</v>
       </c>
       <c r="E75" t="str">
-        <v>מסך כניסה — תפריט בחירת עמדה: טקסט מופיע כחול במקרים מסוימים. תוקן ע"י הוספת color: #0f172a לסלקט</v>
+        <v>כן</v>
       </c>
       <c r="F75" t="str">
-        <v>Done</v>
+        <v>#74</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B76">
-        <v>75</v>
+      <c r="B76" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C76" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D76" t="str">
-        <v>Feature</v>
+        <v>החלפת משתמש בעמדה — מציג רק משתמשים עם הרשאה לעמדה הנוכחית (approved_workstations). מנהלים ומשתמשים ללא הגבלה תמיד מוצגים.</v>
       </c>
       <c r="E76" t="str">
-        <v>החלפת משתמש בעמדה — מציג רק משתמשים עם הרשאה לעמדה הנוכחית (approved_workstations). מנהלים ומשתמשים ללא הגבלה תמיד מוצגים.</v>
+        <v>כן</v>
       </c>
       <c r="F76" t="str">
-        <v>Done</v>
+        <v>#75</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B77">
-        <v>76</v>
+      <c r="B77" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C77" t="str">
-        <v>2026-06-20</v>
+        <v>Bug+Feature</v>
       </c>
       <c r="D77" t="str">
-        <v>Bug+Feature</v>
+        <v>חלון סטריפים — (1) תא מוסר: סטריפ שהועבר נשאר גלוי בתא (תוקן: מקור strips במקום myTableStrips + swLeafAssign מיידי). (2) תא מקבל: גרירה לתא אחר = קבלה אוטומטית של ההעברה, ללא צורך בכפתור נפרד.</v>
       </c>
       <c r="E77" t="str">
-        <v>חלון סטריפים — (1) תא מוסר: סטריפ שהועבר נשאר גלוי בתא (תוקן: מקור strips במקום myTableStrips + swLeafAssign מיידי). (2) תא מקבל: גרירה לתא אחר = קבלה אוטומטית של ההעברה, ללא צורך בכפתור נפרד.</v>
+        <v>כן</v>
       </c>
       <c r="F77" t="str">
-        <v>Done</v>
+        <v>#76</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B78">
-        <v>77</v>
+      <c r="B78" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C78" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D78" t="str">
-        <v>Bug</v>
+        <v>חלון סטריפים מוסר: (1) picker עמדות לא הופיע כשהפילטר הספציפי (relevant_sectors) לא מצא — כעת fallback לכל העמדות האחרות. (2) ריכוז קשרים הציג כל העמדות (targetPid=null) — תוקן באותו fallback. שני התיקונים ב-onDrop וב-handleTransfer.</v>
       </c>
       <c r="E78" t="str">
-        <v>חלון סטריפים מוסר: (1) picker עמדות לא הופיע כשהפילטר הספציפי (relevant_sectors) לא מצא — כעת fallback לכל העמדות האחרות. (2) ריכוז קשרים הציג כל העמדות (targetPid=null) — תוקן באותו fallback. שני התיקונים ב-onDrop וב-handleTransfer.</v>
+        <v>כן</v>
       </c>
       <c r="F78" t="str">
-        <v>Done</v>
+        <v>#77</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B79">
-        <v>78</v>
+      <c r="B79" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C79" t="str">
-        <v>2026-06-20</v>
+        <v>UI</v>
       </c>
       <c r="D79" t="str">
-        <v>UI</v>
+        <v>חלון סטריפים — תג מוסר/מקבל הועבר מבאנר נפרד מתחת לכותרת לתוך שורת הכותרת עצמה (צד ימין)</v>
       </c>
       <c r="E79" t="str">
-        <v>חלון סטריפים — תג מוסר/מקבל הועבר מבאנר נפרד מתחת לכותרת לתוך שורת הכותרת עצמה (צד ימין)</v>
+        <v>כן</v>
       </c>
       <c r="F79" t="str">
-        <v>Done</v>
+        <v>#78</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B80">
-        <v>79</v>
+      <c r="B80" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C80" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D80" t="str">
-        <v>Bug</v>
+        <v>חלון סטריפים — סטריפ שנמסר (pending_transfer) לא ניתן לגרירה חזרה ללוח. רק תא מקבל מאפשר גרירה של pending_transfer (כי שם גרירה = קבלה).</v>
       </c>
       <c r="E80" t="str">
-        <v>חלון סטריפים — סטריפ שנמסר (pending_transfer) לא ניתן לגרירה חזרה ללוח. רק תא מקבל מאפשר גרירה של pending_transfer (כי שם גרירה = קבלה).</v>
+        <v>כן</v>
       </c>
       <c r="F80" t="str">
-        <v>Done</v>
+        <v>#79</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B81">
-        <v>80</v>
+      <c r="B81" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C81" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D81" t="str">
-        <v>Feature</v>
+        <v>חלון סטריפים — גרירת סטריפ שנמסר (pending_transfer) לתא רגיל מבטלת העברה דרך API (/transfers/:id/cancel). גרירה שוב מאופשרת לכל הסטריפים.</v>
       </c>
       <c r="E81" t="str">
-        <v>חלון סטריפים — גרירת סטריפ שנמסר (pending_transfer) לתא רגיל מבטלת העברה דרך API (/transfers/:id/cancel). גרירה שוב מאופשרת לכל הסטריפים.</v>
+        <v>כן</v>
       </c>
       <c r="F81" t="str">
-        <v>Done</v>
+        <v>#80</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B82">
-        <v>81</v>
+      <c r="B82" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C82" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D82" t="str">
-        <v>Bug</v>
+        <v>חלון סטריפים — picker עמדות בתא מוסר הציג כל העמדות כשלא היו מתאימות ספציפיות. תוקן: אין fallback לכולם — מציג רק עמדות עם relevant_sectors/classic_receive_points מתאים לסקטור. אם 0 → שלח ללא יעד, 1 → שלח ישירות, 2+ → picker. גם תוקן ב-contacts targetPid.</v>
       </c>
       <c r="E82" t="str">
-        <v>חלון סטריפים — picker עמדות בתא מוסר הציג כל העמדות כשלא היו מתאימות ספציפיות. תוקן: אין fallback לכולם — מציג רק עמדות עם relevant_sectors/classic_receive_points מתאים לסקטור. אם 0 → שלח ללא יעד, 1 → שלח ישירות, 2+ → picker. גם תוקן ב-contacts targetPid.</v>
+        <v>כן</v>
       </c>
       <c r="F82" t="str">
-        <v>Done</v>
+        <v>#81</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B83">
-        <v>82</v>
+      <c r="B83" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C83" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D83" t="str">
-        <v>Feature</v>
+        <v>חלון סטריפים — גרירה בתוך אותו תא משנה סדר (swLeafOrder). קו כחול מציין נקודת הכנסה. תאי מוסר/מקבל לא מושפעים.</v>
       </c>
       <c r="E83" t="str">
-        <v>חלון סטריפים — גרירה בתוך אותו תא משנה סדר (swLeafOrder). קו כחול מציין נקודת הכנסה. תאי מוסר/מקבל לא מושפעים.</v>
+        <v>כן</v>
       </c>
       <c r="F83" t="str">
-        <v>Done</v>
+        <v>#82</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B84">
-        <v>83</v>
+      <c r="B84" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C84" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D84" t="str">
-        <v>Bug</v>
+        <v>פאנל קשרים נפתח אוטומטית עם כל העמדות כשלא זוהתה עמדת יעד ספציפית. תוקן: פאנל נפתח רק כשיש targetPid ידוע.</v>
       </c>
       <c r="E84" t="str">
-        <v>פאנל קשרים נפתח אוטומטית עם כל העמדות כשלא זוהתה עמדת יעד ספציפית. תוקן: פאנל נפתח רק כשיש targetPid ידוע.</v>
+        <v>כן</v>
       </c>
       <c r="F84" t="str">
-        <v>Done</v>
+        <v>#83</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B85">
-        <v>84</v>
+      <c r="B85" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C85" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D85" t="str">
-        <v>Bug</v>
+        <v>פאנל קשרים אחרי העברה: כשיש מספר עמדות מחוברות לסקטור, מציג רק את הקשרים של אותן עמדות ספציפיות (לא כל העמדות). הוספת state contactsSummarySpecificIds.</v>
       </c>
       <c r="E85" t="str">
-        <v>פאנל קשרים אחרי העברה: כשיש מספר עמדות מחוברות לסקטור, מציג רק את הקשרים של אותן עמדות ספציפיות (לא כל העמדות). הוספת state contactsSummarySpecificIds.</v>
+        <v>כן</v>
       </c>
       <c r="F85" t="str">
-        <v>Done</v>
+        <v>#84</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B86">
-        <v>85</v>
+      <c r="B86" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C86" t="str">
-        <v>2026-06-20</v>
+        <v>Bug</v>
       </c>
       <c r="D86" t="str">
-        <v>Bug</v>
+        <v>חלון סטריפים — ציורי עט על הרקע (לא על פמ) נעלמו כשכובה מצב עט. תוקן: canvas נשאר zIndex:5 גם כשכבוי (מעל content div zIndex:2), עם pointerEvents:none.</v>
       </c>
       <c r="E86" t="str">
-        <v>חלון סטריפים — ציורי עט על הרקע (לא על פמ) נעלמו כשכובה מצב עט. תוקן: canvas נשאר zIndex:5 גם כשכבוי (מעל content div zIndex:2), עם pointerEvents:none.</v>
+        <v>כן</v>
       </c>
       <c r="F86" t="str">
-        <v>Done</v>
+        <v>#85</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B87">
-        <v>86</v>
+      <c r="B87" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C87" t="str">
-        <v>2026-06-20</v>
+        <v>Bug Fix</v>
       </c>
       <c r="D87" t="str">
-        <v>Bug Fix</v>
+        <v>חלון סטריפים: ציורי רקע (pen strokes on background) לא נשמרים / מוצגים מתחת לרקע</v>
       </c>
       <c r="E87" t="str">
-        <v>חלון סטריפים: ציורי רקע (pen strokes on background) לא נשמרים / מוצגים מתחת לרקע</v>
+        <v>כן</v>
       </c>
       <c r="F87" t="str">
-        <v>Fixed: added stable swDoRedraw useCallback + useEffect on swStrokes+swPenMode change; bumped canvas zIndex to 15 when pen-mode off</v>
+        <v>#86 — Fixed: added stable swDoRedraw useCallback + useEffect on swStrokes+swPenMode change; bumped canvas zIndex to 15 when pen-mode off</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B88">
-        <v>87</v>
+      <c r="B88" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C88" t="str">
-        <v>2026-06-20</v>
+        <v>Bug Fix</v>
       </c>
       <c r="D88" t="str">
-        <v>Bug Fix</v>
+        <v>חלון סטריפים: ציורי רקע לא תמיד נשמרים על התא</v>
       </c>
       <c r="E88" t="str">
-        <v>חלון סטריפים: ציורי רקע לא תמיד נשמרים על התא</v>
+        <v>כן</v>
       </c>
       <c r="F88" t="str">
-        <v>Removed duplicate redraw useEffect; upgraded swDoRedraw to use requestAnimationFrame so layout completes before canvas is measured+drawn</v>
+        <v>#87 — Removed duplicate redraw useEffect; upgraded swDoRedraw to use requestAnimationFrame so layout completes before canvas is measured+drawn</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B89">
-        <v>88</v>
+      <c r="B89" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C89" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D89" t="str">
-        <v>Feature</v>
+        <v>חלון סטריפים: גרירת פמ"מ חופשית בתוך תא (מיקום חופשי, לא רשימה)</v>
       </c>
       <c r="E89" t="str">
-        <v>חלון סטריפים: גרירת פמ"מ חופשית בתוך תא (מיקום חופשי, לא רשימה)</v>
+        <v>כן</v>
       </c>
       <c r="F89" t="str">
-        <v>Free absolute positioning per strip per leaf (swFreePos). Drag within same cell sets Y position; collision avoidance prevents overlap; blue line indicator; persisted to localStorage.</v>
+        <v>#88 — Free absolute positioning per strip per leaf (swFreePos). Drag within same cell sets Y position; collision avoidance prevents overlap; blue line indicator; persisted to localStorage.</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B90">
-        <v>89</v>
+      <c r="B90" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C90" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D90" t="str">
-        <v>Feature</v>
+        <v>חלון סטריפים: כפתורי יישור פמ"מ למעלה/למטה בכותרת כל תא</v>
       </c>
       <c r="E90" t="str">
-        <v>חלון סטריפים: כפתורי יישור פמ"מ למעלה/למטה בכותרת כל תא</v>
+        <v>כן</v>
       </c>
       <c r="F90" t="str">
-        <v>Added ⬆ and ⬇ buttons in each leaf header — ⬆ snaps all strips to top (stacked from y=4), ⬇ snaps to bottom of cell using clientHeight</v>
+        <v>#89 — Added ⬆ and ⬇ buttons in each leaf header — ⬆ snaps all strips to top (stacked from y=4), ⬇ snaps to bottom of cell using clientHeight</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B91">
-        <v>90</v>
+      <c r="B91" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C91" t="str">
-        <v>2026-06-20</v>
+        <v>Bug Fix</v>
       </c>
       <c r="D91" t="str">
-        <v>Bug Fix</v>
+        <v>עט ברקע חלון סטריפים - קווים לא נשמרים</v>
       </c>
       <c r="E91" t="str">
-        <v>עט ברקע חלון סטריפים - קווים לא נשמרים</v>
+        <v>כן</v>
       </c>
       <c r="F91" t="str">
-        <v>הוסר requestAnimationFrame מ-swDoRedraw (useEffect כבר רץ אחרי layout). הוסף guard: אם swIsDrawing.current=true מדלג על clear+redraw כדי לא למחוק ציור פעיל</v>
+        <v>#90 — הוסר requestAnimationFrame מ-swDoRedraw (useEffect כבר רץ אחרי layout). הוסף guard: אם swIsDrawing.current=true מדלג על clear+redraw כדי לא למחוק ציור פעיל</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B92">
-        <v>91</v>
+      <c r="B92" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C92" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D92" t="str">
-        <v>Feature</v>
+        <v>שדות חדשים לפמ"מ: הועבר לעמדה + כיוון פ"מ</v>
       </c>
       <c r="E92" t="str">
-        <v>שדות חדשים לפמ"מ: הועבר לעמדה + כיוון פ"מ</v>
+        <v>כן</v>
       </c>
       <c r="F92" t="str">
-        <v>הועבר לעמדה: שם עמדה מ-workstation_preset_id (JOIN בשרת). כיוון פ"מ: מחושב מ-coord_n של בסיס המראה vs בסיס נחיתה — דרומה/צפונה. זמין בכל תצוגות הסטריפ, בפילטרים ובשורות ה-table mode</v>
+        <v>#91 — הועבר לעמדה: שם עמדה מ-workstation_preset_id (JOIN בשרת). כיוון פ"מ: מחושב מ-coord_n של בסיס המראה vs בסיס נחיתה — דרומה/צפונה. זמין בכל תצוגות הסטריפ, בפילטרים ובשורות ה-table mode</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
         <v>1.0.0</v>
       </c>
-      <c r="B93">
-        <v>92</v>
+      <c r="B93" t="str">
+        <v>2026-06-20</v>
       </c>
       <c r="C93" t="str">
-        <v>2026-06-20</v>
+        <v>Feature</v>
       </c>
       <c r="D93" t="str">
-        <v>Feature</v>
+        <v>הזנת נ"צ בסיס בפורמט מעלות-דקות-שניות</v>
       </c>
       <c r="E93" t="str">
-        <v>הזנת נ"צ בסיס בפורמט מעלות-דקות-שניות</v>
+        <v>כן</v>
       </c>
       <c r="F93" t="str">
-        <v>טופס "✈️ בסיסים" ב-admin: שדות coord_n/coord_e הוחלפו ב-3 תתי-שדות לכל קואורדינטה (מעלות/דקות/שניות). המרה ל-decimal בשמירה, המרה מ-decimal בעריכה. תצוגת הרשימה מציגה פורמט 32°15′30″N</v>
+        <v>#92 — טופס "✈️ בסיסים" ב-admin: שדות coord_n/coord_e הוחלפו ב-3 תתי-שדות לכל קואורדינטה (מעלות/דקות/שניות). המרה ל-decimal בשמירה, המרה מ-decimal בעריכה. תצוגת הרשימה מציגה פורמט 32°15′30″N</v>
       </c>
     </row>
     <row r="94">
@@ -2274,10 +2282,10 @@
         <v>ייצוא מלא של כל ה-DB מ-Replit ל-Neon — 86 טבלאות, 4,404 שורות</v>
       </c>
       <c r="E94" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F94" t="str">
-        <v/>
+        <v>833e093</v>
       </c>
     </row>
     <row r="95">
@@ -2294,10 +2302,10 @@
         <v>החזרת חיבור DB ל-Replit המקומי (ביטול Neon)</v>
       </c>
       <c r="E95" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F95" t="str">
-        <v/>
+        <v>6c0a652</v>
       </c>
     </row>
     <row r="96">
@@ -2594,10 +2602,10 @@
         <v>הוספת תשתית בדיקות (vitest) + בדיקות יחידה ל-utils הטהורים</v>
       </c>
       <c r="E110" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F110" t="str">
-        <v/>
+        <v>ad78dd8, 8af51de</v>
       </c>
     </row>
     <row r="111">
@@ -3074,7 +3082,7 @@
         <v>איחוד ופיצול עמדות — בקר אחד מנהל כמה עמדות/סקטורים במסך מאוחד (combine), עם פיצול חזרה לעמדות נפרדות</v>
       </c>
       <c r="E134" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F134" t="str">
         <v>feature/position-merge-split (פיתוח מקבילי)</v>
@@ -3474,10 +3482,10 @@
         <v>מצב תצוגת מפה ICON מטוס / פ"מ — toggle ריצה + ב"מ בעמדה + override פר-פ"מ, פונקציונליות זהה</v>
       </c>
       <c r="E154" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F154" t="str">
-        <v/>
+        <v>f4a2d0d, 28a5a63</v>
       </c>
     </row>
     <row r="155">
@@ -3494,10 +3502,10 @@
         <v>מפה כפולה — חלון נקודות העברה ימני למפה2 + שיוך נ"צ→מפה (Slice 3)</v>
       </c>
       <c r="E155" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F155" t="str">
-        <v/>
+        <v>d04afbb, 748efde, 4fb902c</v>
       </c>
     </row>
     <row r="156">
@@ -3514,10 +3522,10 @@
         <v>מספור גרסאות לקובץ הדרישות — כל דרישה חדשה מעלה patch (1.0.0→1.0.1) עם תאריך+שעה</v>
       </c>
       <c r="E156" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F156" t="str">
-        <v/>
+        <v>מומש בסקיל הישן (1.0.0→1.0.3); הסקיל ה-portable אינו ממספר גרסאות</v>
       </c>
     </row>
     <row r="157">
@@ -3534,10 +3542,10 @@
         <v>הצגת מספר גרסה + תאריך ושעה של הגרסה במסך הכניסה (LOGIN)</v>
       </c>
       <c r="E157" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F157" t="str">
-        <v/>
+        <v>16f7d25</v>
       </c>
     </row>
     <row r="158">
@@ -3554,916 +3562,1195 @@
         <v>העברה בדיבור (לחץ קול): תמיכה בהעברה לאזור במפה אם מוגדר — פקודות "לאזור/עבור לאזור/תמשיך לאזור/תמשיך ל/עבור ל/ל", משולב עם הנחיית גבהים. דוגמה: "בננה לאזור 700 צפון"</v>
       </c>
       <c r="E158" t="str">
-        <v/>
+        <v>כן</v>
       </c>
       <c r="F158" t="str">
-        <v/>
+        <v>קיים בקוד: SectorDashboard — פקודות לאזור / עבור לאזור / תמשיך לאזור</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
+        <v/>
+      </c>
+      <c r="B159" t="str">
         <v>2026-07-08 11:43</v>
       </c>
-      <c r="B159" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C159" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D159" t="str">
         <v>בהגדרת עמדה: אפשרות לקבע נקודת העברה כ"שלמה" או כ"חץ בלבד"</v>
       </c>
-      <c r="D159" t="str">
-        <v/>
-      </c>
       <c r="E159" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F159" t="str">
+        <v>d815b02 + PR #2 (27348a2)</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
+        <v/>
+      </c>
+      <c r="B160" t="str">
         <v>2026-07-08 11:43</v>
       </c>
-      <c r="B160" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C160" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D160" t="str">
         <v>הקטנת נקודת העברה מסוג "חץ" בחצי</v>
       </c>
-      <c r="D160" t="str">
-        <v/>
-      </c>
       <c r="E160" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F160" t="str">
+        <v>d815b02</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
+        <v/>
+      </c>
+      <c r="B161" t="str">
         <v>2026-07-08 11:43</v>
       </c>
-      <c r="B161" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C161" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D161" t="str">
         <v>פ"מ שמתקבל בנקודת העברה: להוסיף פעולת "אשר" (אישרתי קבלה, עדיין לא עבר אליי) ו"דחה"+הערה, לצד "קבל" הקיים</v>
       </c>
-      <c r="D161" t="str">
-        <v/>
-      </c>
       <c r="E161" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F161" t="str">
+        <v>d815b02</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
+        <v/>
+      </c>
+      <c r="B162" t="str">
         <v>2026-07-08 11:43</v>
       </c>
-      <c r="B162" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C162" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D162" t="str">
         <v>בדחייה עם הערה: להקפיץ POPUP בעמדה שמסרה עם ההערה</v>
       </c>
-      <c r="D162" t="str">
-        <v/>
-      </c>
       <c r="E162" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F162" t="str">
+        <v>d815b02</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
+        <v/>
+      </c>
+      <c r="B163" t="str">
         <v>2026-07-08 11:43</v>
       </c>
-      <c r="B163" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C163" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D163" t="str">
         <v>בעמדה שמסרה: פ"מ שאושר יצבע רקע ירוק, נדחה כתום (אדום נשאר לקונפליקט)</v>
       </c>
-      <c r="D163" t="str">
-        <v/>
-      </c>
       <c r="E163" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F163" t="str">
+        <v>d815b02</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
+        <v/>
+      </c>
+      <c r="B164" t="str">
         <v>2026-07-12 19:28</v>
       </c>
-      <c r="B164" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C164" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D164" t="str">
         <v>דו-לשוניות: לכל שדה/פעולה/טקסט שם עברי (קיים) + שם אנגלי</v>
       </c>
-      <c r="D164" t="str">
-        <v/>
-      </c>
       <c r="E164" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F164" t="str">
+        <v>94ff122 — 1393/1393 מפתחות מתורגמים</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
+        <v/>
+      </c>
+      <c r="B165" t="str">
         <v>2026-07-12 19:28</v>
       </c>
-      <c r="B165" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C165" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D165" t="str">
         <v>בורר שפה (עברית/אנגלית) במסך LOGIN, ברירת מחדל עברית</v>
       </c>
-      <c r="D165" t="str">
-        <v/>
-      </c>
       <c r="E165" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F165" t="str">
+        <v>94ceba3</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
+        <v/>
+      </c>
+      <c r="B166" t="str">
         <v>2026-07-12 19:28</v>
       </c>
-      <c r="B166" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C166" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D166" t="str">
         <v>בחירת השפה ב-LOGIN משפיעה על כל המערכת (כולל RTL/LTR מלא)</v>
       </c>
-      <c r="D166" t="str">
-        <v/>
-      </c>
       <c r="E166" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F166" t="str">
+        <v>487ee1c, 9cd1153 — RTL/LTR מלא</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
+        <v/>
+      </c>
+      <c r="B167" t="str">
         <v>2026-07-13 17:32</v>
       </c>
-      <c r="B167" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C167" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D167" t="str">
         <v>טבלת תרגומים: שם שדה טכני | שם עברי | שם אנגלי — לעריכה בלי שינוי קוד</v>
       </c>
-      <c r="D167" t="str">
-        <v/>
-      </c>
       <c r="E167" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F167" t="str">
+        <v>abf81fb</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
+        <v/>
+      </c>
+      <c r="B168" t="str">
         <v>2026-07-13 17:32</v>
       </c>
-      <c r="B168" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C168" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D168" t="str">
         <v>הטבלה מחולקת לקבוצות לוגיות (לפי דומיין) לניווט נוח</v>
       </c>
-      <c r="D168" t="str">
-        <v/>
-      </c>
       <c r="E168" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F168" t="str">
+        <v>abf81fb</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
+        <v/>
+      </c>
+      <c r="B169" t="str">
         <v>2026-07-13 17:32</v>
       </c>
-      <c r="B169" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C169" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D169" t="str">
         <v>כל שדה/פעולה חדשים נרשמים אוטומטית לטבלה</v>
       </c>
-      <c r="D169" t="str">
-        <v/>
-      </c>
       <c r="E169" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F169" t="str">
+        <v>2d89d7d — CI guard אוכף רישום בטבלה</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
+        <v/>
+      </c>
+      <c r="B170" t="str">
         <v>2026-07-15 10:04</v>
       </c>
-      <c r="B170" t="str">
+      <c r="C170" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C170" t="str">
+      <c r="D170" t="str">
         <v>איחוד עמדות: העברת פ"מ מהעמדה המאוחדת מזוהה כאילו העמדה השנייה מסרה, לא אני — צד מוסר/מקבל שגוי</v>
       </c>
-      <c r="D170" t="str">
-        <v/>
-      </c>
       <c r="E170" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F170" t="str">
+        <v>c0871a9, b5f015e</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
+        <v/>
+      </c>
+      <c r="B171" t="str">
         <v>2026-07-15 10:04</v>
       </c>
-      <c r="B171" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C171" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D171" t="str">
         <v>הוספת "עמדת מקור" + "עמדה נוכחית מאוחדת" לפ"מ; במאוחד — אני המוסר, קבלה = אליי; בפיצול — ביטול העמדה המאוחדת וחזרה לעמדת המקור</v>
       </c>
-      <c r="D171" t="str">
-        <v/>
-      </c>
       <c r="E171" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F171" t="str">
+        <v>c0871a9, b5f015e</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
+        <v/>
+      </c>
+      <c r="B172" t="str">
         <v>2026-07-15 16:59</v>
       </c>
-      <c r="B172" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C172" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D172" t="str">
         <v>תפריט "יצירה" חדש בסרגל העליון (מסגרת ליצירות עתידיות)</v>
       </c>
-      <c r="D172" t="str">
-        <v/>
-      </c>
       <c r="E172" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F172" t="str">
+        <v>0063cb0</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
+        <v/>
+      </c>
+      <c r="B173" t="str">
         <v>2026-07-15 16:59</v>
       </c>
-      <c r="B173" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C173" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D173" t="str">
         <v>נקודת העברה פרוביזורית (זמנית) בין 2 עמדות — לא במסך ניהול. טופס: שם, עמדה שנייה, הערות</v>
       </c>
-      <c r="D173" t="str">
-        <v/>
-      </c>
       <c r="E173" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F173" t="str">
+        <v>0606e4c, 0063cb0</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
+        <v/>
+      </c>
+      <c r="B174" t="str">
         <v>2026-07-15 16:59</v>
       </c>
-      <c r="B174" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C174" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D174" t="str">
         <v>אישור נקודה זמנית בעמדה השנייה: תפריט "יצירה" מהבהב + "אשר נקודת העברה זמנית"</v>
       </c>
-      <c r="D174" t="str">
-        <v/>
-      </c>
       <c r="E174" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F174" t="str">
+        <v>0063cb0</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
+        <v/>
+      </c>
+      <c r="B175" t="str">
         <v>2026-07-15 16:59</v>
       </c>
-      <c r="B175" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C175" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D175" t="str">
         <v>נקודה זמנית נשמרת ב-DB זמנית; נמחקת אוטומטית אם לא שמו בה פ"ממים מעל 12 שעות ואחרי חצות</v>
       </c>
-      <c r="D175" t="str">
-        <v/>
-      </c>
       <c r="E175" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F175" t="str">
+        <v>קיים בקוד: cleanupProvisionalTransferPoints — מעל 12 שעות וגם אחרי חצות</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
+        <v/>
+      </c>
+      <c r="B176" t="str">
         <v>2026-07-17 01:43</v>
       </c>
-      <c r="B176" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C176" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D176" t="str">
         <v>תוכנית אספקה: פירוק המערכת ל-17 אבני בניין עם תכולות לכל אחת (DELIVERY_PLAN.md)</v>
       </c>
-      <c r="D176" t="str">
-        <v/>
-      </c>
       <c r="E176" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F176" t="str">
+        <v>DELIVERY_PLAN.md</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
+        <v/>
+      </c>
+      <c r="B177" t="str">
         <v>2026-07-17 01:43</v>
       </c>
-      <c r="B177" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C177" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D177" t="str">
         <v>אומדני זמן פיתוח ריאליים לכל אבן בניין — כאילו נבנה בבית תוכנה חיצוני (ימי-אדם + יומן)</v>
       </c>
-      <c r="D177" t="str">
-        <v/>
-      </c>
       <c r="E177" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F177" t="str">
+        <v>DELIVERY_PLAN.md — אומדנים, לא מאומתים</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
+        <v/>
+      </c>
+      <c r="B178" t="str">
         <v>2026-07-17 01:43</v>
       </c>
-      <c r="B178" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C178" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D178" t="str">
         <v>תוכנית שחרור בגרסאות R1-R6 — מסירת המערכת למשתמש בחלקים, כל גרסה עומדת בפני עצמה</v>
       </c>
-      <c r="D178" t="str">
-        <v/>
-      </c>
       <c r="E178" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F178" t="str">
+        <v>DELIVERY_PLAN.md — R1-R6</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
+        <v/>
+      </c>
+      <c r="B179" t="str">
         <v>2026-07-17 01:43</v>
       </c>
-      <c r="B179" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C179" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D179" t="str">
         <v>7 סטוריות חדשות (US-110..US-116) שקיימות בקוד וחסרות ב-USER_STORIES.md — i18n, תמות, real-time, audit, נק' העברה זמניות, Query</v>
       </c>
-      <c r="D179" t="str">
-        <v/>
-      </c>
       <c r="E179" t="str">
         <v/>
+      </c>
+      <c r="F179" t="str">
+        <v>לא בוצע: USER_STORIES.md מגיע עד US-103, אין US-110 עד US-116</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
+        <v/>
+      </c>
+      <c r="B180" t="str">
         <v>2026-07-17 16:37</v>
       </c>
-      <c r="B180" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C180" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D180" t="str">
         <v>תרגום ה-NDA לאנגלית + ייצוא ל-Word (LTR)</v>
       </c>
-      <c r="D180" t="str">
-        <v/>
-      </c>
       <c r="E180" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F180" t="str">
+        <v>legal/NDA-en.md + NDA-en.docx</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
+        <v/>
+      </c>
+      <c r="B181" t="str">
         <v>2026-07-20 13:20</v>
       </c>
-      <c r="B181" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C181" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D181" t="str">
         <v>הערכת CTO: מוכנות המערכת ל-production והכנסה לחיל האוויר — דירוג Go/No-Go לכל היבט + עלויות בישראל + המלצה rebuild מול המשך</v>
       </c>
-      <c r="D181" t="str">
-        <v/>
-      </c>
       <c r="E181" t="str">
         <v/>
+      </c>
+      <c r="F181" t="str">
+        <v>לא נמצא קובץ בריפו — ככל הנראה נמסר כניתוח בשיחה בלבד</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
+        <v/>
+      </c>
+      <c r="B182" t="str">
         <v>2026-07-21 11:00</v>
       </c>
-      <c r="B182" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C182" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D182" t="str">
         <v>דסק משימה כללי: הגדרת מבנה דסק במסך הניהול (כמו אפיון מסך סטריפים)</v>
       </c>
-      <c r="D182" t="str">
-        <v>כן</v>
-      </c>
       <c r="E182" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F182" t="str">
         <v/>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
+        <v/>
+      </c>
+      <c r="B183" t="str">
         <v>2026-07-21 11:00</v>
       </c>
-      <c r="B183" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C183" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D183" t="str">
         <v>דסק משימה כללי: שירות "מסך ניהול אמצעים" — כפתורים עם מצבים/צבע/טקסט/פונט/גודל/מיקום + טריגר בעמדה אחרת</v>
       </c>
-      <c r="D183" t="str">
-        <v>כן</v>
-      </c>
       <c r="E183" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F183" t="str">
         <v/>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
+        <v/>
+      </c>
+      <c r="B184" t="str">
         <v>2026-07-21 11:00</v>
       </c>
-      <c r="B184" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C184" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D184" t="str">
         <v>דסק משימה כללי: שירות טקסט חופשי בכתב יד — חלונות עם שורות הפרדה/רווח/כותרות</v>
       </c>
-      <c r="D184" t="str">
-        <v>כן</v>
-      </c>
       <c r="E184" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F184" t="str">
         <v/>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
+        <v/>
+      </c>
+      <c r="B185" t="str">
         <v>2026-07-21 11:00</v>
       </c>
-      <c r="B185" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C185" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D185" t="str">
         <v>דסק משימה כללי: מוד טבלה חכמה — עמודות (טקסט/מספר/V-X/תפריט), עיצוב מותנה, חישובים, שורת סיכום</v>
       </c>
-      <c r="D185" t="str">
-        <v>כן</v>
-      </c>
       <c r="E185" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F185" t="str">
         <v/>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
+        <v/>
+      </c>
+      <c r="B186" t="str">
         <v>2026-07-21 11:00</v>
       </c>
-      <c r="B186" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C186" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D186" t="str">
         <v>דסק משימה כללי: בניית דסק בגרירת שירותים למיקומים בחלון ושמירה</v>
       </c>
-      <c r="D186" t="str">
-        <v>כן</v>
-      </c>
       <c r="E186" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F186" t="str">
         <v/>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
+        <v/>
+      </c>
+      <c r="B187" t="str">
         <v>2026-07-21 11:00</v>
       </c>
-      <c r="B187" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C187" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D187" t="str">
         <v>דסק משימה כללי: עמדה מסוג "דסק משימה כללי" + שיתוף שירות בין עמדות עם סנכרון</v>
       </c>
-      <c r="D187" t="str">
-        <v>כן</v>
-      </c>
       <c r="E187" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F187" t="str">
         <v/>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
+        <v/>
+      </c>
+      <c r="B188" t="str">
         <v>2026-07-21 11:05</v>
       </c>
-      <c r="B188" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C188" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D188" t="str">
         <v>הפקת מסמך USER STORIES מפורט לכל המערכת + תמחור שעות עבודה של תוכניתן רגיל</v>
       </c>
-      <c r="D188" t="str">
-        <v/>
-      </c>
       <c r="E188" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F188" t="str">
+        <v>USER_STORIES_FULL.md + MVP_PRICING.html</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
+        <v/>
+      </c>
+      <c r="B189" t="str">
         <v>2026-07-21 11:18</v>
       </c>
-      <c r="B189" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C189" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D189" t="str">
         <v>הוצאת מסמך הסטוריות בפורמט קריא (HTML מעוצב) במקום קובץ MD</v>
       </c>
-      <c r="D189" t="str">
-        <v/>
-      </c>
       <c r="E189" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F189" t="str">
+        <v>USER_STORIES_FULL.html</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
+        <v/>
+      </c>
+      <c r="B190" t="str">
         <v>2026-07-21 15:01</v>
       </c>
-      <c r="B190" t="str">
+      <c r="C190" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C190" t="str">
+      <c r="D190" t="str">
         <v>דסק משימה כללי: כפתור + ליצירת דסק לא עובד (אין משוב שגיאה)</v>
       </c>
-      <c r="D190" t="str">
-        <v>כן</v>
-      </c>
       <c r="E190" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F190" t="str">
         <v/>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
+        <v/>
+      </c>
+      <c r="B191" t="str">
         <v>2026-07-21 15:01</v>
       </c>
-      <c r="B191" t="str">
+      <c r="C191" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C191" t="str">
+      <c r="D191" t="str">
         <v>דסק משימה כללי: חסר אייקון בתפריט הצד ליד "דסקי משימה"</v>
       </c>
-      <c r="D191" t="str">
-        <v>כן</v>
-      </c>
       <c r="E191" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F191" t="str">
         <v/>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
+        <v/>
+      </c>
+      <c r="B192" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B192" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C192" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D192" t="str">
         <v>דסק משימה: אמצעים קבועים ונתוני טבלה בהגדרת עמדה — פתיחת הדסק לתצוגת הגדרה (כולל מיקום)</v>
       </c>
-      <c r="D192" t="str">
-        <v>כן</v>
-      </c>
       <c r="E192" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F192" t="str">
         <v/>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
+        <v/>
+      </c>
+      <c r="B193" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B193" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C193" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D193" t="str">
         <v>דסק משימה: הגדרת גודל כפתור באמצעים</v>
       </c>
-      <c r="D193" t="str">
-        <v>כן</v>
-      </c>
       <c r="E193" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F193" t="str">
         <v/>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
+        <v/>
+      </c>
+      <c r="B194" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B194" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C194" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D194" t="str">
         <v>דסק משימה: פעולות מגע במקום קליק ימני (מסך מגע)</v>
       </c>
-      <c r="D194" t="str">
-        <v>כן</v>
-      </c>
       <c r="E194" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F194" t="str">
         <v/>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
+        <v/>
+      </c>
+      <c r="B195" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B195" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C195" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D195" t="str">
         <v>דסק משימה: פלנלית — ניקוי מלא או מחיקה לפי מיקום הסמן</v>
       </c>
-      <c r="D195" t="str">
-        <v>כן</v>
-      </c>
       <c r="E195" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F195" t="str">
         <v/>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
+        <v/>
+      </c>
+      <c r="B196" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B196" t="str">
+      <c r="C196" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C196" t="str">
+      <c r="D196" t="str">
         <v>דסק משימה: כניסה לעמדת דסק שנוצרה כשהדף פתוח העלתה מוד טבלאי (רענון presets)</v>
       </c>
-      <c r="D196" t="str">
-        <v>כן</v>
-      </c>
       <c r="E196" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F196" t="str">
         <v/>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
+        <v/>
+      </c>
+      <c r="B197" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B197" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C197" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D197" t="str">
         <v>דסק משימה: לא להציג שרבוטי עט בתצוגת ההגדרה</v>
       </c>
-      <c r="D197" t="str">
-        <v>כן</v>
-      </c>
       <c r="E197" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F197" t="str">
         <v/>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
+        <v/>
+      </c>
+      <c r="B198" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B198" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C198" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D198" t="str">
         <v>דסק משימה: שינוי גודל כפתור בגרירה (ידית ◢)</v>
       </c>
-      <c r="D198" t="str">
-        <v>כן</v>
-      </c>
       <c r="E198" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F198" t="str">
         <v/>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
+        <v/>
+      </c>
+      <c r="B199" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B199" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C199" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D199" t="str">
         <v>דסק משימה: "מחק הכל" + אייקון מחק שמוחק במעבר הסמן</v>
       </c>
-      <c r="D199" t="str">
-        <v>כן</v>
-      </c>
       <c r="E199" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F199" t="str">
         <v/>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
+        <v/>
+      </c>
+      <c r="B200" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B200" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C200" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D200" t="str">
         <v>דסק משימה: בונה נוסחאות ויזואלי בטבלה (שדה→אופרטור→שדה)</v>
       </c>
-      <c r="D200" t="str">
-        <v>כן</v>
-      </c>
       <c r="E200" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F200" t="str">
         <v/>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
+        <v/>
+      </c>
+      <c r="B201" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B201" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C201" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D201" t="str">
         <v>דסק משימה: סרגל עליון סטנדרטי — שם עמדה/בקר+החלף/הודעה לעמדה/שעון</v>
       </c>
-      <c r="D201" t="str">
-        <v>כן</v>
-      </c>
       <c r="E201" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F201" t="str">
         <v/>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
+        <v/>
+      </c>
+      <c r="B202" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B202" t="str">
+      <c r="C202" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C202" t="str">
+      <c r="D202" t="str">
         <v>מסך ניהול: השורה האחרונה בכל קטגוריה בתפריט הצד נחתכה (flex shrink)</v>
       </c>
-      <c r="D202" t="str">
-        <v>כן</v>
-      </c>
       <c r="E202" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F202" t="str">
         <v/>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
+        <v/>
+      </c>
+      <c r="B203" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B203" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C203" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D203" t="str">
         <v>מסך ניהול: איחוד עיצוב כותרות הקטגוריות בתפריט הצד</v>
       </c>
-      <c r="D203" t="str">
-        <v>כן</v>
-      </c>
       <c r="E203" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F203" t="str">
         <v/>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
+        <v/>
+      </c>
+      <c r="B204" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B204" t="str">
+      <c r="C204" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C204" t="str">
+      <c r="D204" t="str">
         <v>דסק משימה: ערכי תפריט בטבלה — הפסיק נבלע; הוחלף בתת-טבלת ערכים</v>
       </c>
-      <c r="D204" t="str">
-        <v>כן</v>
-      </c>
       <c r="E204" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F204" t="str">
         <v/>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
+        <v/>
+      </c>
+      <c r="B205" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B205" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C205" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D205" t="str">
         <v>דסק משימה: ספליטרים מותאמי מגע/עט בין חלונות הדסק, שמירה פר-עמדה</v>
       </c>
-      <c r="D205" t="str">
-        <v>כן</v>
-      </c>
       <c r="E205" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F205" t="str">
         <v/>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
+        <v/>
+      </c>
+      <c r="B206" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B206" t="str">
+      <c r="C206" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C206" t="str">
+      <c r="D206" t="str">
         <v>דסק משימה: כמות בעמודת V/X ספרה כל תא שסומן אי-פעם</v>
       </c>
-      <c r="D206" t="str">
-        <v>כן</v>
-      </c>
       <c r="E206" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F206" t="str">
         <v/>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
+        <v/>
+      </c>
+      <c r="B207" t="str">
         <v>2026-07-22 10:31</v>
       </c>
-      <c r="B207" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C207" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D207" t="str">
         <v>דסק משימה: הגדרה בעמודת V/X מה נספר — ✔ או ✘</v>
       </c>
-      <c r="D207" t="str">
-        <v>כן</v>
-      </c>
       <c r="E207" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F207" t="str">
         <v/>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
+        <v/>
+      </c>
+      <c r="B208" t="str">
         <v>2026-07-22 11:07</v>
       </c>
-      <c r="B208" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C208" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D208" t="str">
         <v>דסק משימה: כפתורי אמצעים מסתדרים אוטומטית בלי לעלות אחד על השני</v>
       </c>
-      <c r="D208" t="str">
-        <v/>
-      </c>
       <c r="E208" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F208" t="str">
+        <v>30feabd</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
+        <v/>
+      </c>
+      <c r="B209" t="str">
         <v>2026-07-22 11:17</v>
       </c>
-      <c r="B209" t="str">
+      <c r="C209" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C209" t="str">
+      <c r="D209" t="str">
         <v>מסך ניהול: שכפול עמדה — כפתור השמירה נשאר כבוי (presetFormInitial=null)</v>
       </c>
-      <c r="D209" t="str">
-        <v/>
-      </c>
       <c r="E209" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F209" t="str">
+        <v>cb06894</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
+        <v/>
+      </c>
+      <c r="B210" t="str">
         <v>2026-07-22 11:17</v>
       </c>
-      <c r="B210" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C210" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D210" t="str">
         <v>דסק משימה: רשימת השיתוף מציגה רק עמדות מסוג דסק משימה</v>
       </c>
-      <c r="D210" t="str">
-        <v/>
-      </c>
       <c r="E210" t="str">
-        <v/>
+        <v>כן</v>
+      </c>
+      <c r="F210" t="str">
+        <v>cb06894</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
+        <v/>
+      </c>
+      <c r="B211" t="str">
         <v>2026-07-22 11:17</v>
       </c>
-      <c r="B211" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C211" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D211" t="str">
         <v>דסק משימה: שיתוף דו-כיווני — הגדרה בעמדה אחת משתקפת אוטומטית בשנייה</v>
       </c>
-      <c r="D211" t="str">
-        <v/>
-      </c>
       <c r="E211" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F211" t="str">
+        <v>cb06894</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v/>
+      </c>
+      <c r="B212" t="str">
+        <v>2026-07-22 11:26</v>
+      </c>
+      <c r="C212" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D212" t="str">
+        <v>סקיל requirements-tracker לא מופעל אוטומטית על כל בקשת משתמש</v>
+      </c>
+      <c r="E212" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F212" t="str">
+        <v>hook UserPromptSubmit + מיון בסקריפט</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v/>
+      </c>
+      <c r="B213" t="str">
+        <v>2026-07-22 11:26</v>
+      </c>
+      <c r="C213" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D213" t="str">
+        <v>ניהול קובץ הדרישות ממוין לפי תאריך ושעה</v>
+      </c>
+      <c r="E213" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F213" t="str">
+        <v>hook UserPromptSubmit + מיון בסקריפט</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v/>
+      </c>
+      <c r="B214" t="str">
+        <v>2026-07-22 11:26</v>
+      </c>
+      <c r="C214" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D214" t="str">
+        <v>עיגון ב-CLAUDE.md + hook אוטומטי: רישום כל בקשה לקובץ הדרישות</v>
+      </c>
+      <c r="E214" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F214" t="str">
+        <v>hook UserPromptSubmit + מיון בסקריפט</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v/>
+      </c>
+      <c r="B215" t="str">
+        <v>2026-07-22 11:33</v>
+      </c>
+      <c r="C215" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D215" t="str">
+        <v>עדכון רטרואקטיבי של עמודת "בוצע?" לפי מה שמומש בפועל</v>
+      </c>
+      <c r="E215" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F215" t="str">
+        <v>בוצע בסשן זה — 2026-07-22</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v/>
+      </c>
+      <c r="B216" t="str">
+        <v>2026-07-22 11:37</v>
+      </c>
+      <c r="C216" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D216" t="str">
+        <v>דסק משימה: שיתוף רק עם עמדות דסק שבחרו את אותו דסק</v>
+      </c>
+      <c r="E216" t="str">
+        <v/>
+      </c>
+      <c r="F216" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v/>
+      </c>
+      <c r="B217" t="str">
+        <v>2026-07-22 11:43</v>
+      </c>
+      <c r="C217" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D217" t="str">
+        <v>דסק משימה: סרגל עליון בעיצוב הסטנדרטי של כל העמדות (לוגו, כפתור עמדה כחול, משתמש ירוק, שעון)</v>
+      </c>
+      <c r="E217" t="str">
+        <v/>
+      </c>
+      <c r="F217" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F211"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F217"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(mission-desk): real sticky notes + the standard compose modal
Messages and notes now reuse the existing components instead of a
custom implementation: the shared StickyNotesLayer with the standard
'פתקיות' top-bar button (badges, closed-notes dropdown, new-note flow,
15s polling — identical to SectorDashboard), and the message dialog is
the standard purple compose modal (💬, Enter-to-send, 📨 שלח) with a
recipients picker, posting to workstation-messages as before.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,15 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F217"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="72.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F220"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4748,9 +4740,66 @@
         <v/>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v/>
+      </c>
+      <c r="B218" t="str">
+        <v>2026-07-22 11:54</v>
+      </c>
+      <c r="C218" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D218" t="str">
+        <v>דמו מיראז' — אפליקציה נפרדת לניהול משתמשים והרשאות עם API: אפליקציה+מספר אישי → הרשאה+תפקידים</v>
+      </c>
+      <c r="E218" t="str">
+        <v/>
+      </c>
+      <c r="F218" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v/>
+      </c>
+      <c r="B219" t="str">
+        <v>2026-07-22 11:54</v>
+      </c>
+      <c r="C219" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D219" t="str">
+        <v>CHECKBOX במסך LOGIN: בחירה בין משתמשי המערכת להתחברות דרך מיראז'; ברירת מחדל — מיראז'</v>
+      </c>
+      <c r="E219" t="str">
+        <v/>
+      </c>
+      <c r="F219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>2026-07-22 11:55</v>
+      </c>
+      <c r="B220" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C220" t="str">
+        <v>דסק משימה: הודעות ופתקיות — להשתמש ברכיבים הקיימים (compose + פתקיות של שאר העמדות), לא מימוש חדש</v>
+      </c>
+      <c r="D220" t="str">
+        <v/>
+      </c>
+      <c r="E220" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F217"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F220"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mission-desk): drop the invented 'message a position' top-bar button
Other positions have no such button in their bar — messaging happens
through context flows. Removed the chip, modal and its state; incoming
burst-alert toasts and the buttons-service alert triggers are untouched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F220"/>
+  <dimension ref="A1:F222"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4782,24 +4790,67 @@
     </row>
     <row r="220">
       <c r="A220" t="str">
+        <v/>
+      </c>
+      <c r="B220" t="str">
         <v>2026-07-22 11:55</v>
       </c>
-      <c r="B220" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C220" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D220" t="str">
         <v>דסק משימה: הודעות ופתקיות — להשתמש ברכיבים הקיימים (compose + פתקיות של שאר העמדות), לא מימוש חדש</v>
       </c>
-      <c r="D220" t="str">
-        <v/>
-      </c>
       <c r="E220" t="str">
+        <v/>
+      </c>
+      <c r="F220" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v/>
+      </c>
+      <c r="B221" t="str">
+        <v>2026-07-22 12:41</v>
+      </c>
+      <c r="C221" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D221" t="str">
+        <v>דסק משימה: הסרת כפתור "הודעה לעמדה" מהסרגל — לא קיים בסרגל של שאר העמדות</v>
+      </c>
+      <c r="E221" t="str">
+        <v/>
+      </c>
+      <c r="F221" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v/>
+      </c>
+      <c r="B222" t="str">
+        <v>2026-07-22 12:44</v>
+      </c>
+      <c r="C222" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D222" t="str">
+        <v>כניסה דרך מיראז' נכשלת ('שגיאה בכניסה') — נבדק עם 5229214 אורן בן דור</v>
+      </c>
+      <c r="E222" t="str">
+        <v/>
+      </c>
+      <c r="F222" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F220"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F222"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: docker packaging, delivery & legal docs, user stories, project settings
- Dockerfile + docker-compose + .dockerignore (DATABASE_URL injected at
  runtime, never baked into the image)
- DELIVERY_PLAN, MVP_PRICING, USER_STORIES (full md/html/xlsx), legal/NDA (he+en)
- .claude settings: requirements-tracker hook + permissions; tracker skill docs
- mirage auth data update, requirements xlsx log, refreshed e2e screenshots

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,15 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F226"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="72.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F230"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4928,9 +4920,77 @@
         <v/>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>2026-07-22 15:43</v>
+      </c>
+      <c r="B227" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C227" t="str">
+        <v>תמחור תכולות MVP: אומדן שעות עבודה של מתכנת רגיל ומחיר, מפורט לכל שורת תכולה</v>
+      </c>
+      <c r="D227" t="str">
+        <v/>
+      </c>
+      <c r="E227" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>2026-07-22 15:43</v>
+      </c>
+      <c r="B228" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C228" t="str">
+        <v>ייצוא תמחור ה-MVP לפורמט מעוצב — נוצר MVP_PRICING.html (RTL, מוכן להדפסה/PDF)</v>
+      </c>
+      <c r="D228" t="str">
+        <v/>
+      </c>
+      <c r="E228" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>2026-07-22 15:43</v>
+      </c>
+      <c r="B229" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="C229" t="str">
+        <v>אומדן לדוגמה לתכולת פתקיות שיעמוד מול ביקורת חיצונית (WBS+PERT, Function Points, אימות מול קוד קיים)</v>
+      </c>
+      <c r="D229" t="str">
+        <v/>
+      </c>
+      <c r="E229" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>2026-07-22 15:50</v>
+      </c>
+      <c r="B230" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C230" t="str">
+        <v>התאמת תמחור ה-MVP לתמחור בימי עבודה (כמקובל אצל מתכנתים) — גישור שעות נטו מול ימי עבודה בפועל</v>
+      </c>
+      <c r="D230" t="str">
+        <v/>
+      </c>
+      <c r="E230" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F226"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F230"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mirage): Railway-ready — honor injected PORT, bind IPv6 dual-stack
Railway injects PORT and its private network (*.railway.internal) only
reaches services listening on IPv6, so '0.0.0.0'+MIRAGE_PORT made the
service unreachable there. Local behavior unchanged (7300, IPv4 still
served via dual-stack; verified with a live health check).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F230"/>
+  <dimension ref="A1:F231"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4988,9 +4988,26 @@
         <v/>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>2026-07-22 21:23</v>
+      </c>
+      <c r="B231" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C231" t="str">
+        <v>מיראז: התאמה לריצה כשירות ב-Railway (PORT + רשת פנימית) + הוראות פריסה</v>
+      </c>
+      <c r="D231" t="str">
+        <v/>
+      </c>
+      <c r="E231" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F231"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(docker): include mirage/ in the runtime image
A Railway service created from this repo auto-builds the Dockerfile,
whose runtime stage only copied server/dist/public — so a mirage
service crashed on boot with MODULE_NOT_FOUND (mirage/server.js absent
from the container). The folder is tiny and express is already a prod
dependency, so one image now serves both start commands.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F231"/>
+  <dimension ref="A1:F232"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5005,9 +5005,26 @@
         <v/>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>2026-07-23 08:15</v>
+      </c>
+      <c r="B232" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C232" t="str">
+        <v>מיראז ב-Railway קרס (MODULE_NOT_FOUND) — ה-Dockerfile לא כלל את תיקיית mirage</v>
+      </c>
+      <c r="D232" t="str">
+        <v/>
+      </c>
+      <c r="E232" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F231"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F232"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(mirage): users live in Neon (mirage_users) with file fallback
Pluggable store: Postgres when DATABASE_URL/MIRAGE_DATABASE_URL is set
(production — admin edits survive Railway redeploys), data.json
otherwise (local dev + the 16 offline tests, unchanged). First boot
against an empty table imports the existing data.json users once.
Verified live against Neon: seed import (5 users), create/authorize/
update/duplicate-409/delete all through the DB.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F232"/>
+  <dimension ref="A1:F234"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5022,9 +5022,43 @@
         <v/>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>2026-07-23 08:50</v>
+      </c>
+      <c r="B233" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C233" t="str">
+        <v>מיראז בענן: רשימת העמדות לא נטענת — חסר קישור לשרת SKY-KING (SKYKING_URL)</v>
+      </c>
+      <c r="D233" t="str">
+        <v/>
+      </c>
+      <c r="E233" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>2026-07-23 09:08</v>
+      </c>
+      <c r="B234" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C234" t="str">
+        <v>מיראז: מעבר מ-data.json ל-DB ב-Neon (טבלת mirage_users) — עריכות שורדות פריסות; fallback לקובץ בפיתוח</v>
+      </c>
+      <c r="D234" t="str">
+        <v/>
+      </c>
+      <c r="E234" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F232"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F234"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mirage): quoted workstation names no longer truncated; picker grouped by base and role
Names containing gershayim (בת"ק...) broke unescaped HTML attributes in
the admin screen — the checkbox label and the saved workstation name
were cut at the quote. All interpolated values now HTML-escaped.
The allowed-workstations picker is grouped by parent base (בסיס אב)
with tower/yaba/general sub-groups; /api/workstation-options now
enriches each workstation with role + base name (aviation-bases),
gracefully degrading when unavailable. Verified in a real browser
against live data: 23 stations, quoted names intact, groups rendered.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F234"/>
+  <dimension ref="A1:F240"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4922,143 +4922,281 @@
     </row>
     <row r="227">
       <c r="A227" t="str">
+        <v/>
+      </c>
+      <c r="B227" t="str">
         <v>2026-07-22 15:43</v>
       </c>
-      <c r="B227" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C227" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D227" t="str">
         <v>תמחור תכולות MVP: אומדן שעות עבודה של מתכנת רגיל ומחיר, מפורט לכל שורת תכולה</v>
       </c>
-      <c r="D227" t="str">
-        <v/>
-      </c>
       <c r="E227" t="str">
+        <v/>
+      </c>
+      <c r="F227" t="str">
         <v/>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
+        <v/>
+      </c>
+      <c r="B228" t="str">
         <v>2026-07-22 15:43</v>
       </c>
-      <c r="B228" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C228" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D228" t="str">
         <v>ייצוא תמחור ה-MVP לפורמט מעוצב — נוצר MVP_PRICING.html (RTL, מוכן להדפסה/PDF)</v>
       </c>
-      <c r="D228" t="str">
-        <v/>
-      </c>
       <c r="E228" t="str">
+        <v/>
+      </c>
+      <c r="F228" t="str">
         <v/>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
+        <v/>
+      </c>
+      <c r="B229" t="str">
         <v>2026-07-22 15:43</v>
       </c>
-      <c r="B229" t="str">
-        <v>תכולה חדשה</v>
-      </c>
       <c r="C229" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D229" t="str">
         <v>אומדן לדוגמה לתכולת פתקיות שיעמוד מול ביקורת חיצונית (WBS+PERT, Function Points, אימות מול קוד קיים)</v>
       </c>
-      <c r="D229" t="str">
-        <v/>
-      </c>
       <c r="E229" t="str">
+        <v/>
+      </c>
+      <c r="F229" t="str">
         <v/>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
+        <v/>
+      </c>
+      <c r="B230" t="str">
         <v>2026-07-22 15:50</v>
       </c>
-      <c r="B230" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C230" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D230" t="str">
         <v>התאמת תמחור ה-MVP לתמחור בימי עבודה (כמקובל אצל מתכנתים) — גישור שעות נטו מול ימי עבודה בפועל</v>
       </c>
-      <c r="D230" t="str">
-        <v/>
-      </c>
       <c r="E230" t="str">
+        <v/>
+      </c>
+      <c r="F230" t="str">
         <v/>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
+        <v/>
+      </c>
+      <c r="B231" t="str">
         <v>2026-07-22 21:23</v>
       </c>
-      <c r="B231" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C231" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D231" t="str">
         <v>מיראז: התאמה לריצה כשירות ב-Railway (PORT + רשת פנימית) + הוראות פריסה</v>
       </c>
-      <c r="D231" t="str">
-        <v/>
-      </c>
       <c r="E231" t="str">
+        <v/>
+      </c>
+      <c r="F231" t="str">
         <v/>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
+        <v/>
+      </c>
+      <c r="B232" t="str">
         <v>2026-07-23 08:15</v>
       </c>
-      <c r="B232" t="str">
+      <c r="C232" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C232" t="str">
+      <c r="D232" t="str">
         <v>מיראז ב-Railway קרס (MODULE_NOT_FOUND) — ה-Dockerfile לא כלל את תיקיית mirage</v>
       </c>
-      <c r="D232" t="str">
-        <v/>
-      </c>
       <c r="E232" t="str">
+        <v/>
+      </c>
+      <c r="F232" t="str">
         <v/>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
+        <v/>
+      </c>
+      <c r="B233" t="str">
         <v>2026-07-23 08:50</v>
       </c>
-      <c r="B233" t="str">
+      <c r="C233" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C233" t="str">
+      <c r="D233" t="str">
         <v>מיראז בענן: רשימת העמדות לא נטענת — חסר קישור לשרת SKY-KING (SKYKING_URL)</v>
       </c>
-      <c r="D233" t="str">
-        <v/>
-      </c>
       <c r="E233" t="str">
+        <v/>
+      </c>
+      <c r="F233" t="str">
         <v/>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
+        <v/>
+      </c>
+      <c r="B234" t="str">
         <v>2026-07-23 09:08</v>
       </c>
-      <c r="B234" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C234" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D234" t="str">
         <v>מיראז: מעבר מ-data.json ל-DB ב-Neon (טבלת mirage_users) — עריכות שורדות פריסות; fallback לקובץ בפיתוח</v>
       </c>
-      <c r="D234" t="str">
-        <v/>
-      </c>
       <c r="E234" t="str">
+        <v/>
+      </c>
+      <c r="F234" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v/>
+      </c>
+      <c r="B235" t="str">
+        <v>2026-07-23 09:18</v>
+      </c>
+      <c r="C235" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D235" t="str">
+        <v>מיראז: DB נפרד משלו ב-Neon (לא משותף עם SKY-KING) — MIRAGE_DATABASE_URL</v>
+      </c>
+      <c r="E235" t="str">
+        <v/>
+      </c>
+      <c r="F235" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v/>
+      </c>
+      <c r="B236" t="str">
+        <v>2026-07-23 11:18</v>
+      </c>
+      <c r="C236" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D236" t="str">
+        <v>סביבות תרגול (כמו גלקסיה): סביבות טסות 1-10 בסכמת DB משותפת, סביבות 11-50 בסכמות נפרדות</v>
+      </c>
+      <c r="E236" t="str">
+        <v/>
+      </c>
+      <c r="F236" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v/>
+      </c>
+      <c r="B237" t="str">
+        <v>2026-07-23 11:18</v>
+      </c>
+      <c r="C237" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D237" t="str">
+        <v>מסך כניסה: בחירת סביבת עבודה שממפה לסכמת ה-DB הרלוונטית</v>
+      </c>
+      <c r="E237" t="str">
+        <v/>
+      </c>
+      <c r="F237" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v/>
+      </c>
+      <c r="B238" t="str">
+        <v>2026-07-23 11:18</v>
+      </c>
+      <c r="C238" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D238" t="str">
+        <v>סרגל עליון (ימין): תצוגת הסביבה המחוברת</v>
+      </c>
+      <c r="E238" t="str">
+        <v/>
+      </c>
+      <c r="F238" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>2026-07-23 13:19</v>
+      </c>
+      <c r="B239" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C239" t="str">
+        <v>מיראז: שמות עמדות עם גרשיים נחתכים במסך הניהול (escaping)</v>
+      </c>
+      <c r="D239" t="str">
+        <v/>
+      </c>
+      <c r="E239" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>2026-07-23 13:19</v>
+      </c>
+      <c r="B240" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C240" t="str">
+        <v>מיראז: חלוקת העמדות המורשות לפי מגדל/יב"א ולפי בסיס אב</v>
+      </c>
+      <c r="D240" t="str">
+        <v/>
+      </c>
+      <c r="E240" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F234"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F240"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mirage): local workstation list — IPv4 default, Neon cold-start timeout, error logging
Two stacked causes of the false 'SKY-KING unavailable' locally:
default localhost resolved to ::1 while the dev server is IPv4-only
(now 127.0.0.1), and the 3s fetch timeout aborted on Neon cold starts
(~5.5s first query; now 10s). Failures are logged instead of silent.
npm run mirage now loads .env when present (--env-file-if-exists), so
the local mirage uses its own Neon DB like production.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F240"/>
+  <dimension ref="A1:F241"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5194,9 +5194,26 @@
         <v/>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>2026-07-23 17:28</v>
+      </c>
+      <c r="B241" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C241" t="str">
+        <v>מיראז מקומי (localhost): לא מצליח להביא את העמדות מ-SKY-KING</v>
+      </c>
+      <c r="D241" t="str">
+        <v/>
+      </c>
+      <c r="E241" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F240"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F241"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(server): mirage bridge tolerates Neon cold start (10s timeout, IPv4 default)
The 4s timeout aborted while the mirage's own Neon DB was waking up
(~6s), so the first login of the day returned a false
'mirage_unavailable' — locally and in production alike. Also default
to 127.0.0.1 (Node fetch prefers ::1). Verified end-to-end locally:
login via the Vite proxy answers in ~1.1s.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F241"/>
+  <dimension ref="A1:F242"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5211,9 +5211,26 @@
         <v/>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>2026-07-23 20:53</v>
+      </c>
+      <c r="B242" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C242" t="str">
+        <v>מקומי: כניסת מיראז דרך localhost:5000 לא עובדת</v>
+      </c>
+      <c r="D242" t="str">
+        <v/>
+      </c>
+      <c r="E242" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F241"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F242"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
test+docs: adapt e2e to env-picker login; note training-environments service
After merging training-environments the login screen defaults to mirage
auth and adds an env picker + X-Env header; e2e helpers now switch to
internal auth and scope the workstation <select> away from #env-select.
Bumped a load-sensitive assertion. SHARED_LANGUAGE lists the new
training-environments service (#21).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F242"/>
+  <dimension ref="A1:F247"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5162,75 +5170,187 @@
     </row>
     <row r="239">
       <c r="A239" t="str">
+        <v/>
+      </c>
+      <c r="B239" t="str">
         <v>2026-07-23 13:19</v>
       </c>
-      <c r="B239" t="str">
+      <c r="C239" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C239" t="str">
+      <c r="D239" t="str">
         <v>מיראז: שמות עמדות עם גרשיים נחתכים במסך הניהול (escaping)</v>
       </c>
-      <c r="D239" t="str">
-        <v/>
-      </c>
       <c r="E239" t="str">
+        <v/>
+      </c>
+      <c r="F239" t="str">
         <v/>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
+        <v/>
+      </c>
+      <c r="B240" t="str">
         <v>2026-07-23 13:19</v>
       </c>
-      <c r="B240" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C240" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D240" t="str">
         <v>מיראז: חלוקת העמדות המורשות לפי מגדל/יב"א ולפי בסיס אב</v>
       </c>
-      <c r="D240" t="str">
-        <v/>
-      </c>
       <c r="E240" t="str">
+        <v/>
+      </c>
+      <c r="F240" t="str">
         <v/>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
+        <v/>
+      </c>
+      <c r="B241" t="str">
         <v>2026-07-23 17:28</v>
       </c>
-      <c r="B241" t="str">
+      <c r="C241" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C241" t="str">
+      <c r="D241" t="str">
         <v>מיראז מקומי (localhost): לא מצליח להביא את העמדות מ-SKY-KING</v>
       </c>
-      <c r="D241" t="str">
-        <v/>
-      </c>
       <c r="E241" t="str">
+        <v/>
+      </c>
+      <c r="F241" t="str">
         <v/>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
+        <v/>
+      </c>
+      <c r="B242" t="str">
         <v>2026-07-23 20:53</v>
       </c>
-      <c r="B242" t="str">
+      <c r="C242" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C242" t="str">
+      <c r="D242" t="str">
         <v>מקומי: כניסת מיראז דרך localhost:5000 לא עובדת</v>
       </c>
-      <c r="D242" t="str">
-        <v/>
-      </c>
       <c r="E242" t="str">
+        <v/>
+      </c>
+      <c r="F242" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v/>
+      </c>
+      <c r="B243" t="str">
+        <v>2026-07-23 22:13</v>
+      </c>
+      <c r="C243" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D243" t="str">
+        <v>איחוד ענף איחוד/פיצול עמדות (position-merge-split) לענף הראשי</v>
+      </c>
+      <c r="E243" t="str">
+        <v/>
+      </c>
+      <c r="F243" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v/>
+      </c>
+      <c r="B244" t="str">
+        <v>2026-07-24 08:01</v>
+      </c>
+      <c r="C244" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D244" t="str">
+        <v>בגרירת פ"מ מורחב על מפת אזורים — קדקודי הפוליגונים (נקודות שחורות) "מפצלים" את הכרטיס והוא לא נצמד לקצה אזור</v>
+      </c>
+      <c r="E244" t="str">
+        <v/>
+      </c>
+      <c r="F244" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v/>
+      </c>
+      <c r="B245" t="str">
+        <v>2026-07-24 08:32</v>
+      </c>
+      <c r="C245" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D245" t="str">
+        <v>השגת/הטמעת סמלי בסיסי חה"א, יב"אות ומערך הבקרה כ-assets במערכת</v>
+      </c>
+      <c r="E245" t="str">
+        <v/>
+      </c>
+      <c r="F245" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v/>
+      </c>
+      <c r="B246" t="str">
+        <v>2026-07-24 08:32</v>
+      </c>
+      <c r="C246" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D246" t="str">
+        <v>מסך טעינה של עמדה לפי בסיס: אנימציית סמל הבסיס + סמל מערך הבקרה מסתובבים</v>
+      </c>
+      <c r="E246" t="str">
+        <v/>
+      </c>
+      <c r="F246" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v/>
+      </c>
+      <c r="B247" t="str">
+        <v>2026-07-24 08:32</v>
+      </c>
+      <c r="C247" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D247" t="str">
+        <v>סרגל עליון: הצגת אייקון הבסיס/מערך הבקרה בעליית המערכת</v>
+      </c>
+      <c r="E247" t="str">
+        <v/>
+      </c>
+      <c r="F247" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F242"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F247"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(mission-desk): image and fixed-text services
Two new config-only (read-only at the station) desk services:
- image: paste a screenshot (Ctrl+V) or pick/drop a file in the admin
  editor; stored as a raster data URL in config (SVG rejected —
  isImageDataUrl, unit-tested), auto-downscaled to ~1600px, fit
  contain/cover. Rendered as <img> in the station.
- label: fixed text with font/size/bold/align/color set in the admin,
  with a live preview; rendered read-only in the station.
Server accepts the new service_type values (no migration — VARCHAR(12)
+ JSONB config). Verified: 289 unit tests, API smoke incl. invalid-type
rejection, and a live Playwright render (image loads, label shows).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,15 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F247"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="72.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F259"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5348,9 +5340,249 @@
         <v/>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v/>
+      </c>
+      <c r="B248" t="str">
+        <v>2026-07-26 11:42</v>
+      </c>
+      <c r="C248" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D248" t="str">
+        <v>הורדת הסמלים האמיתיים מהאינטרנט (בסיסי חה"א + מיח"ה) והטמעתם ברכיב RotatingEmblems במקום ה-placeholders</v>
+      </c>
+      <c r="E248" t="str">
+        <v/>
+      </c>
+      <c r="F248" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v/>
+      </c>
+      <c r="B249" t="str">
+        <v>2026-07-26 12:08</v>
+      </c>
+      <c r="C249" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D249" t="str">
+        <v>להחליף מקף כפול/מקף ארוך (em-dash של AI) למקף בודד "-" בכל הפרויקט</v>
+      </c>
+      <c r="E249" t="str">
+        <v/>
+      </c>
+      <c r="F249" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v/>
+      </c>
+      <c r="B250" t="str">
+        <v>2026-07-26 12:15</v>
+      </c>
+      <c r="C250" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D250" t="str">
+        <v>פ"מ מורחב על מפה עם אזורים מתנהג בגרירה כמו פ"מ צף רגיל (מיקום חופשי) במקום להקצות אזור</v>
+      </c>
+      <c r="E250" t="str">
+        <v/>
+      </c>
+      <c r="F250" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v/>
+      </c>
+      <c r="B251" t="str">
+        <v>2026-07-26 12:15</v>
+      </c>
+      <c r="C251" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D251" t="str">
+        <v>להעביר את 3 כפתורי בחירת סוג תצוגת הפ"מ (מורחב/מוקטן/אייקון) ואת הגדל/הקטן מהסרגל התחתון לסרגל השמאלי (מתחת לתצוגת הסגירות)</v>
+      </c>
+      <c r="E251" t="str">
+        <v/>
+      </c>
+      <c r="F251" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v/>
+      </c>
+      <c r="B252" t="str">
+        <v>2026-07-26 12:39</v>
+      </c>
+      <c r="C252" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D252" t="str">
+        <v>החלפת סמל מיח"ה (מערך הבקרה) לרשמי + הוספת סמלי 509 ו-506 (מקורות שסופקו)</v>
+      </c>
+      <c r="E252" t="str">
+        <v/>
+      </c>
+      <c r="F252" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v/>
+      </c>
+      <c r="B253" t="str">
+        <v>2026-07-28 14:34</v>
+      </c>
+      <c r="C253" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D253" t="str">
+        <v>יצירת סקיל /pricing (תמחור): מתודולוגיית אומדן — שעות נטו + ימי עבודה, שני בסיסי תמחור, PERT/FP/מדידת קוד</v>
+      </c>
+      <c r="E253" t="str">
+        <v/>
+      </c>
+      <c r="F253" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v/>
+      </c>
+      <c r="B254" t="str">
+        <v>2026-07-29 16:54</v>
+      </c>
+      <c r="C254" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D254" t="str">
+        <v>דסק משימה: שירות תמונה — הדבקת print-screen ב-paste או הדבקת קובץ בהגדרה</v>
+      </c>
+      <c r="E254" t="str">
+        <v/>
+      </c>
+      <c r="F254" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v/>
+      </c>
+      <c r="B255" t="str">
+        <v>2026-07-29 16:54</v>
+      </c>
+      <c r="C255" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D255" t="str">
+        <v>דסק משימה: שירות טקסט קבוע — נקבע בהגדרת עמדה, עם הגדרת פונט וגודל</v>
+      </c>
+      <c r="E255" t="str">
+        <v/>
+      </c>
+      <c r="F255" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v/>
+      </c>
+      <c r="B256" t="str">
+        <v>2026-07-29 17:00</v>
+      </c>
+      <c r="C256" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D256" t="str">
+        <v>כפתורי בחירת סוג-תצוגת פ"מ בסרגל השמאלי — להגדיל ולהציגם כתצוגה מקדימה חיה של האייקון האמיתי על המפה (או"ק/טייסת רנדומלי להמחשה)</v>
+      </c>
+      <c r="E256" t="str">
+        <v/>
+      </c>
+      <c r="F256" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v/>
+      </c>
+      <c r="B257" t="str">
+        <v>2026-07-29 17:00</v>
+      </c>
+      <c r="C257" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D257" t="str">
+        <v>תצוגת פ"מ "מוקטן" — טקסט מוקטן, והזזת תפריט 3 הנקודות (⋮) לצד כדי שלא יסתיר את האו"ק</v>
+      </c>
+      <c r="E257" t="str">
+        <v/>
+      </c>
+      <c r="F257" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v/>
+      </c>
+      <c r="B258" t="str">
+        <v>2026-07-29 17:00</v>
+      </c>
+      <c r="C258" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D258" t="str">
+        <v>סוג תצוגת פ"מ חדש "כתב יד" — או"ק(מס' מטוסים)/טייסת (לדוג' בננה(2)/120; בפיצול בננה1+3/120)</v>
+      </c>
+      <c r="E258" t="str">
+        <v/>
+      </c>
+      <c r="F258" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v/>
+      </c>
+      <c r="B259" t="str">
+        <v>2026-07-29 17:00</v>
+      </c>
+      <c r="C259" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D259" t="str">
+        <v>פ"מ המחובר לכמה אזורים סמוכים — לצייר פוליגון מקיף בצבע שונה מהאזורים; צבע מחזורי שונה לכל פ"מ עד סוף הרשימה וחזרה</v>
+      </c>
+      <c r="E259" t="str">
+        <v/>
+      </c>
+      <c r="F259" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F247"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F259"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(mission-desk): configure image & fixed-text from the position setup view
Image and label could only be set in the desk-services admin tab; the
user expected to set them where the fixed buttons/rows are set — inside
'open desk for setup' at the position. Extracted the two config editors
into a shared configEditors module (avoids the MissionDeskAdmin↔View
import cycle) and, in adminMode, MissionDeskView now renders them inline
and saves to the service config (PUT /mission-desk-services/:id), with
optimistic local update. Verified live: editors appear in setup mode,
typed label persists to config.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F259"/>
+  <dimension ref="A1:F260"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5580,9 +5580,26 @@
         <v/>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>2026-07-29 17:20</v>
+      </c>
+      <c r="B260" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="C260" t="str">
+        <v>דסק משימה: תמונה וטקסט קבוע ניתנים להגדרה רק ב-tab הדסקים — צריך גם במצב ההגדרה בעמדה</v>
+      </c>
+      <c r="D260" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E260" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F259"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F260"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(mission-desk): WYSIWYG image/label in setup mode
In the position setup view, image and fixed-text now render exactly as
the operator will see them — the image fills the area with its fit, the
label renders full-size with its font/size/color/align — and a compact
floating toolbar carries the editing controls (paste/file/fit/remove for
image; text/size/font/bold/align/color for label). Replaces the
form-plus-thumbnail editors in that context; the desk-services admin tab
keeps its form editors. Verified live: full-area rendering + toolbars.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F260"/>
+  <dimension ref="A1:F261"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5597,9 +5597,26 @@
         <v/>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>2026-07-29 17:37</v>
+      </c>
+      <c r="B261" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C261" t="str">
+        <v>דסק משימה: במצב הגדרה תמונה/טקסט קבוע יוצגו WYSIWYG (כמו שהמפעיל יראה) עם כלי עריכה</v>
+      </c>
+      <c r="D261" t="str">
+        <v/>
+      </c>
+      <c r="E261" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F260"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F261"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(mission-desk): rich-text fixed-label — type on the board, style per segment
Replaces the single-style label editor with an on-canvas contentEditable
editor: you type directly where the text renders, select any part and
apply size/font/bold/color to just that selection. Stored as a runs[]
model (per-segment style) — normalized/merged via normalizeLabelRuns
(pure, unit-tested), legacy 'text' still honored. Station renders the
runs as React spans (never innerHTML from config — no injection). Used
in both the setup overlay and the desk-services tab. Verified live:
typing produces runs, per-segment sizing persists as distinct runs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F261"/>
+  <dimension ref="A1:F263"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5582,41 +5582,84 @@
     </row>
     <row r="260">
       <c r="A260" t="str">
+        <v/>
+      </c>
+      <c r="B260" t="str">
         <v>2026-07-29 17:20</v>
       </c>
-      <c r="B260" t="str">
+      <c r="C260" t="str">
         <v>תקלה</v>
       </c>
-      <c r="C260" t="str">
+      <c r="D260" t="str">
         <v>דסק משימה: תמונה וטקסט קבוע ניתנים להגדרה רק ב-tab הדסקים — צריך גם במצב ההגדרה בעמדה</v>
       </c>
-      <c r="D260" t="str">
-        <v>כן</v>
-      </c>
       <c r="E260" t="str">
+        <v>כן</v>
+      </c>
+      <c r="F260" t="str">
         <v/>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
+        <v/>
+      </c>
+      <c r="B261" t="str">
         <v>2026-07-29 17:37</v>
       </c>
-      <c r="B261" t="str">
-        <v>שיפור לתכולה קיימת</v>
-      </c>
       <c r="C261" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D261" t="str">
         <v>דסק משימה: במצב הגדרה תמונה/טקסט קבוע יוצגו WYSIWYG (כמו שהמפעיל יראה) עם כלי עריכה</v>
       </c>
-      <c r="D261" t="str">
-        <v/>
-      </c>
       <c r="E261" t="str">
+        <v/>
+      </c>
+      <c r="F261" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v/>
+      </c>
+      <c r="B262" t="str">
+        <v>2026-07-29 17:46</v>
+      </c>
+      <c r="C262" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D262" t="str">
+        <v>פריסת Railway לא עולה — לבדוק גורם (bind ל-PORT/host, start command, build, env vars, healthcheck)</v>
+      </c>
+      <c r="E262" t="str">
+        <v/>
+      </c>
+      <c r="F262" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>2026-07-29 17:53</v>
+      </c>
+      <c r="B263" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="C263" t="str">
+        <v>דסק משימה: טקסט קבוע — עורך rich-text בלוח עצמו, עיצוב פר-תו/מקטע (גודל/פונט/צבע/מודגש)</v>
+      </c>
+      <c r="D263" t="str">
+        <v>כן</v>
+      </c>
+      <c r="E263" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F261"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F263"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(requirements): log today's GAPI requests
Rows added by the requirements-tracker hook across today's session:
GAPI dev/prod database wiring, the schema alignment to SKY-KING naming,
sync latency, the landed status and the retraction rule.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F319"/>
+  <dimension ref="A1:F323"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -6788,9 +6788,89 @@
         <v/>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v/>
+      </c>
+      <c r="B320" t="str">
+        <v>2026-07-30 21:23</v>
+      </c>
+      <c r="C320" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D320" t="str">
+        <v>שינוי תווית בממשק GAPI: "בתעופה" יהיה "באוויר"</v>
+      </c>
+      <c r="E320" t="str">
+        <v/>
+      </c>
+      <c r="F320" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v/>
+      </c>
+      <c r="B321" t="str">
+        <v>2026-07-30 21:23</v>
+      </c>
+      <c r="C321" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D321" t="str">
+        <v>סימון "נחת" ב-GAPI יכבה אוטומטית את "באוויר" (בנוסף למסר המחיקה ל-SKY-KING)</v>
+      </c>
+      <c r="E321" t="str">
+        <v/>
+      </c>
+      <c r="F321" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v/>
+      </c>
+      <c r="B322" t="str">
+        <v>2026-07-30 21:26</v>
+      </c>
+      <c r="C322" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D322" t="str">
+        <v>כניסה למסך LOGIN של SKY-KING עם סיסמה שרירותית הצליחה - אכיפת הסיסמה מול מיראז' לא פעלה</v>
+      </c>
+      <c r="E322" t="str">
+        <v/>
+      </c>
+      <c r="F322" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v/>
+      </c>
+      <c r="B323" t="str">
+        <v>2026-07-30 21:29</v>
+      </c>
+      <c r="C323" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D323" t="str">
+        <v>דחיפת כל העבודה ל-GitHub - commit לכל השינויים הפתוחים (מכל הסשנים) + push לענף</v>
+      </c>
+      <c r="E323" t="str">
+        <v/>
+      </c>
+      <c r="F323" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F319"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F323"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(process): סקילי /ship ו-/worktree, hook לבמפ גרסה, ועדכון CLAUDE.md
קימוט עבודת התהליך שהצטברה בעץ הראשי, לבקשת המשתמש.

- /worktree - עץ נפרד לכל סוכן: הקמה, בדיקת בידוד, פורטים, ניקוי
- /ship - קימוט ודחיפה שמתחילים תמיד ב-npm run version:bump
- hooks/version-bump-reminder.mjs + רישומו ב-.claude/settings.json
- CLAUDE.md - שני איסורים חדשים (דחיפה בלי במפ, שני סוכנים בעץ אחד)
  והפניות לשני הסקילים
- project-requirements.xlsx - שורות דרישה שנוספו לאורך היום

גרסה: 1.0.33. הבמפ היה הכרחי ולא טקסי - 1.0.32 כבר תפוסה על main
(מיזוג ההקפה התלת מימדית), ושתי גרסאות באותו מספר עם תאריכים שונים
היו הופכות את מסך הכניסה לעדות לא אמינה על מה שרץ בפועל.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-requirements.xlsx
+++ b/project-requirements.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F695"/>
+  <dimension ref="A1:F704"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -14308,9 +14308,189 @@
         <v/>
       </c>
     </row>
+    <row r="696">
+      <c r="A696" t="str">
+        <v/>
+      </c>
+      <c r="B696" t="str">
+        <v>2026-08-11 09:49</v>
+      </c>
+      <c r="C696" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D696" t="str">
+        <v>תצוגת מז"א: שכבת Windy אינה מעוגנת/מתלכדת עם מפת השדה שמוצגת בפועל בעמדה</v>
+      </c>
+      <c r="E696" t="str">
+        <v/>
+      </c>
+      <c r="F696" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="str">
+        <v/>
+      </c>
+      <c r="B697" t="str">
+        <v>2026-08-11 10:15</v>
+      </c>
+      <c r="C697" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D697" t="str">
+        <v>מז"א בעמדת 305 (מפה מעוגנת): כמעט מדויק אך מוסט בכמה מיילים</v>
+      </c>
+      <c r="E697" t="str">
+        <v/>
+      </c>
+      <c r="F697" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="str">
+        <v/>
+      </c>
+      <c r="B698" t="str">
+        <v>2026-08-11 10:15</v>
+      </c>
+      <c r="C698" t="str">
+        <v>תקלה</v>
+      </c>
+      <c r="D698" t="str">
+        <v>מז"א בעמדת שדה מעוגנת ללא תמונת מפה (הקפה תל נוף): לא מעוגן טוב, נדרש זום פנימה משמעותי</v>
+      </c>
+      <c r="E698" t="str">
+        <v/>
+      </c>
+      <c r="F698" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="str">
+        <v/>
+      </c>
+      <c r="B699" t="str">
+        <v>2026-08-11 10:22</v>
+      </c>
+      <c r="C699" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D699" t="str">
+        <v>שדות תקלה ברמת מטוס בפ"מ (לא דרך GAPI): דגל תקלה כן/לא שמוצג באדום, מהות התקלה, פירוט חופשי</v>
+      </c>
+      <c r="E699" t="str">
+        <v/>
+      </c>
+      <c r="F699" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="str">
+        <v/>
+      </c>
+      <c r="B700" t="str">
+        <v>2026-08-11 10:22</v>
+      </c>
+      <c r="C700" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D700" t="str">
+        <v>תפריט מהויות תקלה מנוהל במסך ניהול מערכת (הוספה/עריכה/מחיקה)</v>
+      </c>
+      <c r="E700" t="str">
+        <v/>
+      </c>
+      <c r="F700" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="str">
+        <v/>
+      </c>
+      <c r="B701" t="str">
+        <v>2026-08-11 10:22</v>
+      </c>
+      <c r="C701" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D701" t="str">
+        <v>שדה תקלות מרוכז ברמת פ"מ: שרשור כל תקלות המטוסים - "תקלה למספר X", וב-HINT המהות והפירוט</v>
+      </c>
+      <c r="E701" t="str">
+        <v/>
+      </c>
+      <c r="F701" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="str">
+        <v/>
+      </c>
+      <c r="B702" t="str">
+        <v>2026-08-11 10:26</v>
+      </c>
+      <c r="C702" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D702" t="str">
+        <v>טבלת נקודות מכוון (העברת מטרה לתקיפה) בפ"מ - שורה לכל נ"צ תקיפה: שם מטרה, שם נקודת מכוון, נ"צ 17 ספרות, גובה ברגליים, HD, AN, AN מזערי, מרעום (מ"ש), הערה, חימוש (תפריט), כמות פצצות</v>
+      </c>
+      <c r="E702" t="str">
+        <v/>
+      </c>
+      <c r="F702" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="str">
+        <v/>
+      </c>
+      <c r="B703" t="str">
+        <v>2026-08-11 10:26</v>
+      </c>
+      <c r="C703" t="str">
+        <v>תכולה חדשה</v>
+      </c>
+      <c r="D703" t="str">
+        <v>העברת טבלת נקודות המכוון ב-GAPI (אינטגרציה דו-כיוונית עם השו"ב החיצוני)</v>
+      </c>
+      <c r="E703" t="str">
+        <v/>
+      </c>
+      <c r="F703" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="str">
+        <v/>
+      </c>
+      <c r="B704" t="str">
+        <v>2026-08-11 14:45</v>
+      </c>
+      <c r="C704" t="str">
+        <v>שיפור לתכולה קיימת</v>
+      </c>
+      <c r="D704" t="str">
+        <v>יישור עוגן מפת 305 לפי השוואת קו החוף שבמפה מול קו החוף של WINDY</v>
+      </c>
+      <c r="E704" t="str">
+        <v/>
+      </c>
+      <c r="F704" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F695"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F704"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>